<commit_message>
📊 업데이트 - 2026-09-14 15:59
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R19"/>
+  <dimension ref="A1:R24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,7 +541,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -556,12 +556,12 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>16.3</t>
+          <t>49.1</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>24.8</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -575,35 +575,35 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>355</v>
+        <v>362</v>
       </c>
       <c r="O2" t="n">
-        <v>56.9</v>
+        <v>57.5</v>
       </c>
       <c r="P2" t="n">
-        <v>41.1</v>
+        <v>40.6</v>
       </c>
       <c r="Q2" t="n">
-        <v>64.8</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="R2" t="n">
-        <v>45.9</v>
+        <v>46.1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2:35</t>
+          <t>1:10</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>Colorado Rockies</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -613,12 +613,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>67.0</t>
+          <t>69.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>33.0</t>
+          <t>31.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -657,55 +657,55 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>484</v>
+        <v>394</v>
       </c>
       <c r="O3" t="n">
-        <v>56.6</v>
+        <v>57.6</v>
       </c>
       <c r="P3" t="n">
-        <v>41.3</v>
+        <v>40.1</v>
       </c>
       <c r="Q3" t="n">
-        <v>64.90000000000001</v>
+        <v>64</v>
       </c>
       <c r="R3" t="n">
-        <v>47.3</v>
+        <v>46.4</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>3:10</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Chiba Lotte Marines</t>
+          <t>Cincinnati Reds</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>69.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>31.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>5-2</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -720,17 +720,17 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>19.7</t>
+          <t>33.8</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>13.8</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -739,60 +739,60 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>758</v>
+        <v>394</v>
       </c>
       <c r="O4" t="n">
-        <v>53.6</v>
+        <v>57.6</v>
       </c>
       <c r="P4" t="n">
-        <v>44.3</v>
+        <v>40.1</v>
       </c>
       <c r="Q4" t="n">
-        <v>65.7</v>
+        <v>64</v>
       </c>
       <c r="R4" t="n">
-        <v>47.6</v>
+        <v>46.4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>3:15</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Seibu Lions</t>
+          <t>St.Louis Cardinals</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Nippon Ham Fighters</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>70.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>30.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -802,79 +802,79 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>8.9</t>
+          <t>20.8</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>6.7</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N5" t="n">
-        <v>514</v>
+        <v>362</v>
       </c>
       <c r="O5" t="n">
-        <v>45.5</v>
+        <v>57.5</v>
       </c>
       <c r="P5" t="n">
-        <v>52.7</v>
+        <v>40.6</v>
       </c>
       <c r="Q5" t="n">
-        <v>65.59999999999999</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="R5" t="n">
-        <v>45.7</v>
+        <v>46.1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>3:20</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>66.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>34.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -884,79 +884,79 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>27.1</t>
+          <t>10.6</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>9.9</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N6" t="n">
-        <v>879</v>
+        <v>540</v>
       </c>
       <c r="O6" t="n">
-        <v>48.8</v>
+        <v>57.2</v>
       </c>
       <c r="P6" t="n">
-        <v>49.4</v>
+        <v>40.9</v>
       </c>
       <c r="Q6" t="n">
-        <v>66.7</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="R6" t="n">
-        <v>47.1</v>
+        <v>47.6</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>5:10</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>KT Wiz Suwon</t>
+          <t>Arizona Diamondbacks</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Lotte Giants</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>71.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>29.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>5-6</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -966,79 +966,79 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>64.4</t>
+          <t>42.1</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>39.2</t>
+          <t>19.4</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N7" t="n">
-        <v>879</v>
+        <v>325</v>
       </c>
       <c r="O7" t="n">
-        <v>48.8</v>
+        <v>58.8</v>
       </c>
       <c r="P7" t="n">
-        <v>49.4</v>
+        <v>39.4</v>
       </c>
       <c r="Q7" t="n">
-        <v>66.7</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="R7" t="n">
-        <v>47.1</v>
+        <v>47.4</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>7:40</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>Cleveland Guardians</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>71.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>29.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1048,74 +1048,74 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>42.1</t>
+          <t>19.7</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>19.4</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N8" t="n">
-        <v>586</v>
+        <v>325</v>
       </c>
       <c r="O8" t="n">
-        <v>46.9</v>
+        <v>58.8</v>
       </c>
       <c r="P8" t="n">
-        <v>51.2</v>
+        <v>39.4</v>
       </c>
       <c r="Q8" t="n">
-        <v>66.7</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="R8" t="n">
-        <v>45.4</v>
+        <v>47.4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>8:20</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>San Francisco Giants</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>33.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>67.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>3-6</t>
+          <t>2-5</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1130,17 +1130,17 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>58.3</t>
+          <t>32.4</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>33.0</t>
+          <t>12.9</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1149,25 +1149,25 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>550</v>
+        <v>303</v>
       </c>
       <c r="O9" t="n">
-        <v>45.8</v>
+        <v>41.3</v>
       </c>
       <c r="P9" t="n">
-        <v>52.4</v>
+        <v>56.8</v>
       </c>
       <c r="Q9" t="n">
-        <v>66.40000000000001</v>
+        <v>66.7</v>
       </c>
       <c r="R9" t="n">
-        <v>45.8</v>
+        <v>46.5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>3:20</t>
+          <t>8:40</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1177,7 +1177,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>Atlanta Braves</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1187,17 +1187,17 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>61.0</t>
+          <t>71.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>39.0</t>
+          <t>29.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>6-5</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1212,17 +1212,17 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>10.6</t>
+          <t>70.0</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>45.4</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1231,55 +1231,55 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>796</v>
+        <v>325</v>
       </c>
       <c r="O10" t="n">
-        <v>53.6</v>
+        <v>58.8</v>
       </c>
       <c r="P10" t="n">
-        <v>44.2</v>
+        <v>39.4</v>
       </c>
       <c r="Q10" t="n">
-        <v>66.2</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="R10" t="n">
-        <v>47.1</v>
+        <v>47.4</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>5:10</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Boston Red Sox</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>63.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>37.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1294,12 +1294,12 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>29.7</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>11.3</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1313,40 +1313,40 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>697</v>
+        <v>960</v>
       </c>
       <c r="O11" t="n">
-        <v>54.9</v>
+        <v>51.4</v>
       </c>
       <c r="P11" t="n">
-        <v>42.8</v>
+        <v>46.7</v>
       </c>
       <c r="Q11" t="n">
-        <v>65.3</v>
+        <v>66.5</v>
       </c>
       <c r="R11" t="n">
-        <v>47.2</v>
+        <v>47.1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>5:10</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1361,7 +1361,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>4-6</t>
+          <t>2-3</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1376,12 +1376,12 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>64.4</t>
+          <t>8.9</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>39.2</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1395,16 +1395,16 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>747</v>
+        <v>757</v>
       </c>
       <c r="O12" t="n">
-        <v>45.6</v>
+        <v>45.8</v>
       </c>
       <c r="P12" t="n">
-        <v>52.3</v>
+        <v>52.2</v>
       </c>
       <c r="Q12" t="n">
-        <v>66.7</v>
+        <v>66.8</v>
       </c>
       <c r="R12" t="n">
         <v>45.4</v>
@@ -1413,17 +1413,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>7:10</t>
+          <t>2:35</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>Washington Nationals</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Houston Astros</t>
+          <t>Los Angeles Angels</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1433,12 +1433,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>59.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>41.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1458,12 +1458,12 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>18.5</t>
+          <t>31.1</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>5.6</t>
+          <t>12.1</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1477,35 +1477,35 @@
         </is>
       </c>
       <c r="N13" t="n">
-        <v>886</v>
+        <v>825</v>
       </c>
       <c r="O13" t="n">
-        <v>54</v>
+        <v>54.1</v>
       </c>
       <c r="P13" t="n">
-        <v>43.9</v>
+        <v>43.8</v>
       </c>
       <c r="Q13" t="n">
-        <v>65.5</v>
+        <v>66.5</v>
       </c>
       <c r="R13" t="n">
-        <v>46</v>
+        <v>46.7</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>2:35</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Boston Red Sox</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Cincinnati Reds</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1515,17 +1515,17 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>61.0</t>
+          <t>51.0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>39.0</t>
+          <t>49.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1540,12 +1540,12 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>22.0</t>
+          <t>20.8</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>7.3</t>
+          <t>6.7</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1559,60 +1559,60 @@
         </is>
       </c>
       <c r="N14" t="n">
-        <v>796</v>
+        <v>944</v>
       </c>
       <c r="O14" t="n">
-        <v>53.6</v>
+        <v>51</v>
       </c>
       <c r="P14" t="n">
-        <v>44.2</v>
+        <v>47.1</v>
       </c>
       <c r="Q14" t="n">
         <v>66.2</v>
       </c>
       <c r="R14" t="n">
-        <v>47.1</v>
+        <v>46.8</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>17:05</t>
+          <t>2:35</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>TSG Hawks</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Fubon Guardians</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>61.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>39.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1622,12 +1622,12 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>49.1</t>
+          <t>33.8</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>24.8</t>
+          <t>13.8</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1637,20 +1637,20 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N15" t="n">
-        <v>796</v>
+        <v>890</v>
       </c>
       <c r="O15" t="n">
-        <v>53.6</v>
+        <v>49</v>
       </c>
       <c r="P15" t="n">
-        <v>44.2</v>
+        <v>49.2</v>
       </c>
       <c r="Q15" t="n">
-        <v>66.2</v>
+        <v>66.7</v>
       </c>
       <c r="R15" t="n">
         <v>47.1</v>
@@ -1659,37 +1659,37 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>2:35</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Rakuten Monkeys</t>
+          <t>Atlanta Braves</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Chinatrust Brothers</t>
+          <t>Philadelphia Phillies</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>CPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>58.0</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>42.0</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1704,12 +1704,12 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>31.1</t>
+          <t>49.1</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>12.1</t>
+          <t>24.8</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1723,60 +1723,60 @@
         </is>
       </c>
       <c r="N16" t="n">
-        <v>932</v>
+        <v>874</v>
       </c>
       <c r="O16" t="n">
-        <v>50.6</v>
+        <v>53.8</v>
       </c>
       <c r="P16" t="n">
-        <v>47.4</v>
+        <v>44.1</v>
       </c>
       <c r="Q16" t="n">
-        <v>66.09999999999999</v>
+        <v>66.7</v>
       </c>
       <c r="R16" t="n">
-        <v>46.8</v>
+        <v>46.6</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>2:37</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1786,69 +1786,69 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>53.1</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>28.2</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N17" t="n">
-        <v>899</v>
+        <v>766</v>
       </c>
       <c r="O17" t="n">
-        <v>49.4</v>
+        <v>53.9</v>
       </c>
       <c r="P17" t="n">
-        <v>48.6</v>
+        <v>44</v>
       </c>
       <c r="Q17" t="n">
-        <v>66.5</v>
+        <v>65.7</v>
       </c>
       <c r="R17" t="n">
-        <v>47.4</v>
+        <v>47.7</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>2:40</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>LG Twins</t>
+          <t>Los Angeles Dodgers</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1868,17 +1868,17 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>42.1</t>
+          <t>64.4</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>19.4</t>
+          <t>39.2</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -1887,101 +1887,511 @@
         </is>
       </c>
       <c r="N18" t="n">
-        <v>899</v>
+        <v>781</v>
       </c>
       <c r="O18" t="n">
-        <v>49.4</v>
+        <v>46.7</v>
       </c>
       <c r="P18" t="n">
-        <v>48.6</v>
+        <v>51.3</v>
       </c>
       <c r="Q18" t="n">
-        <v>66.5</v>
+        <v>66.3</v>
       </c>
       <c r="R18" t="n">
-        <v>47.4</v>
+        <v>46.1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>4:07</t>
+          <t>3:10</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
+          <t>Minnesota Twins</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>43.0</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>57.0</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2-5</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>29.7</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>11.3</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>706</v>
+      </c>
+      <c r="O19" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="P19" t="n">
+        <v>52.3</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>66.59999999999999</v>
+      </c>
+      <c r="R19" t="n">
+        <v>45.2</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>7:40</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Cincinnati Reds</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Los Angeles Dodgers</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>37.0</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>63.0</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>5-7</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>64.4</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>39.2</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N20" t="n">
+        <v>458</v>
+      </c>
+      <c r="O20" t="n">
+        <v>44.3</v>
+      </c>
+      <c r="P20" t="n">
+        <v>53.9</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>65.90000000000001</v>
+      </c>
+      <c r="R20" t="n">
+        <v>46.3</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>8:07</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
           <t>Toronto Blue Jays</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Detroit Tigers</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>44.0</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>56.0</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>19.7</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="N21" t="n">
+        <v>757</v>
+      </c>
+      <c r="O21" t="n">
+        <v>45.8</v>
+      </c>
+      <c r="P21" t="n">
+        <v>52.2</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>66.8</v>
+      </c>
+      <c r="R21" t="n">
+        <v>45.4</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>8:10</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>New York Mets</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
         <is>
           <t>Baltimore Orioles</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>MLB</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>49.0</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>51.0</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>22.0</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>7.3</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N22" t="n">
+        <v>948</v>
+      </c>
+      <c r="O22" t="n">
+        <v>51.9</v>
+      </c>
+      <c r="P22" t="n">
+        <v>46.2</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>66.2</v>
+      </c>
+      <c r="R22" t="n">
+        <v>46.4</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>8:40</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Minnesota Twins</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>New York Yankees</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
         <is>
           <t>4-5</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="J23" t="inlineStr">
         <is>
           <t>53.1</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="K23" t="inlineStr">
         <is>
           <t>28.2</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
         <is>
           <t>원정승</t>
         </is>
       </c>
-      <c r="N19" t="n">
-        <v>899</v>
-      </c>
-      <c r="O19" t="n">
-        <v>49.4</v>
-      </c>
-      <c r="P19" t="n">
-        <v>48.6</v>
-      </c>
-      <c r="Q19" t="n">
-        <v>66.5</v>
-      </c>
-      <c r="R19" t="n">
-        <v>47.4</v>
+      <c r="N23" t="n">
+        <v>816</v>
+      </c>
+      <c r="O23" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="P23" t="n">
+        <v>50.6</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>66.8</v>
+      </c>
+      <c r="R23" t="n">
+        <v>46.7</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>TSG Hawks</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Rakuten Monkeys</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>CPB</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>53.0</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>5-3</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>18.5</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>5.6</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="N24" t="n">
+        <v>916</v>
+      </c>
+      <c r="O24" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="P24" t="n">
+        <v>45.3</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>66.59999999999999</v>
+      </c>
+      <c r="R24" t="n">
+        <v>46.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-09-15 16:16
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R24"/>
+  <dimension ref="A1:R20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -516,12 +516,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -556,12 +556,12 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>49.1</t>
+          <t>51.8</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>24.8</t>
+          <t>27.1</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -575,60 +575,60 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>362</v>
+        <v>370</v>
       </c>
       <c r="O2" t="n">
-        <v>57.5</v>
+        <v>57.3</v>
       </c>
       <c r="P2" t="n">
-        <v>40.6</v>
+        <v>40.8</v>
       </c>
       <c r="Q2" t="n">
-        <v>64.90000000000001</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="R2" t="n">
-        <v>46.1</v>
+        <v>46.2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1:10</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>69.0</t>
+          <t>30.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>31.0</t>
+          <t>70.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>6-3</t>
+          <t>2-3</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -638,12 +638,12 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>54.4</t>
+          <t>9.7</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>29.4</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -653,64 +653,64 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N3" t="n">
-        <v>394</v>
+        <v>199</v>
       </c>
       <c r="O3" t="n">
-        <v>57.6</v>
+        <v>40.2</v>
       </c>
       <c r="P3" t="n">
-        <v>40.1</v>
+        <v>58.3</v>
       </c>
       <c r="Q3" t="n">
-        <v>64</v>
+        <v>68.3</v>
       </c>
       <c r="R3" t="n">
-        <v>46.4</v>
+        <v>48.2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>3:10</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Cincinnati Reds</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>69.0</t>
+          <t>32.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>31.0</t>
+          <t>68.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>5-2</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -720,12 +720,12 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>33.8</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>13.8</t>
+          <t>31.8</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -735,34 +735,34 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N4" t="n">
-        <v>394</v>
+        <v>273</v>
       </c>
       <c r="O4" t="n">
-        <v>57.6</v>
+        <v>43.2</v>
       </c>
       <c r="P4" t="n">
-        <v>40.1</v>
+        <v>55.3</v>
       </c>
       <c r="Q4" t="n">
-        <v>64</v>
+        <v>67.8</v>
       </c>
       <c r="R4" t="n">
-        <v>46.4</v>
+        <v>48.4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>3:15</t>
+          <t>7:40</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>St.Louis Cardinals</t>
+          <t>Cleveland Guardians</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -777,12 +777,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>70.0</t>
+          <t>71.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>30.0</t>
+          <t>29.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -802,12 +802,12 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>20.8</t>
+          <t>19.7</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>6.7</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -821,35 +821,35 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>362</v>
+        <v>333</v>
       </c>
       <c r="O5" t="n">
-        <v>57.5</v>
+        <v>58.6</v>
       </c>
       <c r="P5" t="n">
-        <v>40.6</v>
+        <v>39.6</v>
       </c>
       <c r="Q5" t="n">
-        <v>64.90000000000001</v>
+        <v>67.3</v>
       </c>
       <c r="R5" t="n">
-        <v>46.1</v>
+        <v>47.4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>3:20</t>
+          <t>9:40</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Colorado Rockies</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -859,22 +859,22 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>66.0</t>
+          <t>31.0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>34.0</t>
+          <t>69.0</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>4-8</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -884,12 +884,12 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>10.6</t>
+          <t>80.9</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>59.8</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -899,29 +899,29 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N6" t="n">
-        <v>540</v>
+        <v>228</v>
       </c>
       <c r="O6" t="n">
-        <v>57.2</v>
+        <v>41.2</v>
       </c>
       <c r="P6" t="n">
-        <v>40.9</v>
+        <v>57.5</v>
       </c>
       <c r="Q6" t="n">
-        <v>65.40000000000001</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="R6" t="n">
-        <v>47.6</v>
+        <v>48.7</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>5:10</t>
+          <t>10:40</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -931,7 +931,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -941,22 +941,22 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>71.0</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>29.0</t>
+          <t>64.0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -966,12 +966,12 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>42.1</t>
+          <t>43.5</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>19.4</t>
+          <t>20.4</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -981,64 +981,64 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N7" t="n">
-        <v>325</v>
+        <v>420</v>
       </c>
       <c r="O7" t="n">
-        <v>58.8</v>
+        <v>42.4</v>
       </c>
       <c r="P7" t="n">
-        <v>39.4</v>
+        <v>55.7</v>
       </c>
       <c r="Q7" t="n">
-        <v>67.09999999999999</v>
+        <v>68.3</v>
       </c>
       <c r="R7" t="n">
-        <v>47.4</v>
+        <v>47.6</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Cleveland Guardians</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>71.0</t>
+          <t>44.0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>29.0</t>
+          <t>56.0</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1048,79 +1048,79 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>19.7</t>
+          <t>25.8</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N8" t="n">
-        <v>325</v>
+        <v>767</v>
       </c>
       <c r="O8" t="n">
-        <v>58.8</v>
+        <v>45.8</v>
       </c>
       <c r="P8" t="n">
-        <v>39.4</v>
+        <v>52.3</v>
       </c>
       <c r="Q8" t="n">
-        <v>67.09999999999999</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="R8" t="n">
-        <v>47.4</v>
+        <v>45.4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>8:20</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>San Francisco Giants</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>33.0</t>
+          <t>54.0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>67.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2-5</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1130,74 +1130,74 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>32.4</t>
+          <t>24.5</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>12.9</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N9" t="n">
-        <v>303</v>
+        <v>957</v>
       </c>
       <c r="O9" t="n">
-        <v>41.3</v>
+        <v>53.1</v>
       </c>
       <c r="P9" t="n">
-        <v>56.8</v>
+        <v>45.2</v>
       </c>
       <c r="Q9" t="n">
-        <v>66.7</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="R9" t="n">
-        <v>46.5</v>
+        <v>46.8</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Atlanta Braves</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>71.0</t>
+          <t>61.0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>29.0</t>
+          <t>39.0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>6-5</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1212,17 +1212,17 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>70.0</t>
+          <t>46.3</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>45.4</t>
+          <t>22.6</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1231,19 +1231,19 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>325</v>
+        <v>819</v>
       </c>
       <c r="O10" t="n">
-        <v>58.8</v>
+        <v>53.7</v>
       </c>
       <c r="P10" t="n">
-        <v>39.4</v>
+        <v>44.2</v>
       </c>
       <c r="Q10" t="n">
-        <v>67.09999999999999</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="R10" t="n">
-        <v>47.4</v>
+        <v>47.1</v>
       </c>
     </row>
     <row r="11">
@@ -1254,12 +1254,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1269,22 +1269,22 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>2-3</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1294,12 +1294,12 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>9.7</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1309,64 +1309,64 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N11" t="n">
-        <v>960</v>
+        <v>791</v>
       </c>
       <c r="O11" t="n">
-        <v>51.4</v>
+        <v>46.6</v>
       </c>
       <c r="P11" t="n">
-        <v>46.7</v>
+        <v>51.5</v>
       </c>
       <c r="Q11" t="n">
-        <v>66.5</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="R11" t="n">
-        <v>47.1</v>
+        <v>46</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>44.0</t>
+          <t>43.0</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>56.0</t>
+          <t>57.0</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>4-6</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1376,12 +1376,12 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>8.9</t>
+          <t>44.9</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>21.5</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1395,55 +1395,55 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>757</v>
+        <v>716</v>
       </c>
       <c r="O12" t="n">
         <v>45.8</v>
       </c>
       <c r="P12" t="n">
-        <v>52.2</v>
+        <v>52.4</v>
       </c>
       <c r="Q12" t="n">
-        <v>66.8</v>
+        <v>66.5</v>
       </c>
       <c r="R12" t="n">
-        <v>45.4</v>
+        <v>45.3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2:35</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Washington Nationals</t>
+          <t>Samsung Lions</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Los Angeles Angels</t>
+          <t>Lotte Giants</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>59.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>41.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>7-5</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1458,12 +1458,12 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>31.1</t>
+          <t>81.7</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>12.1</t>
+          <t>60.9</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1477,60 +1477,60 @@
         </is>
       </c>
       <c r="N13" t="n">
-        <v>825</v>
+        <v>957</v>
       </c>
       <c r="O13" t="n">
-        <v>54.1</v>
+        <v>53.7</v>
       </c>
       <c r="P13" t="n">
-        <v>43.8</v>
+        <v>44.3</v>
       </c>
       <c r="Q13" t="n">
-        <v>66.5</v>
+        <v>65.8</v>
       </c>
       <c r="R13" t="n">
-        <v>46.7</v>
+        <v>46.6</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2:35</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Boston Red Sox</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>51.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>49.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>5-7</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1540,12 +1540,12 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>20.8</t>
+          <t>64.4</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>6.7</t>
+          <t>39.2</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1555,39 +1555,39 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="N14" t="n">
-        <v>944</v>
+        <v>855</v>
       </c>
       <c r="O14" t="n">
-        <v>51</v>
+        <v>48.9</v>
       </c>
       <c r="P14" t="n">
-        <v>47.1</v>
+        <v>49.2</v>
       </c>
       <c r="Q14" t="n">
-        <v>66.2</v>
+        <v>66.3</v>
       </c>
       <c r="R14" t="n">
-        <v>46.8</v>
+        <v>46.9</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2:35</t>
+          <t>7:40</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Cincinnati Reds</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>Los Angeles Dodgers</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1597,17 +1597,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>48.0</t>
+          <t>37.0</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>52.0</t>
+          <t>63.0</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>5-7</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1622,12 +1622,12 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>33.8</t>
+          <t>64.4</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>13.8</t>
+          <t>39.2</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1641,35 +1641,35 @@
         </is>
       </c>
       <c r="N15" t="n">
-        <v>890</v>
+        <v>464</v>
       </c>
       <c r="O15" t="n">
-        <v>49</v>
+        <v>44.2</v>
       </c>
       <c r="P15" t="n">
-        <v>49.2</v>
+        <v>54.1</v>
       </c>
       <c r="Q15" t="n">
-        <v>66.7</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="R15" t="n">
-        <v>47.1</v>
+        <v>46.8</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2:35</t>
+          <t>8:45</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Atlanta Braves</t>
+          <t>St.Louis Cardinals</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies</t>
+          <t>San Francisco Giants</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1679,17 +1679,17 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>58.0</t>
+          <t>62.0</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>42.0</t>
+          <t>38.0</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1704,12 +1704,12 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>49.1</t>
+          <t>33.8</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>24.8</t>
+          <t>13.8</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1723,35 +1723,35 @@
         </is>
       </c>
       <c r="N16" t="n">
-        <v>874</v>
+        <v>779</v>
       </c>
       <c r="O16" t="n">
-        <v>53.8</v>
+        <v>53.7</v>
       </c>
       <c r="P16" t="n">
-        <v>44.1</v>
+        <v>44.3</v>
       </c>
       <c r="Q16" t="n">
-        <v>66.7</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="R16" t="n">
-        <v>46.6</v>
+        <v>47.6</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2:37</t>
+          <t>10:38</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Toronto Blue Jays</t>
+          <t>Los Angeles Angels</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>Seattle Mariners</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1761,17 +1761,17 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>62.0</t>
+          <t>52.0</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>38.0</t>
+          <t>48.0</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1786,12 +1786,12 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>53.1</t>
+          <t>12.3</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>28.2</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1805,60 +1805,60 @@
         </is>
       </c>
       <c r="N17" t="n">
-        <v>766</v>
+        <v>973</v>
       </c>
       <c r="O17" t="n">
-        <v>53.9</v>
+        <v>51.3</v>
       </c>
       <c r="P17" t="n">
-        <v>44</v>
+        <v>46.8</v>
       </c>
       <c r="Q17" t="n">
-        <v>65.7</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="R17" t="n">
-        <v>47.7</v>
+        <v>47.2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2:40</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>Fubon Guardians</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers</t>
+          <t>Wei Chuan Dragons</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>45.0</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>55.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>4-6</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1868,12 +1868,12 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>64.4</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>39.2</t>
+          <t>0.8</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1883,59 +1883,59 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N18" t="n">
-        <v>781</v>
+        <v>807</v>
       </c>
       <c r="O18" t="n">
+        <v>54</v>
+      </c>
+      <c r="P18" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>65.8</v>
+      </c>
+      <c r="R18" t="n">
         <v>46.7</v>
-      </c>
-      <c r="P18" t="n">
-        <v>51.3</v>
-      </c>
-      <c r="Q18" t="n">
-        <v>66.3</v>
-      </c>
-      <c r="R18" t="n">
-        <v>46.1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>3:10</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>TSG Hawks</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Cleveland Guardians</t>
+          <t>Chinatrust Brothers</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>43.0</t>
+          <t>45.0</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>57.0</t>
+          <t>55.0</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2-5</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1969,60 +1969,60 @@
         </is>
       </c>
       <c r="N19" t="n">
-        <v>706</v>
+        <v>791</v>
       </c>
       <c r="O19" t="n">
-        <v>45.9</v>
+        <v>46.6</v>
       </c>
       <c r="P19" t="n">
-        <v>52.3</v>
+        <v>51.5</v>
       </c>
       <c r="Q19" t="n">
-        <v>66.59999999999999</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="R19" t="n">
-        <v>45.2</v>
+        <v>46</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Cincinnati Reds</t>
+          <t>Uni Lions</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers</t>
+          <t>Rakuten Monkeys</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>CPB</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>37.0</t>
+          <t>53.0</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>63.0</t>
+          <t>47.0</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>5-7</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -2032,12 +2032,12 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>64.4</t>
+          <t>23.3</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>39.2</t>
+          <t>7.9</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -2047,351 +2047,23 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="N20" t="n">
-        <v>458</v>
+        <v>961</v>
       </c>
       <c r="O20" t="n">
-        <v>44.3</v>
+        <v>51.8</v>
       </c>
       <c r="P20" t="n">
-        <v>53.9</v>
+        <v>46.3</v>
       </c>
       <c r="Q20" t="n">
-        <v>65.90000000000001</v>
+        <v>66.2</v>
       </c>
       <c r="R20" t="n">
-        <v>46.3</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>8:07</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Toronto Blue Jays</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Detroit Tigers</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>44.0</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>56.0</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>3-4</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>19.7</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>6.1</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>원정승</t>
-        </is>
-      </c>
-      <c r="N21" t="n">
-        <v>757</v>
-      </c>
-      <c r="O21" t="n">
-        <v>45.8</v>
-      </c>
-      <c r="P21" t="n">
-        <v>52.2</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>66.8</v>
-      </c>
-      <c r="R21" t="n">
-        <v>45.4</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>8:10</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>New York Mets</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Baltimore Orioles</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>53.0</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>47.0</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>4-3</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>22.0</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>7.3</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="N22" t="n">
-        <v>948</v>
-      </c>
-      <c r="O22" t="n">
-        <v>51.9</v>
-      </c>
-      <c r="P22" t="n">
-        <v>46.2</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>66.2</v>
-      </c>
-      <c r="R22" t="n">
-        <v>46.4</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>8:40</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Minnesota Twins</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>New York Yankees</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>46.0</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>54.0</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>4-5</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>53.1</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>28.2</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>원정승</t>
-        </is>
-      </c>
-      <c r="N23" t="n">
-        <v>816</v>
-      </c>
-      <c r="O23" t="n">
-        <v>47.5</v>
-      </c>
-      <c r="P23" t="n">
-        <v>50.6</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>66.8</v>
-      </c>
-      <c r="R23" t="n">
-        <v>46.7</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>19:35</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>TSG Hawks</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Rakuten Monkeys</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>CPB</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>53.0</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>46.0</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>5-3</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>18.5</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>5.6</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>★</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="N24" t="n">
-        <v>916</v>
-      </c>
-      <c r="O24" t="n">
-        <v>52.9</v>
-      </c>
-      <c r="P24" t="n">
-        <v>45.3</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>66.59999999999999</v>
-      </c>
-      <c r="R24" t="n">
-        <v>46.9</v>
+        <v>46.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-09-16 16:53
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R11"/>
+  <dimension ref="A1:AA11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,60 +449,105 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>최종_홈승확률</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>최종_원정승확률</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>FB_예상스코어</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>FB_예측결과</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>오버6.5예측</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>오버8.5예측</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>오버10.5예측</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>오버8.5보정</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>오버8.5추천</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>오버10.5보정</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>오버10.5추천</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
         <is>
           <t>신호등급</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>신뢰도</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
         <is>
           <t>추천픽</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>판정근거</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>유효표본</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
         <is>
           <t>유사경기수</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>유사_홈승실적</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>유사_원정실적</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>유사_오버8.5</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>유사_오버10.5</t>
         </is>
@@ -535,48 +580,87 @@
       <c r="F2" t="n">
         <v>75</v>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" t="n">
+        <v>35</v>
+      </c>
+      <c r="H2" t="n">
+        <v>65</v>
+      </c>
+      <c r="I2" t="inlineStr">
         <is>
           <t>2-5</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
         <v>28.4</v>
       </c>
-      <c r="K2" t="n">
+      <c r="M2" t="n">
         <v>10.6</v>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
         <is>
           <t>⏭</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O2" t="n">
-        <v>50</v>
-      </c>
-      <c r="P2" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X2" t="n">
+        <v>50</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>50</v>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -609,48 +693,87 @@
       <c r="F3" t="n">
         <v>46</v>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" t="n">
+        <v>52.4</v>
+      </c>
+      <c r="H3" t="n">
+        <v>47.6</v>
+      </c>
+      <c r="I3" t="inlineStr">
         <is>
           <t>5-3</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
         <v>42.1</v>
       </c>
-      <c r="K3" t="n">
+      <c r="M3" t="n">
         <v>19.4</v>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
         <is>
           <t>⏭</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O3" t="n">
-        <v>50</v>
-      </c>
-      <c r="P3" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W3" t="n">
+        <v>0</v>
+      </c>
+      <c r="X3" t="n">
+        <v>50</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>50</v>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -683,48 +806,87 @@
       <c r="F4" t="n">
         <v>67</v>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" t="n">
+        <v>39.8</v>
+      </c>
+      <c r="H4" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="I4" t="inlineStr">
         <is>
           <t>4-5</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J4" t="n">
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
         <v>55.7</v>
       </c>
-      <c r="K4" t="n">
+      <c r="M4" t="n">
         <v>30.6</v>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
         <is>
           <t>⏭</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O4" t="n">
-        <v>50</v>
-      </c>
-      <c r="P4" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X4" t="n">
+        <v>50</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>50</v>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -757,48 +919,87 @@
       <c r="F5" t="n">
         <v>64</v>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="H5" t="n">
+        <v>58.4</v>
+      </c>
+      <c r="I5" t="inlineStr">
         <is>
           <t>3-5</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J5" t="n">
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
         <v>46.3</v>
       </c>
-      <c r="K5" t="n">
+      <c r="M5" t="n">
         <v>22.6</v>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
         <is>
           <t>⏭</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" t="n">
-        <v>50</v>
-      </c>
-      <c r="P5" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X5" t="n">
+        <v>50</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>50</v>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -831,48 +1032,87 @@
       <c r="F6" t="n">
         <v>56</v>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="H6" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="I6" t="inlineStr">
         <is>
           <t>4-6</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J6" t="n">
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
         <v>49.1</v>
       </c>
-      <c r="K6" t="n">
+      <c r="M6" t="n">
         <v>24.8</v>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
         <is>
           <t>⏭</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" t="n">
-        <v>50</v>
-      </c>
-      <c r="P6" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X6" t="n">
+        <v>50</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>50</v>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -905,48 +1145,87 @@
       <c r="F7" t="n">
         <v>54</v>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" t="n">
+        <v>47.6</v>
+      </c>
+      <c r="H7" t="n">
+        <v>52.4</v>
+      </c>
+      <c r="I7" t="inlineStr">
         <is>
           <t>4-5</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J7" t="n">
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L7" t="n">
         <v>53.1</v>
       </c>
-      <c r="K7" t="n">
+      <c r="M7" t="n">
         <v>28.2</v>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
         <is>
           <t>⏭</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" t="n">
-        <v>50</v>
-      </c>
-      <c r="P7" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V7" t="n">
+        <v>0</v>
+      </c>
+      <c r="W7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X7" t="n">
+        <v>50</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>50</v>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -979,48 +1258,87 @@
       <c r="F8" t="n">
         <v>41</v>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G8" t="n">
+        <v>55.4</v>
+      </c>
+      <c r="H8" t="n">
+        <v>44.6</v>
+      </c>
+      <c r="I8" t="inlineStr">
         <is>
           <t>5-4</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J8" t="n">
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
         <v>55.7</v>
       </c>
-      <c r="K8" t="n">
+      <c r="M8" t="n">
         <v>30.6</v>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
         <is>
           <t>⏭</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="n">
-        <v>0</v>
-      </c>
-      <c r="O8" t="n">
-        <v>50</v>
-      </c>
-      <c r="P8" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V8" t="n">
+        <v>0</v>
+      </c>
+      <c r="W8" t="n">
+        <v>0</v>
+      </c>
+      <c r="X8" t="n">
+        <v>50</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>50</v>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1053,48 +1371,87 @@
       <c r="F9" t="n">
         <v>59</v>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G9" t="n">
+        <v>44.6</v>
+      </c>
+      <c r="H9" t="n">
+        <v>55.4</v>
+      </c>
+      <c r="I9" t="inlineStr">
         <is>
           <t>4-6</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J9" t="n">
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L9" t="n">
         <v>42.1</v>
       </c>
-      <c r="K9" t="n">
+      <c r="M9" t="n">
         <v>19.4</v>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
         <is>
           <t>⏭</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="n">
-        <v>0</v>
-      </c>
-      <c r="O9" t="n">
-        <v>50</v>
-      </c>
-      <c r="P9" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V9" t="n">
+        <v>0</v>
+      </c>
+      <c r="W9" t="n">
+        <v>0</v>
+      </c>
+      <c r="X9" t="n">
+        <v>50</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>50</v>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA9" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1127,48 +1484,87 @@
       <c r="F10" t="n">
         <v>57</v>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G10" t="n">
+        <v>45.8</v>
+      </c>
+      <c r="H10" t="n">
+        <v>54.2</v>
+      </c>
+      <c r="I10" t="inlineStr">
         <is>
           <t>3-5</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J10" t="n">
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L10" t="n">
         <v>40.7</v>
       </c>
-      <c r="K10" t="n">
+      <c r="M10" t="n">
         <v>18.4</v>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
         <is>
           <t>⏭</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="n">
-        <v>0</v>
-      </c>
-      <c r="O10" t="n">
-        <v>50</v>
-      </c>
-      <c r="P10" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R10" t="inlineStr">
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V10" t="n">
+        <v>0</v>
+      </c>
+      <c r="W10" t="n">
+        <v>0</v>
+      </c>
+      <c r="X10" t="n">
+        <v>50</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>50</v>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1201,48 +1597,87 @@
       <c r="F11" t="n">
         <v>43</v>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G11" t="n">
+        <v>54.2</v>
+      </c>
+      <c r="H11" t="n">
+        <v>45.8</v>
+      </c>
+      <c r="I11" t="inlineStr">
         <is>
           <t>4-3</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J11" t="n">
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L11" t="n">
         <v>29.7</v>
       </c>
-      <c r="K11" t="n">
+      <c r="M11" t="n">
         <v>11.3</v>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
         <is>
           <t>⏭</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="n">
-        <v>0</v>
-      </c>
-      <c r="O11" t="n">
-        <v>50</v>
-      </c>
-      <c r="P11" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R11" t="inlineStr">
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W11" t="n">
+        <v>0</v>
+      </c>
+      <c r="X11" t="n">
+        <v>50</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>50</v>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA11" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-09-16 18:03
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA11"/>
+  <dimension ref="A1:AA15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -556,44 +556,44 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>8:40</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>Chicago Cubs</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Atlanta Braves</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>25</v>
+        <v>66</v>
       </c>
       <c r="F2" t="n">
-        <v>75</v>
+        <v>34</v>
       </c>
       <c r="G2" t="n">
-        <v>35</v>
+        <v>63.5</v>
       </c>
       <c r="H2" t="n">
-        <v>65</v>
+        <v>36.5</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2-5</t>
+          <t>7-4</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -602,111 +602,107 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>28.4</v>
+        <v>70</v>
       </c>
       <c r="M2" t="n">
-        <v>10.6</v>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>45.4</v>
+      </c>
+      <c r="N2" t="n">
+        <v>50.4</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="P2" t="n">
+        <v>31.5</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>⏭</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr"/>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>확률·표본·모델합의 기준 미달</t>
+          <t>Forebet·과거모델 합의</t>
         </is>
       </c>
       <c r="V2" t="n">
-        <v>0</v>
+        <v>45.13</v>
       </c>
       <c r="W2" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="X2" t="n">
-        <v>50</v>
+        <v>59.8</v>
       </c>
       <c r="Y2" t="n">
-        <v>50</v>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>40.2</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>43.8</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>26.9</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>9:40</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Chiba Lotte Marines</t>
+          <t>Colorado Rockies</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Rakuten Gold. Eagles</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>54</v>
+        <v>30</v>
       </c>
       <c r="F3" t="n">
-        <v>46</v>
+        <v>70</v>
       </c>
       <c r="G3" t="n">
-        <v>52.4</v>
+        <v>36.9</v>
       </c>
       <c r="H3" t="n">
-        <v>47.6</v>
+        <v>63.1</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>4-8</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -715,25 +711,21 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>42.1</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="M3" t="n">
-        <v>19.4</v>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>62.1</v>
+      </c>
+      <c r="N3" t="n">
+        <v>64.7</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>오버</t>
+        </is>
+      </c>
+      <c r="P3" t="n">
+        <v>45.6</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -742,41 +734,41 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>⏭</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr"/>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>확률·표본·모델합의 기준 미달</t>
+          <t>Forebet·과거모델 합의</t>
         </is>
       </c>
       <c r="V3" t="n">
-        <v>0</v>
+        <v>38.02</v>
       </c>
       <c r="W3" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="X3" t="n">
-        <v>50</v>
+        <v>47.2</v>
       </c>
       <c r="Y3" t="n">
-        <v>50</v>
-      </c>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AA3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>52.8</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>58.8</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>40.1</v>
       </c>
     </row>
     <row r="4">
@@ -787,12 +779,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>LG Twins</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -801,20 +793,20 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="F4" t="n">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="G4" t="n">
-        <v>39.8</v>
+        <v>42.4</v>
       </c>
       <c r="H4" t="n">
-        <v>60.2</v>
+        <v>57.6</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>4-6</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -828,29 +820,25 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>55.7</v>
+        <v>49.1</v>
       </c>
       <c r="M4" t="n">
-        <v>30.6</v>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>24.8</v>
+      </c>
+      <c r="N4" t="n">
+        <v>51.5</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="P4" t="n">
+        <v>33.2</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -870,69 +858,65 @@
         </is>
       </c>
       <c r="V4" t="n">
-        <v>0</v>
+        <v>42.65</v>
       </c>
       <c r="W4" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="X4" t="n">
-        <v>50</v>
+        <v>40.1</v>
       </c>
       <c r="Y4" t="n">
-        <v>50</v>
-      </c>
-      <c r="Z4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AA4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>59.9</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>52.3</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>35.9</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>7:40</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Lotte Giants</t>
+          <t>Tampa Bay Rays</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>Athletics</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="F5" t="n">
-        <v>64</v>
+        <v>41</v>
       </c>
       <c r="G5" t="n">
-        <v>41.6</v>
+        <v>56.8</v>
       </c>
       <c r="H5" t="n">
-        <v>58.4</v>
+        <v>43.2</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -941,25 +925,21 @@
         </is>
       </c>
       <c r="L5" t="n">
-        <v>46.3</v>
+        <v>55.7</v>
       </c>
       <c r="M5" t="n">
-        <v>22.6</v>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>30.6</v>
+      </c>
+      <c r="N5" t="n">
+        <v>55.7</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="P5" t="n">
+        <v>41</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -983,64 +963,60 @@
         </is>
       </c>
       <c r="V5" t="n">
-        <v>0</v>
+        <v>43.59</v>
       </c>
       <c r="W5" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="X5" t="n">
-        <v>50</v>
+        <v>53.5</v>
       </c>
       <c r="Y5" t="n">
-        <v>50</v>
-      </c>
-      <c r="Z5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AA5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>46.5</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>55.7</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>44.5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>7:40</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>KT Wiz Suwon</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F6" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G6" t="n">
-        <v>46.4</v>
+        <v>44.6</v>
       </c>
       <c r="H6" t="n">
-        <v>53.6</v>
+        <v>55.4</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>4-6</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -1054,29 +1030,25 @@
         </is>
       </c>
       <c r="L6" t="n">
-        <v>49.1</v>
+        <v>40.7</v>
       </c>
       <c r="M6" t="n">
-        <v>24.8</v>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>18.4</v>
+      </c>
+      <c r="N6" t="n">
+        <v>53.5</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="P6" t="n">
+        <v>34.9</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -1096,47 +1068,43 @@
         </is>
       </c>
       <c r="V6" t="n">
-        <v>0</v>
+        <v>41.9</v>
       </c>
       <c r="W6" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="X6" t="n">
-        <v>50</v>
+        <v>47.1</v>
       </c>
       <c r="Y6" t="n">
-        <v>50</v>
-      </c>
-      <c r="Z6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AA6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>52.9</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>40.5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>7:45</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>Washington Nationals</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>Philadelphia Phillies</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -1146,10 +1114,10 @@
         <v>54</v>
       </c>
       <c r="G7" t="n">
-        <v>47.6</v>
+        <v>48.9</v>
       </c>
       <c r="H7" t="n">
-        <v>52.4</v>
+        <v>51.1</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -1172,24 +1140,20 @@
       <c r="M7" t="n">
         <v>28.2</v>
       </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="N7" t="n">
+        <v>51.7</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="P7" t="n">
+        <v>32.7</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1209,42 +1173,38 @@
         </is>
       </c>
       <c r="V7" t="n">
-        <v>0</v>
+        <v>44.87</v>
       </c>
       <c r="W7" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="X7" t="n">
-        <v>50</v>
+        <v>53.2</v>
       </c>
       <c r="Y7" t="n">
-        <v>50</v>
-      </c>
-      <c r="Z7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AA7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>46.8</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>51.3</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>34.2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>8:07</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Athletics</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1253,25 +1213,25 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="F8" t="n">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="G8" t="n">
+        <v>44.6</v>
+      </c>
+      <c r="H8" t="n">
         <v>55.4</v>
       </c>
-      <c r="H8" t="n">
-        <v>44.6</v>
-      </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1280,29 +1240,25 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>55.7</v>
+        <v>29.7</v>
       </c>
       <c r="M8" t="n">
-        <v>30.6</v>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>11.3</v>
+      </c>
+      <c r="N8" t="n">
+        <v>43.8</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="P8" t="n">
+        <v>29.9</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -1322,42 +1278,38 @@
         </is>
       </c>
       <c r="V8" t="n">
-        <v>0</v>
+        <v>41.85</v>
       </c>
       <c r="W8" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="X8" t="n">
-        <v>50</v>
+        <v>47.1</v>
       </c>
       <c r="Y8" t="n">
-        <v>50</v>
-      </c>
-      <c r="Z8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AA8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>52.9</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>36</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>8:10</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Cincinnati Reds</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1366,20 +1318,20 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="F9" t="n">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G9" t="n">
-        <v>44.6</v>
+        <v>43.8</v>
       </c>
       <c r="H9" t="n">
-        <v>55.4</v>
+        <v>56.2</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>4-6</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1393,29 +1345,25 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>42.1</v>
+        <v>29.7</v>
       </c>
       <c r="M9" t="n">
-        <v>19.4</v>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>11.3</v>
+      </c>
+      <c r="N9" t="n">
+        <v>43.8</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="P9" t="n">
+        <v>29.9</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -1435,42 +1383,38 @@
         </is>
       </c>
       <c r="V9" t="n">
-        <v>0</v>
+        <v>43.05</v>
       </c>
       <c r="W9" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="X9" t="n">
-        <v>50</v>
+        <v>43.5</v>
       </c>
       <c r="Y9" t="n">
-        <v>50</v>
-      </c>
-      <c r="Z9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AA9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>56.5</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>36</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>8:40</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1479,16 +1423,16 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="F10" t="n">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="G10" t="n">
-        <v>45.8</v>
+        <v>39.6</v>
       </c>
       <c r="H10" t="n">
-        <v>54.2</v>
+        <v>60.4</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -1506,29 +1450,25 @@
         </is>
       </c>
       <c r="L10" t="n">
-        <v>40.7</v>
+        <v>42.1</v>
       </c>
       <c r="M10" t="n">
-        <v>18.4</v>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>19.4</v>
+      </c>
+      <c r="N10" t="n">
+        <v>56.3</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="P10" t="n">
+        <v>35.2</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -1548,42 +1488,38 @@
         </is>
       </c>
       <c r="V10" t="n">
-        <v>0</v>
+        <v>40.84</v>
       </c>
       <c r="W10" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="X10" t="n">
-        <v>50</v>
+        <v>44.9</v>
       </c>
       <c r="Y10" t="n">
-        <v>50</v>
-      </c>
-      <c r="Z10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AA10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>55.1</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>61</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>40.5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>8:45</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Cleveland Guardians</t>
+          <t>St.Louis Cardinals</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>San Francisco Giants</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1592,16 +1528,16 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F11" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G11" t="n">
-        <v>54.2</v>
+        <v>55.9</v>
       </c>
       <c r="H11" t="n">
-        <v>45.8</v>
+        <v>44.1</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -1619,29 +1555,25 @@
         </is>
       </c>
       <c r="L11" t="n">
-        <v>29.7</v>
+        <v>32.4</v>
       </c>
       <c r="M11" t="n">
-        <v>11.3</v>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>12.9</v>
+      </c>
+      <c r="N11" t="n">
+        <v>47.4</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="P11" t="n">
+        <v>36.8</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -1661,26 +1593,442 @@
         </is>
       </c>
       <c r="V11" t="n">
-        <v>0</v>
+        <v>44.18</v>
       </c>
       <c r="W11" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="X11" t="n">
-        <v>50</v>
+        <v>52.8</v>
       </c>
       <c r="Y11" t="n">
-        <v>50</v>
-      </c>
-      <c r="Z11" t="inlineStr">
+        <v>47.2</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>52.4</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>44.8</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>9:05</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Texas Rangers</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Boston Red Sox</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>56</v>
+      </c>
+      <c r="F12" t="n">
+        <v>44</v>
+      </c>
+      <c r="G12" t="n">
+        <v>56.5</v>
+      </c>
+      <c r="H12" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AA11" t="inlineStr">
+      <c r="L12" t="n">
+        <v>42.1</v>
+      </c>
+      <c r="M12" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="N12" t="n">
+        <v>56.3</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P12" t="n">
+        <v>35.2</v>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>언더</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V12" t="n">
+        <v>46.46</v>
+      </c>
+      <c r="W12" t="n">
+        <v>60</v>
+      </c>
+      <c r="X12" t="n">
+        <v>57.2</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>42.8</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>61.1</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>40.5</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>9:10</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Houston Astros</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Kansas City Royals</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>59</v>
+      </c>
+      <c r="F13" t="n">
+        <v>41</v>
+      </c>
+      <c r="G13" t="n">
+        <v>56.8</v>
+      </c>
+      <c r="H13" t="n">
+        <v>43.2</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
         <is>
           <t>-</t>
         </is>
+      </c>
+      <c r="L13" t="n">
+        <v>38</v>
+      </c>
+      <c r="M13" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="N13" t="n">
+        <v>49.3</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P13" t="n">
+        <v>32.7</v>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>언더</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V13" t="n">
+        <v>43.47</v>
+      </c>
+      <c r="W13" t="n">
+        <v>60</v>
+      </c>
+      <c r="X13" t="n">
+        <v>53.5</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>53</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>38.2</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>10:38</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Los Angeles Angels</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>52</v>
+      </c>
+      <c r="F14" t="n">
+        <v>48</v>
+      </c>
+      <c r="G14" t="n">
+        <v>50.3</v>
+      </c>
+      <c r="H14" t="n">
+        <v>49.7</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L14" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="M14" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="N14" t="n">
+        <v>46.8</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P14" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>언더</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V14" t="n">
+        <v>41.15</v>
+      </c>
+      <c r="W14" t="n">
+        <v>60</v>
+      </c>
+      <c r="X14" t="n">
+        <v>47.8</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>52.2</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>52.1</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Miami Marlins</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>49</v>
+      </c>
+      <c r="F15" t="n">
+        <v>51</v>
+      </c>
+      <c r="G15" t="n">
+        <v>51.8</v>
+      </c>
+      <c r="H15" t="n">
+        <v>48.2</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>6-8</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L15" t="n">
+        <v>80.90000000000001</v>
+      </c>
+      <c r="M15" t="n">
+        <v>59.8</v>
+      </c>
+      <c r="N15" t="n">
+        <v>63.6</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>오버</t>
+        </is>
+      </c>
+      <c r="P15" t="n">
+        <v>44</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V15" t="n">
+        <v>44.61</v>
+      </c>
+      <c r="W15" t="n">
+        <v>60</v>
+      </c>
+      <c r="X15" t="n">
+        <v>56.1</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>57.9</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>38.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-09-17 14:20
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA15"/>
+  <dimension ref="A1:AA12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -556,44 +556,44 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Atlanta Braves</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>66</v>
+        <v>30</v>
       </c>
       <c r="F2" t="n">
-        <v>34</v>
+        <v>70</v>
       </c>
       <c r="G2" t="n">
-        <v>63.5</v>
+        <v>35.6</v>
       </c>
       <c r="H2" t="n">
-        <v>36.5</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>7-4</t>
+          <t>1-3</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -602,21 +602,21 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>70</v>
+        <v>5</v>
       </c>
       <c r="M2" t="n">
-        <v>45.4</v>
+        <v>0.9</v>
       </c>
       <c r="N2" t="n">
-        <v>50.4</v>
+        <v>28.1</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>31.5</v>
+        <v>10.3</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -635,7 +635,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -644,65 +644,65 @@
         </is>
       </c>
       <c r="V2" t="n">
-        <v>45.13</v>
+        <v>30.34</v>
       </c>
       <c r="W2" t="n">
         <v>60</v>
       </c>
       <c r="X2" t="n">
-        <v>59.8</v>
+        <v>44.1</v>
       </c>
       <c r="Y2" t="n">
-        <v>40.2</v>
+        <v>55.9</v>
       </c>
       <c r="Z2" t="n">
-        <v>43.8</v>
+        <v>35.8</v>
       </c>
       <c r="AA2" t="n">
-        <v>26.9</v>
+        <v>13.4</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>9:40</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>30</v>
+        <v>59</v>
       </c>
       <c r="F3" t="n">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="G3" t="n">
-        <v>36.9</v>
+        <v>58.2</v>
       </c>
       <c r="H3" t="n">
-        <v>63.1</v>
+        <v>41.8</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>4-8</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -711,107 +711,103 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>82.40000000000001</v>
+        <v>16.3</v>
       </c>
       <c r="M3" t="n">
-        <v>62.1</v>
+        <v>4.7</v>
       </c>
       <c r="N3" t="n">
-        <v>64.7</v>
+        <v>29.1</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>오버</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>45.6</v>
+        <v>16.2</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
+          <t>언더</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>★★</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>원정승</t>
-        </is>
-      </c>
+      <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Forebet·과거모델 합의</t>
+          <t>확률·표본·모델합의 기준 미달</t>
         </is>
       </c>
       <c r="V3" t="n">
-        <v>38.02</v>
+        <v>40.99</v>
       </c>
       <c r="W3" t="n">
         <v>60</v>
       </c>
       <c r="X3" t="n">
-        <v>47.2</v>
+        <v>57.1</v>
       </c>
       <c r="Y3" t="n">
-        <v>52.8</v>
+        <v>42.9</v>
       </c>
       <c r="Z3" t="n">
-        <v>58.8</v>
+        <v>33.3</v>
       </c>
       <c r="AA3" t="n">
-        <v>40.1</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>KT Wiz Suwon</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E4" t="n">
+        <v>56</v>
+      </c>
+      <c r="F4" t="n">
         <v>44</v>
       </c>
-      <c r="F4" t="n">
-        <v>56</v>
-      </c>
       <c r="G4" t="n">
-        <v>42.4</v>
+        <v>57.8</v>
       </c>
       <c r="H4" t="n">
-        <v>57.6</v>
+        <v>42.2</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>4-6</t>
+          <t>3-1</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -820,21 +816,21 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>49.1</v>
+        <v>3.2</v>
       </c>
       <c r="M4" t="n">
-        <v>24.8</v>
+        <v>0.5</v>
       </c>
       <c r="N4" t="n">
-        <v>51.5</v>
+        <v>26.6</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>33.2</v>
+        <v>9.4</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -858,65 +854,65 @@
         </is>
       </c>
       <c r="V4" t="n">
-        <v>42.65</v>
+        <v>42.05</v>
       </c>
       <c r="W4" t="n">
         <v>60</v>
       </c>
       <c r="X4" t="n">
-        <v>40.1</v>
+        <v>60.4</v>
       </c>
       <c r="Y4" t="n">
-        <v>59.9</v>
+        <v>39.6</v>
       </c>
       <c r="Z4" t="n">
-        <v>52.3</v>
+        <v>34.4</v>
       </c>
       <c r="AA4" t="n">
-        <v>35.9</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Athletics</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="F5" t="n">
-        <v>41</v>
+        <v>61</v>
       </c>
       <c r="G5" t="n">
-        <v>56.8</v>
+        <v>42.2</v>
       </c>
       <c r="H5" t="n">
-        <v>43.2</v>
+        <v>57.8</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -925,25 +921,25 @@
         </is>
       </c>
       <c r="L5" t="n">
-        <v>55.7</v>
+        <v>38</v>
       </c>
       <c r="M5" t="n">
-        <v>30.6</v>
+        <v>16.5</v>
       </c>
       <c r="N5" t="n">
-        <v>55.7</v>
+        <v>35.7</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>41</v>
+        <v>21.9</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -963,65 +959,65 @@
         </is>
       </c>
       <c r="V5" t="n">
-        <v>43.59</v>
+        <v>38.97</v>
       </c>
       <c r="W5" t="n">
         <v>60</v>
       </c>
       <c r="X5" t="n">
-        <v>53.5</v>
+        <v>47</v>
       </c>
       <c r="Y5" t="n">
-        <v>46.5</v>
+        <v>53</v>
       </c>
       <c r="Z5" t="n">
-        <v>55.7</v>
+        <v>34.9</v>
       </c>
       <c r="AA5" t="n">
-        <v>44.5</v>
+        <v>23.6</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>43</v>
+        <v>58</v>
       </c>
       <c r="F6" t="n">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="G6" t="n">
-        <v>44.6</v>
+        <v>57.5</v>
       </c>
       <c r="H6" t="n">
-        <v>55.4</v>
+        <v>42.5</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -1036,15 +1032,15 @@
         <v>18.4</v>
       </c>
       <c r="N6" t="n">
-        <v>53.5</v>
+        <v>36.8</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>34.9</v>
+        <v>22</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1068,43 +1064,43 @@
         </is>
       </c>
       <c r="V6" t="n">
-        <v>41.9</v>
+        <v>40.92</v>
       </c>
       <c r="W6" t="n">
         <v>60</v>
       </c>
       <c r="X6" t="n">
-        <v>47.1</v>
+        <v>56.8</v>
       </c>
       <c r="Y6" t="n">
-        <v>52.9</v>
+        <v>43.2</v>
       </c>
       <c r="Z6" t="n">
-        <v>57.7</v>
+        <v>35.5</v>
       </c>
       <c r="AA6" t="n">
-        <v>40.5</v>
+        <v>23.2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>7:45</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Washington Nationals</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -1114,14 +1110,14 @@
         <v>54</v>
       </c>
       <c r="G7" t="n">
-        <v>48.9</v>
+        <v>42.5</v>
       </c>
       <c r="H7" t="n">
-        <v>51.1</v>
+        <v>57.5</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1135,13 +1131,13 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>53.1</v>
+        <v>31.1</v>
       </c>
       <c r="M7" t="n">
-        <v>28.2</v>
+        <v>12.1</v>
       </c>
       <c r="N7" t="n">
-        <v>51.7</v>
+        <v>41.7</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1149,7 +1145,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>32.7</v>
+        <v>25.3</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1173,65 +1169,65 @@
         </is>
       </c>
       <c r="V7" t="n">
-        <v>44.87</v>
+        <v>42.03</v>
       </c>
       <c r="W7" t="n">
         <v>60</v>
       </c>
       <c r="X7" t="n">
-        <v>53.2</v>
+        <v>37.2</v>
       </c>
       <c r="Y7" t="n">
-        <v>46.8</v>
+        <v>62.8</v>
       </c>
       <c r="Z7" t="n">
-        <v>51.3</v>
+        <v>45.3</v>
       </c>
       <c r="AA7" t="n">
-        <v>34.2</v>
+        <v>29.7</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>8:07</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Toronto Blue Jays</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E8" t="n">
+        <v>57</v>
+      </c>
+      <c r="F8" t="n">
         <v>43</v>
       </c>
-      <c r="F8" t="n">
-        <v>57</v>
-      </c>
       <c r="G8" t="n">
-        <v>44.6</v>
+        <v>56.8</v>
       </c>
       <c r="H8" t="n">
-        <v>55.4</v>
+        <v>43.2</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>7-6</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1240,25 +1236,25 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>29.7</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="M8" t="n">
-        <v>11.3</v>
+        <v>68.3</v>
       </c>
       <c r="N8" t="n">
-        <v>43.8</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
+          <t>오버</t>
+        </is>
+      </c>
+      <c r="P8" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
           <t>PASS</t>
-        </is>
-      </c>
-      <c r="P8" t="n">
-        <v>29.9</v>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>언더</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -1278,38 +1274,38 @@
         </is>
       </c>
       <c r="V8" t="n">
-        <v>41.85</v>
+        <v>42.35</v>
       </c>
       <c r="W8" t="n">
         <v>60</v>
       </c>
       <c r="X8" t="n">
-        <v>47.1</v>
+        <v>56.5</v>
       </c>
       <c r="Y8" t="n">
-        <v>52.9</v>
+        <v>43.5</v>
       </c>
       <c r="Z8" t="n">
-        <v>48.5</v>
+        <v>59.9</v>
       </c>
       <c r="AA8" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>7:40</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>Cincinnati Reds</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>Los Angeles Dodgers</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1318,16 +1314,16 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="F9" t="n">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="G9" t="n">
-        <v>43.8</v>
+        <v>43.2</v>
       </c>
       <c r="H9" t="n">
-        <v>56.2</v>
+        <v>56.8</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -1345,13 +1341,13 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>29.7</v>
+        <v>31.1</v>
       </c>
       <c r="M9" t="n">
-        <v>11.3</v>
+        <v>12.1</v>
       </c>
       <c r="N9" t="n">
-        <v>43.8</v>
+        <v>47.6</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1359,7 +1355,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>29.9</v>
+        <v>35.1</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1383,38 +1379,38 @@
         </is>
       </c>
       <c r="V9" t="n">
-        <v>43.05</v>
+        <v>42.11</v>
       </c>
       <c r="W9" t="n">
         <v>60</v>
       </c>
       <c r="X9" t="n">
-        <v>43.5</v>
+        <v>48</v>
       </c>
       <c r="Y9" t="n">
-        <v>56.5</v>
+        <v>52</v>
       </c>
       <c r="Z9" t="n">
-        <v>48.5</v>
+        <v>53.1</v>
       </c>
       <c r="AA9" t="n">
-        <v>36</v>
+        <v>42.8</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>7:40</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>Pittsburgh Pirates</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1423,20 +1419,20 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="F10" t="n">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="G10" t="n">
-        <v>39.6</v>
+        <v>49.5</v>
       </c>
       <c r="H10" t="n">
-        <v>60.4</v>
+        <v>50.5</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1450,13 +1446,13 @@
         </is>
       </c>
       <c r="L10" t="n">
-        <v>42.1</v>
+        <v>53.1</v>
       </c>
       <c r="M10" t="n">
-        <v>19.4</v>
+        <v>28.2</v>
       </c>
       <c r="N10" t="n">
-        <v>56.3</v>
+        <v>53.9</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1464,7 +1460,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>35.2</v>
+        <v>30.7</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1488,38 +1484,38 @@
         </is>
       </c>
       <c r="V10" t="n">
-        <v>40.84</v>
+        <v>44.62</v>
       </c>
       <c r="W10" t="n">
         <v>60</v>
       </c>
       <c r="X10" t="n">
-        <v>44.9</v>
+        <v>53.2</v>
       </c>
       <c r="Y10" t="n">
-        <v>55.1</v>
+        <v>46.8</v>
       </c>
       <c r="Z10" t="n">
-        <v>61</v>
+        <v>54.1</v>
       </c>
       <c r="AA10" t="n">
-        <v>40.5</v>
+        <v>31.6</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>8:45</t>
+          <t>7:40</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>St.Louis Cardinals</t>
+          <t>Tampa Bay Rays</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>San Francisco Giants</t>
+          <t>Athletics</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1528,20 +1524,20 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>58</v>
+        <v>53.5</v>
       </c>
       <c r="F11" t="n">
-        <v>42</v>
+        <v>46.5</v>
       </c>
       <c r="G11" t="n">
-        <v>55.9</v>
+        <v>49.9</v>
       </c>
       <c r="H11" t="n">
-        <v>44.1</v>
+        <v>50.1</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1555,13 +1551,13 @@
         </is>
       </c>
       <c r="L11" t="n">
-        <v>32.4</v>
+        <v>55.7</v>
       </c>
       <c r="M11" t="n">
-        <v>12.9</v>
+        <v>30.6</v>
       </c>
       <c r="N11" t="n">
-        <v>47.4</v>
+        <v>54.5</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1569,11 +1565,11 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>36.8</v>
+        <v>39.7</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>언더</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -1593,38 +1589,38 @@
         </is>
       </c>
       <c r="V11" t="n">
-        <v>44.18</v>
+        <v>43.88</v>
       </c>
       <c r="W11" t="n">
         <v>60</v>
       </c>
       <c r="X11" t="n">
-        <v>52.8</v>
+        <v>44.5</v>
       </c>
       <c r="Y11" t="n">
-        <v>47.2</v>
+        <v>55.5</v>
       </c>
       <c r="Z11" t="n">
-        <v>52.4</v>
+        <v>54.1</v>
       </c>
       <c r="AA11" t="n">
-        <v>44.8</v>
+        <v>42.8</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>9:05</t>
+          <t>7:45</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>Washington Nationals</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Boston Red Sox</t>
+          <t>Philadelphia Phillies</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1633,25 +1629,25 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="F12" t="n">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="G12" t="n">
-        <v>56.5</v>
+        <v>44.2</v>
       </c>
       <c r="H12" t="n">
-        <v>43.5</v>
+        <v>55.8</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>4-6</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1660,13 +1656,13 @@
         </is>
       </c>
       <c r="L12" t="n">
-        <v>42.1</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="M12" t="n">
-        <v>19.4</v>
+        <v>39.2</v>
       </c>
       <c r="N12" t="n">
-        <v>56.3</v>
+        <v>54.2</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1674,7 +1670,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>35.2</v>
+        <v>35.1</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1698,337 +1694,22 @@
         </is>
       </c>
       <c r="V12" t="n">
-        <v>46.46</v>
+        <v>42.55</v>
       </c>
       <c r="W12" t="n">
         <v>60</v>
       </c>
       <c r="X12" t="n">
-        <v>57.2</v>
+        <v>45.9</v>
       </c>
       <c r="Y12" t="n">
-        <v>42.8</v>
+        <v>54.1</v>
       </c>
       <c r="Z12" t="n">
-        <v>61.1</v>
+        <v>50.8</v>
       </c>
       <c r="AA12" t="n">
-        <v>40.5</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>9:10</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Houston Astros</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Kansas City Royals</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>59</v>
-      </c>
-      <c r="F13" t="n">
-        <v>41</v>
-      </c>
-      <c r="G13" t="n">
-        <v>56.8</v>
-      </c>
-      <c r="H13" t="n">
-        <v>43.2</v>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>5-4</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L13" t="n">
-        <v>38</v>
-      </c>
-      <c r="M13" t="n">
-        <v>16.5</v>
-      </c>
-      <c r="N13" t="n">
-        <v>49.3</v>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="P13" t="n">
-        <v>32.7</v>
-      </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>언더</t>
-        </is>
-      </c>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>⏭</t>
-        </is>
-      </c>
-      <c r="S13" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="T13" t="inlineStr"/>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>확률·표본·모델합의 기준 미달</t>
-        </is>
-      </c>
-      <c r="V13" t="n">
-        <v>43.47</v>
-      </c>
-      <c r="W13" t="n">
-        <v>60</v>
-      </c>
-      <c r="X13" t="n">
-        <v>53.5</v>
-      </c>
-      <c r="Y13" t="n">
-        <v>46.5</v>
-      </c>
-      <c r="Z13" t="n">
-        <v>53</v>
-      </c>
-      <c r="AA13" t="n">
-        <v>38.2</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>10:38</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Los Angeles Angels</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Seattle Mariners</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>52</v>
-      </c>
-      <c r="F14" t="n">
-        <v>48</v>
-      </c>
-      <c r="G14" t="n">
-        <v>50.3</v>
-      </c>
-      <c r="H14" t="n">
-        <v>49.7</v>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>4-3</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L14" t="n">
-        <v>31.1</v>
-      </c>
-      <c r="M14" t="n">
-        <v>12.1</v>
-      </c>
-      <c r="N14" t="n">
-        <v>46.8</v>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="P14" t="n">
-        <v>35.3</v>
-      </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>언더</t>
-        </is>
-      </c>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>⏭</t>
-        </is>
-      </c>
-      <c r="S14" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="T14" t="inlineStr"/>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>확률·표본·모델합의 기준 미달</t>
-        </is>
-      </c>
-      <c r="V14" t="n">
-        <v>41.15</v>
-      </c>
-      <c r="W14" t="n">
-        <v>60</v>
-      </c>
-      <c r="X14" t="n">
-        <v>47.8</v>
-      </c>
-      <c r="Y14" t="n">
-        <v>52.2</v>
-      </c>
-      <c r="Z14" t="n">
-        <v>52.1</v>
-      </c>
-      <c r="AA14" t="n">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>10:40</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Arizona Diamondbacks</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Miami Marlins</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>49</v>
-      </c>
-      <c r="F15" t="n">
-        <v>51</v>
-      </c>
-      <c r="G15" t="n">
-        <v>51.8</v>
-      </c>
-      <c r="H15" t="n">
-        <v>48.2</v>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>6-8</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L15" t="n">
-        <v>80.90000000000001</v>
-      </c>
-      <c r="M15" t="n">
-        <v>59.8</v>
-      </c>
-      <c r="N15" t="n">
-        <v>63.6</v>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>오버</t>
-        </is>
-      </c>
-      <c r="P15" t="n">
-        <v>44</v>
-      </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>⏭</t>
-        </is>
-      </c>
-      <c r="S15" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="T15" t="inlineStr"/>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>확률·표본·모델합의 기준 미달</t>
-        </is>
-      </c>
-      <c r="V15" t="n">
-        <v>44.61</v>
-      </c>
-      <c r="W15" t="n">
-        <v>60</v>
-      </c>
-      <c r="X15" t="n">
-        <v>56.1</v>
-      </c>
-      <c r="Y15" t="n">
-        <v>43.9</v>
-      </c>
-      <c r="Z15" t="n">
-        <v>57.9</v>
-      </c>
-      <c r="AA15" t="n">
-        <v>38.8</v>
+        <v>33.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-09-18 14:19
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -556,22 +556,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>4:10</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>Colorado Rockies</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -581,14 +581,14 @@
         <v>70</v>
       </c>
       <c r="G2" t="n">
-        <v>35.6</v>
+        <v>37</v>
       </c>
       <c r="H2" t="n">
-        <v>64.40000000000001</v>
+        <v>63</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>1-3</t>
+          <t>3-8</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -602,25 +602,25 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>5</v>
+        <v>76.8</v>
       </c>
       <c r="M2" t="n">
-        <v>0.9</v>
+        <v>54</v>
       </c>
       <c r="N2" t="n">
-        <v>28.1</v>
+        <v>61.1</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>언더</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>10.3</v>
+        <v>39.2</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>언더</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -644,22 +644,22 @@
         </is>
       </c>
       <c r="V2" t="n">
-        <v>30.34</v>
+        <v>38.51</v>
       </c>
       <c r="W2" t="n">
         <v>60</v>
       </c>
       <c r="X2" t="n">
-        <v>44.1</v>
+        <v>47.6</v>
       </c>
       <c r="Y2" t="n">
+        <v>52.4</v>
+      </c>
+      <c r="Z2" t="n">
         <v>55.9</v>
       </c>
-      <c r="Z2" t="n">
-        <v>35.8</v>
-      </c>
       <c r="AA2" t="n">
-        <v>13.4</v>
+        <v>34.3</v>
       </c>
     </row>
     <row r="3">
@@ -670,12 +670,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Nippon Ham Fighters</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Seibu Lions</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -684,20 +684,20 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="F3" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="G3" t="n">
-        <v>58.2</v>
+        <v>58.7</v>
       </c>
       <c r="H3" t="n">
-        <v>41.8</v>
+        <v>41.3</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>16.2</v>
+        <v>16</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -749,22 +749,22 @@
         </is>
       </c>
       <c r="V3" t="n">
-        <v>40.99</v>
+        <v>41.32</v>
       </c>
       <c r="W3" t="n">
         <v>60</v>
       </c>
       <c r="X3" t="n">
-        <v>57.1</v>
+        <v>53.8</v>
       </c>
       <c r="Y3" t="n">
-        <v>42.9</v>
+        <v>46.2</v>
       </c>
       <c r="Z3" t="n">
-        <v>33.3</v>
+        <v>33.4</v>
       </c>
       <c r="AA3" t="n">
-        <v>20</v>
+        <v>19.7</v>
       </c>
     </row>
     <row r="4">
@@ -775,12 +775,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -789,20 +789,20 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="F4" t="n">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="G4" t="n">
-        <v>57.8</v>
+        <v>58.7</v>
       </c>
       <c r="H4" t="n">
-        <v>42.2</v>
+        <v>41.3</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>3-1</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -816,13 +816,13 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>3.2</v>
+        <v>14.3</v>
       </c>
       <c r="M4" t="n">
-        <v>0.5</v>
+        <v>3.9</v>
       </c>
       <c r="N4" t="n">
-        <v>26.6</v>
+        <v>24.4</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -830,7 +830,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>9.4</v>
+        <v>13.4</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -854,22 +854,22 @@
         </is>
       </c>
       <c r="V4" t="n">
-        <v>42.05</v>
+        <v>41.32</v>
       </c>
       <c r="W4" t="n">
         <v>60</v>
       </c>
       <c r="X4" t="n">
-        <v>60.4</v>
+        <v>53.8</v>
       </c>
       <c r="Y4" t="n">
-        <v>39.6</v>
+        <v>46.2</v>
       </c>
       <c r="Z4" t="n">
-        <v>34.4</v>
+        <v>27.8</v>
       </c>
       <c r="AA4" t="n">
-        <v>12.4</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="5">
@@ -880,12 +880,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -894,25 +894,25 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>39</v>
+        <v>58</v>
       </c>
       <c r="F5" t="n">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="G5" t="n">
-        <v>42.2</v>
+        <v>57.5</v>
       </c>
       <c r="H5" t="n">
-        <v>57.8</v>
+        <v>42.5</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -921,13 +921,13 @@
         </is>
       </c>
       <c r="L5" t="n">
-        <v>38</v>
+        <v>7.5</v>
       </c>
       <c r="M5" t="n">
-        <v>16.5</v>
+        <v>1.6</v>
       </c>
       <c r="N5" t="n">
-        <v>35.7</v>
+        <v>24.6</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -935,7 +935,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>21.9</v>
+        <v>13</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -959,65 +959,65 @@
         </is>
       </c>
       <c r="V5" t="n">
-        <v>38.97</v>
+        <v>41.68</v>
       </c>
       <c r="W5" t="n">
         <v>60</v>
       </c>
       <c r="X5" t="n">
-        <v>47</v>
+        <v>56.8</v>
       </c>
       <c r="Y5" t="n">
-        <v>53</v>
+        <v>43.2</v>
       </c>
       <c r="Z5" t="n">
-        <v>34.9</v>
+        <v>30.2</v>
       </c>
       <c r="AA5" t="n">
-        <v>23.6</v>
+        <v>16.8</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Chiba Lotte Marines</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Rakuten Gold. Eagles</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>58</v>
+        <v>44</v>
       </c>
       <c r="F6" t="n">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="G6" t="n">
-        <v>57.5</v>
+        <v>41.2</v>
       </c>
       <c r="H6" t="n">
-        <v>42.5</v>
+        <v>58.8</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>5-6</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -1026,25 +1026,25 @@
         </is>
       </c>
       <c r="L6" t="n">
-        <v>40.7</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="M6" t="n">
-        <v>18.4</v>
+        <v>40.4</v>
       </c>
       <c r="N6" t="n">
-        <v>36.8</v>
+        <v>56.9</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>언더</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>22</v>
+        <v>39.7</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>언더</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -1064,22 +1064,22 @@
         </is>
       </c>
       <c r="V6" t="n">
-        <v>40.92</v>
+        <v>42.4</v>
       </c>
       <c r="W6" t="n">
         <v>60</v>
       </c>
       <c r="X6" t="n">
-        <v>56.8</v>
+        <v>36.9</v>
       </c>
       <c r="Y6" t="n">
-        <v>43.2</v>
+        <v>63.1</v>
       </c>
       <c r="Z6" t="n">
-        <v>35.5</v>
+        <v>54</v>
       </c>
       <c r="AA6" t="n">
-        <v>23.2</v>
+        <v>39.5</v>
       </c>
     </row>
     <row r="7">
@@ -1090,12 +1090,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1104,25 +1104,25 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="F7" t="n">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="G7" t="n">
-        <v>42.5</v>
+        <v>55.2</v>
       </c>
       <c r="H7" t="n">
-        <v>57.5</v>
+        <v>44.8</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -1131,13 +1131,13 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>31.1</v>
+        <v>23.3</v>
       </c>
       <c r="M7" t="n">
-        <v>12.1</v>
+        <v>7.9</v>
       </c>
       <c r="N7" t="n">
-        <v>41.7</v>
+        <v>40.6</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1145,7 +1145,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>25.3</v>
+        <v>26.4</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1169,22 +1169,22 @@
         </is>
       </c>
       <c r="V7" t="n">
-        <v>42.03</v>
+        <v>41.35</v>
       </c>
       <c r="W7" t="n">
         <v>60</v>
       </c>
       <c r="X7" t="n">
-        <v>37.2</v>
+        <v>55.5</v>
       </c>
       <c r="Y7" t="n">
-        <v>62.8</v>
+        <v>44.5</v>
       </c>
       <c r="Z7" t="n">
-        <v>45.3</v>
+        <v>46.4</v>
       </c>
       <c r="AA7" t="n">
-        <v>29.7</v>
+        <v>32.6</v>
       </c>
     </row>
     <row r="8">
@@ -1195,12 +1195,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>Lotte Giants</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1209,48 +1209,48 @@
         </is>
       </c>
       <c r="E8" t="n">
+        <v>48</v>
+      </c>
+      <c r="F8" t="n">
+        <v>52</v>
+      </c>
+      <c r="G8" t="n">
+        <v>45.7</v>
+      </c>
+      <c r="H8" t="n">
+        <v>54.3</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>4-5</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
         <v>57</v>
       </c>
-      <c r="F8" t="n">
-        <v>43</v>
-      </c>
-      <c r="G8" t="n">
-        <v>56.8</v>
-      </c>
-      <c r="H8" t="n">
-        <v>43.2</v>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>7-6</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L8" t="n">
-        <v>86.40000000000001</v>
-      </c>
       <c r="M8" t="n">
-        <v>68.3</v>
+        <v>31.8</v>
       </c>
       <c r="N8" t="n">
-        <v>66.59999999999999</v>
+        <v>57.7</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>오버</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>48.5</v>
+        <v>40.6</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1274,56 +1274,56 @@
         </is>
       </c>
       <c r="V8" t="n">
-        <v>42.35</v>
+        <v>39.88</v>
       </c>
       <c r="W8" t="n">
         <v>60</v>
       </c>
       <c r="X8" t="n">
-        <v>56.5</v>
+        <v>42.4</v>
       </c>
       <c r="Y8" t="n">
+        <v>57.6</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>58</v>
+      </c>
+      <c r="AA8" t="n">
         <v>43.5</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>59.9</v>
-      </c>
-      <c r="AA8" t="n">
-        <v>42</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Cincinnati Reds</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers</t>
+          <t>Samsung Lions</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="F9" t="n">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="G9" t="n">
-        <v>43.2</v>
+        <v>46.3</v>
       </c>
       <c r="H9" t="n">
-        <v>56.8</v>
+        <v>53.7</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -1341,13 +1341,13 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>31.1</v>
+        <v>36.6</v>
       </c>
       <c r="M9" t="n">
-        <v>12.1</v>
+        <v>15.5</v>
       </c>
       <c r="N9" t="n">
-        <v>47.6</v>
+        <v>45.5</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1355,7 +1355,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>35.1</v>
+        <v>29.7</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1379,38 +1379,38 @@
         </is>
       </c>
       <c r="V9" t="n">
-        <v>42.11</v>
+        <v>39.8</v>
       </c>
       <c r="W9" t="n">
         <v>60</v>
       </c>
       <c r="X9" t="n">
-        <v>48</v>
+        <v>42.2</v>
       </c>
       <c r="Y9" t="n">
-        <v>52</v>
+        <v>57.8</v>
       </c>
       <c r="Z9" t="n">
-        <v>53.1</v>
+        <v>48.5</v>
       </c>
       <c r="AA9" t="n">
-        <v>42.8</v>
+        <v>34.5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>8:15</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>Houston Astros</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Kansas City Royals</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1419,25 +1419,25 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="F10" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="G10" t="n">
-        <v>49.5</v>
+        <v>58</v>
       </c>
       <c r="H10" t="n">
-        <v>50.5</v>
+        <v>42</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>7-5</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1446,13 +1446,13 @@
         </is>
       </c>
       <c r="L10" t="n">
-        <v>53.1</v>
+        <v>59.6</v>
       </c>
       <c r="M10" t="n">
-        <v>28.2</v>
+        <v>34.2</v>
       </c>
       <c r="N10" t="n">
-        <v>53.9</v>
+        <v>54.8</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>30.7</v>
+        <v>37.4</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1484,38 +1484,38 @@
         </is>
       </c>
       <c r="V10" t="n">
-        <v>44.62</v>
+        <v>43.07</v>
       </c>
       <c r="W10" t="n">
         <v>60</v>
       </c>
       <c r="X10" t="n">
+        <v>56.6</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>43.4</v>
+      </c>
+      <c r="Z10" t="n">
         <v>53.2</v>
       </c>
-      <c r="Y10" t="n">
-        <v>46.8</v>
-      </c>
-      <c r="Z10" t="n">
-        <v>54.1</v>
-      </c>
       <c r="AA10" t="n">
-        <v>31.6</v>
+        <v>38.5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>8:40</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Athletics</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1524,52 +1524,52 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>53.5</v>
+        <v>51</v>
       </c>
       <c r="F11" t="n">
-        <v>46.5</v>
+        <v>49</v>
       </c>
       <c r="G11" t="n">
+        <v>51.3</v>
+      </c>
+      <c r="H11" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L11" t="n">
+        <v>32.4</v>
+      </c>
+      <c r="M11" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="N11" t="n">
         <v>49.9</v>
       </c>
-      <c r="H11" t="n">
-        <v>50.1</v>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>5-4</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L11" t="n">
-        <v>55.7</v>
-      </c>
-      <c r="M11" t="n">
-        <v>30.6</v>
-      </c>
-      <c r="N11" t="n">
-        <v>54.5</v>
-      </c>
       <c r="O11" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>39.7</v>
+        <v>35.2</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -1589,38 +1589,38 @@
         </is>
       </c>
       <c r="V11" t="n">
-        <v>43.88</v>
+        <v>41.97</v>
       </c>
       <c r="W11" t="n">
         <v>60</v>
       </c>
       <c r="X11" t="n">
-        <v>44.5</v>
+        <v>51.7</v>
       </c>
       <c r="Y11" t="n">
-        <v>55.5</v>
+        <v>48.3</v>
       </c>
       <c r="Z11" t="n">
-        <v>54.1</v>
+        <v>55.7</v>
       </c>
       <c r="AA11" t="n">
-        <v>42.8</v>
+        <v>42.6</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>7:45</t>
+          <t>9:05</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Washington Nationals</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies</t>
+          <t>Boston Red Sox</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1629,25 +1629,25 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="F12" t="n">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="G12" t="n">
-        <v>44.2</v>
+        <v>49.8</v>
       </c>
       <c r="H12" t="n">
-        <v>55.8</v>
+        <v>50.2</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>4-6</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1656,13 +1656,13 @@
         </is>
       </c>
       <c r="L12" t="n">
-        <v>64.40000000000001</v>
+        <v>42.1</v>
       </c>
       <c r="M12" t="n">
-        <v>39.2</v>
+        <v>19.4</v>
       </c>
       <c r="N12" t="n">
-        <v>54.2</v>
+        <v>57.2</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1670,7 +1670,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>35.1</v>
+        <v>34</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1694,22 +1694,22 @@
         </is>
       </c>
       <c r="V12" t="n">
-        <v>42.55</v>
+        <v>42.63</v>
       </c>
       <c r="W12" t="n">
         <v>60</v>
       </c>
       <c r="X12" t="n">
-        <v>45.9</v>
+        <v>45.1</v>
       </c>
       <c r="Y12" t="n">
-        <v>54.1</v>
+        <v>54.9</v>
       </c>
       <c r="Z12" t="n">
-        <v>50.8</v>
+        <v>62.3</v>
       </c>
       <c r="AA12" t="n">
-        <v>33.8</v>
+        <v>38.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-09-19 13:16
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA12"/>
+  <dimension ref="A1:AA25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -556,44 +556,44 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>4:10</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>30</v>
+        <v>75</v>
       </c>
       <c r="F2" t="n">
-        <v>70</v>
+        <v>25</v>
       </c>
       <c r="G2" t="n">
-        <v>37</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="H2" t="n">
-        <v>63</v>
+        <v>33.6</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>3-8</t>
+          <t>6-3</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -602,25 +602,25 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>76.8</v>
+        <v>49.1</v>
       </c>
       <c r="M2" t="n">
-        <v>54</v>
+        <v>24.8</v>
       </c>
       <c r="N2" t="n">
-        <v>61.1</v>
+        <v>37.2</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>39.2</v>
+        <v>22</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -635,7 +635,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -644,60 +644,60 @@
         </is>
       </c>
       <c r="V2" t="n">
-        <v>38.51</v>
+        <v>25.46</v>
       </c>
       <c r="W2" t="n">
         <v>60</v>
       </c>
       <c r="X2" t="n">
-        <v>47.6</v>
+        <v>53.6</v>
       </c>
       <c r="Y2" t="n">
-        <v>52.4</v>
+        <v>46.4</v>
       </c>
       <c r="Z2" t="n">
-        <v>55.9</v>
+        <v>33.2</v>
       </c>
       <c r="AA2" t="n">
-        <v>34.3</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="F3" t="n">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="G3" t="n">
-        <v>58.7</v>
+        <v>63.9</v>
       </c>
       <c r="H3" t="n">
-        <v>41.3</v>
+        <v>36.1</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -711,98 +711,102 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>16.3</v>
+        <v>22</v>
       </c>
       <c r="M3" t="n">
-        <v>4.7</v>
+        <v>7.3</v>
       </c>
       <c r="N3" t="n">
-        <v>29.1</v>
+        <v>41.7</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P3" t="n">
+        <v>27</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
           <t>언더</t>
         </is>
       </c>
-      <c r="P3" t="n">
-        <v>16</v>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>언더</t>
-        </is>
-      </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>⏭</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr"/>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>확률·표본·모델합의 기준 미달</t>
+          <t>Forebet·과거모델 합의</t>
         </is>
       </c>
       <c r="V3" t="n">
-        <v>41.32</v>
+        <v>34.38</v>
       </c>
       <c r="W3" t="n">
         <v>60</v>
       </c>
       <c r="X3" t="n">
-        <v>53.8</v>
+        <v>59.2</v>
       </c>
       <c r="Y3" t="n">
-        <v>46.2</v>
+        <v>40.8</v>
       </c>
       <c r="Z3" t="n">
-        <v>33.4</v>
+        <v>48.3</v>
       </c>
       <c r="AA3" t="n">
-        <v>19.7</v>
+        <v>33.6</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>8:10</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>Cleveland Guardians</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>Athletics</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="F4" t="n">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="G4" t="n">
-        <v>58.7</v>
+        <v>63.9</v>
       </c>
       <c r="H4" t="n">
-        <v>41.3</v>
+        <v>36.1</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>6-4</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -816,98 +820,102 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>14.3</v>
+        <v>66.7</v>
       </c>
       <c r="M4" t="n">
-        <v>3.9</v>
+        <v>41.7</v>
       </c>
       <c r="N4" t="n">
-        <v>24.4</v>
+        <v>54.3</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P4" t="n">
+        <v>34.6</v>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
           <t>언더</t>
         </is>
       </c>
-      <c r="P4" t="n">
-        <v>13.4</v>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>언더</t>
-        </is>
-      </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>⏭</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr"/>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>확률·표본·모델합의 기준 미달</t>
+          <t>Forebet·과거모델 합의</t>
         </is>
       </c>
       <c r="V4" t="n">
-        <v>41.32</v>
+        <v>42.16</v>
       </c>
       <c r="W4" t="n">
         <v>60</v>
       </c>
       <c r="X4" t="n">
-        <v>53.8</v>
+        <v>53.4</v>
       </c>
       <c r="Y4" t="n">
-        <v>46.2</v>
+        <v>46.6</v>
       </c>
       <c r="Z4" t="n">
-        <v>27.8</v>
+        <v>50.2</v>
       </c>
       <c r="AA4" t="n">
-        <v>16.5</v>
+        <v>32.3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>10:40</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="F5" t="n">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="G5" t="n">
-        <v>57.5</v>
+        <v>62.3</v>
       </c>
       <c r="H5" t="n">
-        <v>42.5</v>
+        <v>37.7</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -921,103 +929,107 @@
         </is>
       </c>
       <c r="L5" t="n">
-        <v>7.5</v>
+        <v>29.7</v>
       </c>
       <c r="M5" t="n">
-        <v>1.6</v>
+        <v>11.3</v>
       </c>
       <c r="N5" t="n">
-        <v>24.6</v>
+        <v>45.7</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P5" t="n">
+        <v>29.9</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
           <t>언더</t>
         </is>
       </c>
-      <c r="P5" t="n">
-        <v>13</v>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>언더</t>
-        </is>
-      </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>⏭</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr"/>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>확률·표본·모델합의 기준 미달</t>
+          <t>Forebet·과거모델 합의</t>
         </is>
       </c>
       <c r="V5" t="n">
-        <v>41.68</v>
+        <v>43.9</v>
       </c>
       <c r="W5" t="n">
         <v>60</v>
       </c>
       <c r="X5" t="n">
-        <v>56.8</v>
+        <v>52.4</v>
       </c>
       <c r="Y5" t="n">
-        <v>43.2</v>
+        <v>47.6</v>
       </c>
       <c r="Z5" t="n">
-        <v>30.2</v>
+        <v>51</v>
       </c>
       <c r="AA5" t="n">
-        <v>16.8</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>KT Wiz Suwon</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>LG Twins</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>44</v>
+        <v>62</v>
       </c>
       <c r="F6" t="n">
-        <v>56</v>
+        <v>38</v>
       </c>
       <c r="G6" t="n">
-        <v>41.2</v>
+        <v>59.2</v>
       </c>
       <c r="H6" t="n">
-        <v>58.8</v>
+        <v>40.8</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>5-6</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -1026,25 +1038,25 @@
         </is>
       </c>
       <c r="L6" t="n">
-        <v>65.59999999999999</v>
+        <v>6.8</v>
       </c>
       <c r="M6" t="n">
-        <v>40.4</v>
+        <v>1.4</v>
       </c>
       <c r="N6" t="n">
-        <v>56.9</v>
+        <v>23.4</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>39.7</v>
+        <v>13.9</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -1064,65 +1076,65 @@
         </is>
       </c>
       <c r="V6" t="n">
-        <v>42.4</v>
+        <v>42.71</v>
       </c>
       <c r="W6" t="n">
         <v>60</v>
       </c>
       <c r="X6" t="n">
-        <v>36.9</v>
+        <v>55</v>
       </c>
       <c r="Y6" t="n">
-        <v>63.1</v>
+        <v>45</v>
       </c>
       <c r="Z6" t="n">
-        <v>54</v>
+        <v>29</v>
       </c>
       <c r="AA6" t="n">
-        <v>39.5</v>
+        <v>18.1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="F7" t="n">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="G7" t="n">
-        <v>55.2</v>
+        <v>42.3</v>
       </c>
       <c r="H7" t="n">
-        <v>44.8</v>
+        <v>57.7</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -1131,21 +1143,21 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>23.3</v>
+        <v>27.1</v>
       </c>
       <c r="M7" t="n">
-        <v>7.9</v>
+        <v>9.9</v>
       </c>
       <c r="N7" t="n">
-        <v>40.6</v>
+        <v>34</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>26.4</v>
+        <v>16.7</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1169,65 +1181,65 @@
         </is>
       </c>
       <c r="V7" t="n">
-        <v>41.35</v>
+        <v>39.81</v>
       </c>
       <c r="W7" t="n">
         <v>60</v>
       </c>
       <c r="X7" t="n">
-        <v>55.5</v>
+        <v>47.2</v>
       </c>
       <c r="Y7" t="n">
-        <v>44.5</v>
+        <v>52.8</v>
       </c>
       <c r="Z7" t="n">
-        <v>46.4</v>
+        <v>36.3</v>
       </c>
       <c r="AA7" t="n">
-        <v>32.6</v>
+        <v>18.9</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Lotte Giants</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>48</v>
+        <v>66</v>
       </c>
       <c r="F8" t="n">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="G8" t="n">
-        <v>45.7</v>
+        <v>61.5</v>
       </c>
       <c r="H8" t="n">
-        <v>54.3</v>
+        <v>38.5</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1236,25 +1248,25 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>57</v>
+        <v>16.3</v>
       </c>
       <c r="M8" t="n">
-        <v>31.8</v>
+        <v>4.7</v>
       </c>
       <c r="N8" t="n">
-        <v>57.7</v>
+        <v>28</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>40.6</v>
+        <v>16.8</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -1274,65 +1286,65 @@
         </is>
       </c>
       <c r="V8" t="n">
-        <v>39.88</v>
+        <v>39.54</v>
       </c>
       <c r="W8" t="n">
         <v>60</v>
       </c>
       <c r="X8" t="n">
-        <v>42.4</v>
+        <v>54.7</v>
       </c>
       <c r="Y8" t="n">
-        <v>57.6</v>
+        <v>45.3</v>
       </c>
       <c r="Z8" t="n">
-        <v>58</v>
+        <v>31.9</v>
       </c>
       <c r="AA8" t="n">
-        <v>43.5</v>
+        <v>20.8</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="F9" t="n">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="G9" t="n">
-        <v>46.3</v>
+        <v>55.3</v>
       </c>
       <c r="H9" t="n">
-        <v>53.7</v>
+        <v>44.7</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>2-1</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1341,21 +1353,21 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>36.6</v>
+        <v>0.8</v>
       </c>
       <c r="M9" t="n">
-        <v>15.5</v>
+        <v>0.1</v>
       </c>
       <c r="N9" t="n">
-        <v>45.5</v>
+        <v>25.2</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>29.7</v>
+        <v>7.7</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1379,60 +1391,60 @@
         </is>
       </c>
       <c r="V9" t="n">
-        <v>39.8</v>
+        <v>42</v>
       </c>
       <c r="W9" t="n">
         <v>60</v>
       </c>
       <c r="X9" t="n">
-        <v>42.2</v>
+        <v>57.3</v>
       </c>
       <c r="Y9" t="n">
-        <v>57.8</v>
+        <v>42.7</v>
       </c>
       <c r="Z9" t="n">
-        <v>48.5</v>
+        <v>33.3</v>
       </c>
       <c r="AA9" t="n">
-        <v>34.5</v>
+        <v>10.3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>8:15</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Houston Astros</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="F10" t="n">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="G10" t="n">
-        <v>58</v>
+        <v>51.7</v>
       </c>
       <c r="H10" t="n">
-        <v>42</v>
+        <v>48.3</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>7-5</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1446,21 +1458,21 @@
         </is>
       </c>
       <c r="L10" t="n">
-        <v>59.6</v>
+        <v>16.3</v>
       </c>
       <c r="M10" t="n">
-        <v>34.2</v>
+        <v>4.7</v>
       </c>
       <c r="N10" t="n">
-        <v>54.8</v>
+        <v>28</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>37.4</v>
+        <v>16.8</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1484,60 +1496,60 @@
         </is>
       </c>
       <c r="V10" t="n">
-        <v>43.07</v>
+        <v>42.24</v>
       </c>
       <c r="W10" t="n">
         <v>60</v>
       </c>
       <c r="X10" t="n">
-        <v>56.6</v>
+        <v>49.9</v>
       </c>
       <c r="Y10" t="n">
-        <v>43.4</v>
+        <v>50.1</v>
       </c>
       <c r="Z10" t="n">
-        <v>53.2</v>
+        <v>31.9</v>
       </c>
       <c r="AA10" t="n">
-        <v>38.5</v>
+        <v>20.8</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Detroit Tigers</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="F11" t="n">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="G11" t="n">
-        <v>51.3</v>
+        <v>61.4</v>
       </c>
       <c r="H11" t="n">
-        <v>48.7</v>
+        <v>38.6</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1551,13 +1563,13 @@
         </is>
       </c>
       <c r="L11" t="n">
-        <v>32.4</v>
+        <v>57</v>
       </c>
       <c r="M11" t="n">
-        <v>12.9</v>
+        <v>31.8</v>
       </c>
       <c r="N11" t="n">
-        <v>49.9</v>
+        <v>58</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1565,11 +1577,11 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>35.2</v>
+        <v>41.1</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>언더</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -1589,60 +1601,60 @@
         </is>
       </c>
       <c r="V11" t="n">
-        <v>41.97</v>
+        <v>42.71</v>
       </c>
       <c r="W11" t="n">
         <v>60</v>
       </c>
       <c r="X11" t="n">
-        <v>51.7</v>
+        <v>62</v>
       </c>
       <c r="Y11" t="n">
-        <v>48.3</v>
+        <v>38</v>
       </c>
       <c r="Z11" t="n">
-        <v>55.7</v>
+        <v>58.3</v>
       </c>
       <c r="AA11" t="n">
-        <v>42.6</v>
+        <v>44.2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>9:05</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Boston Red Sox</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="F12" t="n">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="G12" t="n">
-        <v>49.8</v>
+        <v>57.3</v>
       </c>
       <c r="H12" t="n">
-        <v>50.2</v>
+        <v>42.7</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>6-3</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1656,13 +1668,13 @@
         </is>
       </c>
       <c r="L12" t="n">
-        <v>42.1</v>
+        <v>54.4</v>
       </c>
       <c r="M12" t="n">
-        <v>19.4</v>
+        <v>29.4</v>
       </c>
       <c r="N12" t="n">
-        <v>57.2</v>
+        <v>57.9</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1670,11 +1682,11 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>34</v>
+        <v>41.7</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>언더</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -1694,22 +1706,1389 @@
         </is>
       </c>
       <c r="V12" t="n">
-        <v>42.63</v>
+        <v>42.27</v>
       </c>
       <c r="W12" t="n">
         <v>60</v>
       </c>
       <c r="X12" t="n">
-        <v>45.1</v>
+        <v>57.8</v>
       </c>
       <c r="Y12" t="n">
-        <v>54.9</v>
+        <v>42.2</v>
       </c>
       <c r="Z12" t="n">
-        <v>62.3</v>
+        <v>59.1</v>
       </c>
       <c r="AA12" t="n">
-        <v>38.9</v>
+        <v>45.9</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Lotte Giants</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Samsung Lions</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>49</v>
+      </c>
+      <c r="F13" t="n">
+        <v>51</v>
+      </c>
+      <c r="G13" t="n">
+        <v>46.8</v>
+      </c>
+      <c r="H13" t="n">
+        <v>53.2</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>7-9</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
+        <v>90.90000000000001</v>
+      </c>
+      <c r="M13" t="n">
+        <v>76.5</v>
+      </c>
+      <c r="N13" t="n">
+        <v>65.8</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>오버</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V13" t="n">
+        <v>40.26</v>
+      </c>
+      <c r="W13" t="n">
+        <v>60</v>
+      </c>
+      <c r="X13" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>56.5</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>40.2</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>7:40</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Pittsburgh Pirates</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Kansas City Royals</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>58</v>
+      </c>
+      <c r="F14" t="n">
+        <v>42</v>
+      </c>
+      <c r="G14" t="n">
+        <v>56.2</v>
+      </c>
+      <c r="H14" t="n">
+        <v>43.8</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>7-5</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L14" t="n">
+        <v>62</v>
+      </c>
+      <c r="M14" t="n">
+        <v>36.7</v>
+      </c>
+      <c r="N14" t="n">
+        <v>52.5</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P14" t="n">
+        <v>34.2</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>언더</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V14" t="n">
+        <v>44.18</v>
+      </c>
+      <c r="W14" t="n">
+        <v>60</v>
+      </c>
+      <c r="X14" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>49.3</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>33.4</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>7:40</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Cincinnati Reds</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Chicago Cubs</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>55</v>
+      </c>
+      <c r="F15" t="n">
+        <v>45</v>
+      </c>
+      <c r="G15" t="n">
+        <v>53.1</v>
+      </c>
+      <c r="H15" t="n">
+        <v>46.9</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L15" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="M15" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="N15" t="n">
+        <v>46</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P15" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>언더</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V15" t="n">
+        <v>42.12</v>
+      </c>
+      <c r="W15" t="n">
+        <v>60</v>
+      </c>
+      <c r="X15" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>49.8</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>46.8</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>31.5</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>8:05</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Baltimore Orioles</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>45</v>
+      </c>
+      <c r="F16" t="n">
+        <v>55</v>
+      </c>
+      <c r="G16" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="H16" t="n">
+        <v>52.7</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>3-4</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L16" t="n">
+        <v>32.4</v>
+      </c>
+      <c r="M16" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="N16" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P16" t="n">
+        <v>33.9</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>언더</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V16" t="n">
+        <v>43.73</v>
+      </c>
+      <c r="W16" t="n">
+        <v>60</v>
+      </c>
+      <c r="X16" t="n">
+        <v>50.8</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>49.2</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>54.7</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>40.9</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>8:10</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Boston Red Sox</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>57</v>
+      </c>
+      <c r="F17" t="n">
+        <v>43</v>
+      </c>
+      <c r="G17" t="n">
+        <v>57.2</v>
+      </c>
+      <c r="H17" t="n">
+        <v>42.8</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L17" t="n">
+        <v>28.4</v>
+      </c>
+      <c r="M17" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="N17" t="n">
+        <v>40.4</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P17" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>언더</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr"/>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V17" t="n">
+        <v>46.19</v>
+      </c>
+      <c r="W17" t="n">
+        <v>60</v>
+      </c>
+      <c r="X17" t="n">
+        <v>57.5</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>8:15</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>New York Mets</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Philadelphia Phillies</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>51</v>
+      </c>
+      <c r="F18" t="n">
+        <v>49</v>
+      </c>
+      <c r="G18" t="n">
+        <v>51.3</v>
+      </c>
+      <c r="H18" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>5-3</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L18" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="M18" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="N18" t="n">
+        <v>49.3</v>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P18" t="n">
+        <v>30.6</v>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>언더</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr"/>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V18" t="n">
+        <v>41.79</v>
+      </c>
+      <c r="W18" t="n">
+        <v>60</v>
+      </c>
+      <c r="X18" t="n">
+        <v>51.8</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>48.2</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>8:40</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Chicago White Sox</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Detroit Tigers</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>54</v>
+      </c>
+      <c r="F19" t="n">
+        <v>46</v>
+      </c>
+      <c r="G19" t="n">
+        <v>50.7</v>
+      </c>
+      <c r="H19" t="n">
+        <v>49.3</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L19" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="M19" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="N19" t="n">
+        <v>40.3</v>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P19" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>언더</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr"/>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V19" t="n">
+        <v>42.32</v>
+      </c>
+      <c r="W19" t="n">
+        <v>60</v>
+      </c>
+      <c r="X19" t="n">
+        <v>45.8</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>54.2</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>46.8</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>30.6</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>9:05</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Texas Rangers</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Toronto Blue Jays</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>53</v>
+      </c>
+      <c r="F20" t="n">
+        <v>47</v>
+      </c>
+      <c r="G20" t="n">
+        <v>49.9</v>
+      </c>
+      <c r="H20" t="n">
+        <v>50.1</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L20" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="M20" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="N20" t="n">
+        <v>41</v>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P20" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>언더</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V20" t="n">
+        <v>43.33</v>
+      </c>
+      <c r="W20" t="n">
+        <v>60</v>
+      </c>
+      <c r="X20" t="n">
+        <v>45.2</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>54.8</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="AA20" t="n">
+        <v>40.8</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>9:10</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Colorado Rockies</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Seattle Mariners</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>45</v>
+      </c>
+      <c r="F21" t="n">
+        <v>55</v>
+      </c>
+      <c r="G21" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="H21" t="n">
+        <v>52.7</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>3-5</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L21" t="n">
+        <v>47.7</v>
+      </c>
+      <c r="M21" t="n">
+        <v>23.7</v>
+      </c>
+      <c r="N21" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P21" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>언더</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V21" t="n">
+        <v>43.65</v>
+      </c>
+      <c r="W21" t="n">
+        <v>60</v>
+      </c>
+      <c r="X21" t="n">
+        <v>50.8</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>49.2</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="AA21" t="n">
+        <v>39.4</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>9:10</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Houston Astros</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Atlanta Braves</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>52</v>
+      </c>
+      <c r="F22" t="n">
+        <v>48</v>
+      </c>
+      <c r="G22" t="n">
+        <v>51.1</v>
+      </c>
+      <c r="H22" t="n">
+        <v>48.9</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L22" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="M22" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="N22" t="n">
+        <v>44.9</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P22" t="n">
+        <v>30.9</v>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>언더</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr"/>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V22" t="n">
+        <v>40.92</v>
+      </c>
+      <c r="W22" t="n">
+        <v>60</v>
+      </c>
+      <c r="X22" t="n">
+        <v>49.7</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>50.3</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>50</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>37.4</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>9:15</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>St.Louis Cardinals</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Washington Nationals</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>45</v>
+      </c>
+      <c r="F23" t="n">
+        <v>55</v>
+      </c>
+      <c r="G23" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="H23" t="n">
+        <v>52.7</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>4-6</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L23" t="n">
+        <v>42.1</v>
+      </c>
+      <c r="M23" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="N23" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P23" t="n">
+        <v>33.6</v>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>언더</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr"/>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V23" t="n">
+        <v>43.65</v>
+      </c>
+      <c r="W23" t="n">
+        <v>60</v>
+      </c>
+      <c r="X23" t="n">
+        <v>50.8</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>49.2</v>
+      </c>
+      <c r="Z23" t="n">
+        <v>58.6</v>
+      </c>
+      <c r="AA23" t="n">
+        <v>38.4</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>New York Yankees</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>54</v>
+      </c>
+      <c r="F24" t="n">
+        <v>46</v>
+      </c>
+      <c r="G24" t="n">
+        <v>51.8</v>
+      </c>
+      <c r="H24" t="n">
+        <v>48.2</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L24" t="n">
+        <v>51.8</v>
+      </c>
+      <c r="M24" t="n">
+        <v>27.1</v>
+      </c>
+      <c r="N24" t="n">
+        <v>51.3</v>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P24" t="n">
+        <v>32.9</v>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>언더</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V24" t="n">
+        <v>43.69</v>
+      </c>
+      <c r="W24" t="n">
+        <v>60</v>
+      </c>
+      <c r="X24" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="Y24" t="n">
+        <v>51.6</v>
+      </c>
+      <c r="Z24" t="n">
+        <v>51.1</v>
+      </c>
+      <c r="AA24" t="n">
+        <v>34.9</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Los Angeles Dodgers</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>San Francisco Giants</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>60</v>
+      </c>
+      <c r="F25" t="n">
+        <v>40</v>
+      </c>
+      <c r="G25" t="n">
+        <v>59.4</v>
+      </c>
+      <c r="H25" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L25" t="n">
+        <v>42.1</v>
+      </c>
+      <c r="M25" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="N25" t="n">
+        <v>54.3</v>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P25" t="n">
+        <v>34.6</v>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>언더</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr"/>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V25" t="n">
+        <v>44.58</v>
+      </c>
+      <c r="W25" t="n">
+        <v>60</v>
+      </c>
+      <c r="X25" t="n">
+        <v>58.5</v>
+      </c>
+      <c r="Y25" t="n">
+        <v>41.5</v>
+      </c>
+      <c r="Z25" t="n">
+        <v>58.4</v>
+      </c>
+      <c r="AA25" t="n">
+        <v>39.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-09-20 14:58
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA25"/>
+  <dimension ref="A1:AA15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -575,20 +575,20 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="F2" t="n">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="G2" t="n">
-        <v>66.40000000000001</v>
+        <v>63.4</v>
       </c>
       <c r="H2" t="n">
-        <v>33.6</v>
+        <v>36.6</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>6-3</t>
+          <t>6-4</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -602,27 +602,27 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>49.1</v>
+        <v>60.8</v>
       </c>
       <c r="M2" t="n">
-        <v>24.8</v>
+        <v>35.5</v>
       </c>
       <c r="N2" t="n">
-        <v>37.2</v>
+        <v>40.9</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P2" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
           <t>언더</t>
         </is>
       </c>
-      <c r="P2" t="n">
-        <v>22</v>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>언더</t>
-        </is>
-      </c>
       <c r="R2" t="inlineStr">
         <is>
           <t>★★</t>
@@ -644,28 +644,28 @@
         </is>
       </c>
       <c r="V2" t="n">
-        <v>25.46</v>
+        <v>37.3</v>
       </c>
       <c r="W2" t="n">
         <v>60</v>
       </c>
       <c r="X2" t="n">
-        <v>53.6</v>
+        <v>54.9</v>
       </c>
       <c r="Y2" t="n">
-        <v>46.4</v>
+        <v>45.1</v>
       </c>
       <c r="Z2" t="n">
-        <v>33.2</v>
+        <v>34.2</v>
       </c>
       <c r="AA2" t="n">
-        <v>21</v>
+        <v>20.4</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -684,20 +684,20 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F3" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G3" t="n">
-        <v>63.9</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="H3" t="n">
-        <v>36.1</v>
+        <v>35.9</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>4-1</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -711,13 +711,13 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>22</v>
+        <v>16.3</v>
       </c>
       <c r="M3" t="n">
-        <v>7.3</v>
+        <v>4.7</v>
       </c>
       <c r="N3" t="n">
-        <v>41.7</v>
+        <v>40.1</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>27</v>
+        <v>25.4</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -753,60 +753,60 @@
         </is>
       </c>
       <c r="V3" t="n">
-        <v>34.38</v>
+        <v>33.14</v>
       </c>
       <c r="W3" t="n">
         <v>60</v>
       </c>
       <c r="X3" t="n">
-        <v>59.2</v>
+        <v>58.2</v>
       </c>
       <c r="Y3" t="n">
-        <v>40.8</v>
+        <v>41.8</v>
       </c>
       <c r="Z3" t="n">
-        <v>48.3</v>
+        <v>48</v>
       </c>
       <c r="AA3" t="n">
-        <v>33.6</v>
+        <v>32.3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Cleveland Guardians</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Athletics</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="F4" t="n">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="G4" t="n">
-        <v>63.9</v>
+        <v>62.5</v>
       </c>
       <c r="H4" t="n">
-        <v>36.1</v>
+        <v>37.5</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>6-4</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -820,13 +820,13 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>66.7</v>
+        <v>46.3</v>
       </c>
       <c r="M4" t="n">
-        <v>41.7</v>
+        <v>22.6</v>
       </c>
       <c r="N4" t="n">
-        <v>54.3</v>
+        <v>52.3</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -834,7 +834,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>34.6</v>
+        <v>33</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -862,38 +862,38 @@
         </is>
       </c>
       <c r="V4" t="n">
-        <v>42.16</v>
+        <v>37.6</v>
       </c>
       <c r="W4" t="n">
         <v>60</v>
       </c>
       <c r="X4" t="n">
-        <v>53.4</v>
+        <v>58.8</v>
       </c>
       <c r="Y4" t="n">
-        <v>46.6</v>
+        <v>41.2</v>
       </c>
       <c r="Z4" t="n">
-        <v>50.2</v>
+        <v>54.3</v>
       </c>
       <c r="AA4" t="n">
-        <v>32.3</v>
+        <v>36.4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>5:10</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>Philadelphia Phillies</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -902,20 +902,20 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="F5" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="G5" t="n">
-        <v>62.3</v>
+        <v>63</v>
       </c>
       <c r="H5" t="n">
-        <v>37.7</v>
+        <v>37</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -929,13 +929,13 @@
         </is>
       </c>
       <c r="L5" t="n">
-        <v>29.7</v>
+        <v>39.3</v>
       </c>
       <c r="M5" t="n">
-        <v>11.3</v>
+        <v>17.4</v>
       </c>
       <c r="N5" t="n">
-        <v>45.7</v>
+        <v>47.6</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -943,7 +943,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>29.9</v>
+        <v>28.7</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -971,22 +971,22 @@
         </is>
       </c>
       <c r="V5" t="n">
-        <v>43.9</v>
+        <v>43.63</v>
       </c>
       <c r="W5" t="n">
         <v>60</v>
       </c>
       <c r="X5" t="n">
-        <v>52.4</v>
+        <v>59.9</v>
       </c>
       <c r="Y5" t="n">
-        <v>47.6</v>
+        <v>40.1</v>
       </c>
       <c r="Z5" t="n">
-        <v>51</v>
+        <v>50.4</v>
       </c>
       <c r="AA5" t="n">
-        <v>36</v>
+        <v>32.4</v>
       </c>
     </row>
     <row r="6">
@@ -1002,7 +1002,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1011,20 +1011,20 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="F6" t="n">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="G6" t="n">
-        <v>59.2</v>
+        <v>57.7</v>
       </c>
       <c r="H6" t="n">
-        <v>40.8</v>
+        <v>42.3</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -1038,13 +1038,13 @@
         </is>
       </c>
       <c r="L6" t="n">
-        <v>6.8</v>
+        <v>3.6</v>
       </c>
       <c r="M6" t="n">
-        <v>1.4</v>
+        <v>0.6</v>
       </c>
       <c r="N6" t="n">
-        <v>23.4</v>
+        <v>26.2</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1052,7 +1052,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>13.9</v>
+        <v>9</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1076,22 +1076,22 @@
         </is>
       </c>
       <c r="V6" t="n">
-        <v>42.71</v>
+        <v>42.64</v>
       </c>
       <c r="W6" t="n">
         <v>60</v>
       </c>
       <c r="X6" t="n">
-        <v>55</v>
+        <v>60.2</v>
       </c>
       <c r="Y6" t="n">
-        <v>45</v>
+        <v>39.8</v>
       </c>
       <c r="Z6" t="n">
-        <v>29</v>
+        <v>33.7</v>
       </c>
       <c r="AA6" t="n">
-        <v>18.1</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="7">
@@ -1116,20 +1116,20 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="F7" t="n">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="G7" t="n">
-        <v>42.3</v>
+        <v>49.7</v>
       </c>
       <c r="H7" t="n">
-        <v>57.7</v>
+        <v>50.3</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1143,13 +1143,13 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>27.1</v>
+        <v>17.4</v>
       </c>
       <c r="M7" t="n">
-        <v>9.9</v>
+        <v>5.1</v>
       </c>
       <c r="N7" t="n">
-        <v>34</v>
+        <v>27.5</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1157,7 +1157,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>16.7</v>
+        <v>16.5</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1181,22 +1181,22 @@
         </is>
       </c>
       <c r="V7" t="n">
-        <v>39.81</v>
+        <v>41.54</v>
       </c>
       <c r="W7" t="n">
         <v>60</v>
       </c>
       <c r="X7" t="n">
-        <v>47.2</v>
+        <v>52.3</v>
       </c>
       <c r="Y7" t="n">
-        <v>52.8</v>
+        <v>47.7</v>
       </c>
       <c r="Z7" t="n">
-        <v>36.3</v>
+        <v>30.9</v>
       </c>
       <c r="AA7" t="n">
-        <v>18.9</v>
+        <v>20.3</v>
       </c>
     </row>
     <row r="8">
@@ -1207,12 +1207,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1221,25 +1221,25 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>66</v>
+        <v>44</v>
       </c>
       <c r="F8" t="n">
-        <v>34</v>
+        <v>56</v>
       </c>
       <c r="G8" t="n">
-        <v>61.5</v>
+        <v>46.5</v>
       </c>
       <c r="H8" t="n">
-        <v>38.5</v>
+        <v>53.5</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>2-3</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1248,13 +1248,13 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>16.3</v>
+        <v>8.9</v>
       </c>
       <c r="M8" t="n">
-        <v>4.7</v>
+        <v>2</v>
       </c>
       <c r="N8" t="n">
-        <v>28</v>
+        <v>25.6</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1262,7 +1262,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>16.8</v>
+        <v>14.5</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1286,22 +1286,22 @@
         </is>
       </c>
       <c r="V8" t="n">
-        <v>39.54</v>
+        <v>39.49</v>
       </c>
       <c r="W8" t="n">
         <v>60</v>
       </c>
       <c r="X8" t="n">
-        <v>54.7</v>
+        <v>50.3</v>
       </c>
       <c r="Y8" t="n">
-        <v>45.3</v>
+        <v>49.7</v>
       </c>
       <c r="Z8" t="n">
-        <v>31.9</v>
+        <v>31.1</v>
       </c>
       <c r="AA8" t="n">
-        <v>20.8</v>
+        <v>18.7</v>
       </c>
     </row>
     <row r="9">
@@ -1317,7 +1317,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1326,25 +1326,25 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="F9" t="n">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="G9" t="n">
-        <v>55.3</v>
+        <v>47.3</v>
       </c>
       <c r="H9" t="n">
-        <v>44.7</v>
+        <v>52.7</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>2-4</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1353,13 +1353,13 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>0.8</v>
+        <v>14.3</v>
       </c>
       <c r="M9" t="n">
-        <v>0.1</v>
+        <v>3.9</v>
       </c>
       <c r="N9" t="n">
-        <v>25.2</v>
+        <v>24.9</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1367,7 +1367,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>7.7</v>
+        <v>12.2</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1391,22 +1391,22 @@
         </is>
       </c>
       <c r="V9" t="n">
-        <v>42</v>
+        <v>41.18</v>
       </c>
       <c r="W9" t="n">
         <v>60</v>
       </c>
       <c r="X9" t="n">
-        <v>57.3</v>
+        <v>50.8</v>
       </c>
       <c r="Y9" t="n">
-        <v>42.7</v>
+        <v>49.2</v>
       </c>
       <c r="Z9" t="n">
-        <v>33.3</v>
+        <v>28.4</v>
       </c>
       <c r="AA9" t="n">
-        <v>10.3</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10">
@@ -1431,25 +1431,25 @@
         </is>
       </c>
       <c r="E10" t="n">
+        <v>47</v>
+      </c>
+      <c r="F10" t="n">
         <v>53</v>
       </c>
-      <c r="F10" t="n">
-        <v>47</v>
-      </c>
       <c r="G10" t="n">
-        <v>51.7</v>
+        <v>49.4</v>
       </c>
       <c r="H10" t="n">
-        <v>48.3</v>
+        <v>50.6</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>2-3</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1458,13 +1458,13 @@
         </is>
       </c>
       <c r="L10" t="n">
-        <v>16.3</v>
+        <v>8.9</v>
       </c>
       <c r="M10" t="n">
-        <v>4.7</v>
+        <v>2</v>
       </c>
       <c r="N10" t="n">
-        <v>28</v>
+        <v>25.6</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1472,7 +1472,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>16.8</v>
+        <v>14.5</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1496,28 +1496,28 @@
         </is>
       </c>
       <c r="V10" t="n">
-        <v>42.24</v>
+        <v>41.54</v>
       </c>
       <c r="W10" t="n">
         <v>60</v>
       </c>
       <c r="X10" t="n">
-        <v>49.9</v>
+        <v>53.1</v>
       </c>
       <c r="Y10" t="n">
-        <v>50.1</v>
+        <v>46.9</v>
       </c>
       <c r="Z10" t="n">
-        <v>31.9</v>
+        <v>31.1</v>
       </c>
       <c r="AA10" t="n">
-        <v>20.8</v>
+        <v>18.7</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1542,10 +1542,10 @@
         <v>39</v>
       </c>
       <c r="G11" t="n">
-        <v>61.4</v>
+        <v>60.9</v>
       </c>
       <c r="H11" t="n">
-        <v>38.6</v>
+        <v>39.1</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -1569,7 +1569,7 @@
         <v>31.8</v>
       </c>
       <c r="N11" t="n">
-        <v>58</v>
+        <v>57.9</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1601,16 +1601,16 @@
         </is>
       </c>
       <c r="V11" t="n">
-        <v>42.71</v>
+        <v>42.9</v>
       </c>
       <c r="W11" t="n">
         <v>60</v>
       </c>
       <c r="X11" t="n">
-        <v>62</v>
+        <v>60.7</v>
       </c>
       <c r="Y11" t="n">
-        <v>38</v>
+        <v>39.3</v>
       </c>
       <c r="Z11" t="n">
         <v>58.3</v>
@@ -1622,7 +1622,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1647,10 +1647,10 @@
         <v>43</v>
       </c>
       <c r="G12" t="n">
-        <v>57.3</v>
+        <v>57.4</v>
       </c>
       <c r="H12" t="n">
-        <v>42.7</v>
+        <v>42.6</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -1674,7 +1674,7 @@
         <v>29.4</v>
       </c>
       <c r="N12" t="n">
-        <v>57.9</v>
+        <v>57.7</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1682,7 +1682,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>41.7</v>
+        <v>40.7</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1706,28 +1706,28 @@
         </is>
       </c>
       <c r="V12" t="n">
-        <v>42.27</v>
+        <v>42.3</v>
       </c>
       <c r="W12" t="n">
         <v>60</v>
       </c>
       <c r="X12" t="n">
-        <v>57.8</v>
+        <v>58.1</v>
       </c>
       <c r="Y12" t="n">
-        <v>42.2</v>
+        <v>41.9</v>
       </c>
       <c r="Z12" t="n">
-        <v>59.1</v>
+        <v>58.7</v>
       </c>
       <c r="AA12" t="n">
-        <v>45.9</v>
+        <v>44.4</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1746,25 +1746,25 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="F13" t="n">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="G13" t="n">
-        <v>46.8</v>
+        <v>55.5</v>
       </c>
       <c r="H13" t="n">
-        <v>53.2</v>
+        <v>44.5</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>7-9</t>
+          <t>8-7</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1779,17 +1779,15 @@
         <v>76.5</v>
       </c>
       <c r="N13" t="n">
-        <v>65.8</v>
+        <v>64.3</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
           <t>오버</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="P13" t="n">
+        <v>48</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1813,38 +1811,38 @@
         </is>
       </c>
       <c r="V13" t="n">
-        <v>40.26</v>
+        <v>40.29</v>
       </c>
       <c r="W13" t="n">
         <v>60</v>
       </c>
       <c r="X13" t="n">
-        <v>43.5</v>
+        <v>57.7</v>
       </c>
       <c r="Y13" t="n">
-        <v>56.5</v>
+        <v>42.3</v>
       </c>
       <c r="Z13" t="n">
-        <v>57.4</v>
+        <v>55.4</v>
       </c>
       <c r="AA13" t="n">
-        <v>40.2</v>
+        <v>38.5</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>5:10</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates</t>
+          <t>Tampa Bay Rays</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Kansas City Royals</t>
+          <t>Boston Red Sox</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1853,20 +1851,20 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="F14" t="n">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="G14" t="n">
-        <v>56.2</v>
+        <v>51.4</v>
       </c>
       <c r="H14" t="n">
-        <v>43.8</v>
+        <v>48.6</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>7-5</t>
+          <t>6-4</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1880,13 +1878,13 @@
         </is>
       </c>
       <c r="L14" t="n">
-        <v>62</v>
+        <v>39.3</v>
       </c>
       <c r="M14" t="n">
-        <v>36.7</v>
+        <v>17.4</v>
       </c>
       <c r="N14" t="n">
-        <v>52.5</v>
+        <v>47.6</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1894,7 +1892,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>34.2</v>
+        <v>28.7</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1918,38 +1916,38 @@
         </is>
       </c>
       <c r="V14" t="n">
-        <v>44.18</v>
+        <v>42.08</v>
       </c>
       <c r="W14" t="n">
         <v>60</v>
       </c>
       <c r="X14" t="n">
-        <v>53.6</v>
+        <v>50.5</v>
       </c>
       <c r="Y14" t="n">
-        <v>46.4</v>
+        <v>49.5</v>
       </c>
       <c r="Z14" t="n">
-        <v>49.3</v>
+        <v>50.4</v>
       </c>
       <c r="AA14" t="n">
-        <v>33.4</v>
+        <v>32.4</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>7:10</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Cincinnati Reds</t>
+          <t>Cleveland Guardians</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Chicago Cubs</t>
+          <t>Athletics</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1958,20 +1956,20 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="F15" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="G15" t="n">
-        <v>53.1</v>
+        <v>57.2</v>
       </c>
       <c r="H15" t="n">
-        <v>46.9</v>
+        <v>42.8</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1985,10 +1983,10 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>43.5</v>
+        <v>33.8</v>
       </c>
       <c r="M15" t="n">
-        <v>20.4</v>
+        <v>13.8</v>
       </c>
       <c r="N15" t="n">
         <v>46</v>
@@ -1999,7 +1997,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>28.7</v>
+        <v>33.7</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -2023,1072 +2021,22 @@
         </is>
       </c>
       <c r="V15" t="n">
-        <v>42.12</v>
+        <v>44.6</v>
       </c>
       <c r="W15" t="n">
         <v>60</v>
       </c>
       <c r="X15" t="n">
-        <v>50.2</v>
+        <v>54.5</v>
       </c>
       <c r="Y15" t="n">
-        <v>49.8</v>
+        <v>45.5</v>
       </c>
       <c r="Z15" t="n">
-        <v>46.8</v>
+        <v>50.1</v>
       </c>
       <c r="AA15" t="n">
-        <v>31.5</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>8:05</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Baltimore Orioles</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Milwaukee Brewers</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>45</v>
-      </c>
-      <c r="F16" t="n">
-        <v>55</v>
-      </c>
-      <c r="G16" t="n">
-        <v>47.3</v>
-      </c>
-      <c r="H16" t="n">
-        <v>52.7</v>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>3-4</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L16" t="n">
-        <v>32.4</v>
-      </c>
-      <c r="M16" t="n">
-        <v>12.9</v>
-      </c>
-      <c r="N16" t="n">
-        <v>49.1</v>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="P16" t="n">
-        <v>33.9</v>
-      </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>언더</t>
-        </is>
-      </c>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>⏭</t>
-        </is>
-      </c>
-      <c r="S16" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="T16" t="inlineStr"/>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>확률·표본·모델합의 기준 미달</t>
-        </is>
-      </c>
-      <c r="V16" t="n">
-        <v>43.73</v>
-      </c>
-      <c r="W16" t="n">
-        <v>60</v>
-      </c>
-      <c r="X16" t="n">
-        <v>50.8</v>
-      </c>
-      <c r="Y16" t="n">
-        <v>49.2</v>
-      </c>
-      <c r="Z16" t="n">
-        <v>54.7</v>
-      </c>
-      <c r="AA16" t="n">
-        <v>40.9</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>8:10</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Tampa Bay Rays</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Boston Red Sox</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E17" t="n">
-        <v>57</v>
-      </c>
-      <c r="F17" t="n">
-        <v>43</v>
-      </c>
-      <c r="G17" t="n">
-        <v>57.2</v>
-      </c>
-      <c r="H17" t="n">
-        <v>42.8</v>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>4-3</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L17" t="n">
-        <v>28.4</v>
-      </c>
-      <c r="M17" t="n">
-        <v>10.6</v>
-      </c>
-      <c r="N17" t="n">
-        <v>40.4</v>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="P17" t="n">
-        <v>25.9</v>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>언더</t>
-        </is>
-      </c>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>⏭</t>
-        </is>
-      </c>
-      <c r="S17" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="T17" t="inlineStr"/>
-      <c r="U17" t="inlineStr">
-        <is>
-          <t>확률·표본·모델합의 기준 미달</t>
-        </is>
-      </c>
-      <c r="V17" t="n">
-        <v>46.19</v>
-      </c>
-      <c r="W17" t="n">
-        <v>60</v>
-      </c>
-      <c r="X17" t="n">
-        <v>57.5</v>
-      </c>
-      <c r="Y17" t="n">
-        <v>42.5</v>
-      </c>
-      <c r="Z17" t="n">
-        <v>44.4</v>
-      </c>
-      <c r="AA17" t="n">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>8:15</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>New York Mets</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Philadelphia Phillies</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E18" t="n">
-        <v>51</v>
-      </c>
-      <c r="F18" t="n">
-        <v>49</v>
-      </c>
-      <c r="G18" t="n">
-        <v>51.3</v>
-      </c>
-      <c r="H18" t="n">
-        <v>48.7</v>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>5-3</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L18" t="n">
-        <v>39.3</v>
-      </c>
-      <c r="M18" t="n">
-        <v>17.4</v>
-      </c>
-      <c r="N18" t="n">
-        <v>49.3</v>
-      </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="P18" t="n">
-        <v>30.6</v>
-      </c>
-      <c r="Q18" t="inlineStr">
-        <is>
-          <t>언더</t>
-        </is>
-      </c>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>⏭</t>
-        </is>
-      </c>
-      <c r="S18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="T18" t="inlineStr"/>
-      <c r="U18" t="inlineStr">
-        <is>
-          <t>확률·표본·모델합의 기준 미달</t>
-        </is>
-      </c>
-      <c r="V18" t="n">
-        <v>41.79</v>
-      </c>
-      <c r="W18" t="n">
-        <v>60</v>
-      </c>
-      <c r="X18" t="n">
-        <v>51.8</v>
-      </c>
-      <c r="Y18" t="n">
-        <v>48.2</v>
-      </c>
-      <c r="Z18" t="n">
-        <v>52.6</v>
-      </c>
-      <c r="AA18" t="n">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>8:40</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Chicago White Sox</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Detroit Tigers</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E19" t="n">
-        <v>54</v>
-      </c>
-      <c r="F19" t="n">
-        <v>46</v>
-      </c>
-      <c r="G19" t="n">
-        <v>50.7</v>
-      </c>
-      <c r="H19" t="n">
-        <v>49.3</v>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>4-3</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L19" t="n">
-        <v>20.8</v>
-      </c>
-      <c r="M19" t="n">
-        <v>6.7</v>
-      </c>
-      <c r="N19" t="n">
         <v>40.3</v>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="P19" t="n">
-        <v>24.6</v>
-      </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>언더</t>
-        </is>
-      </c>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>⏭</t>
-        </is>
-      </c>
-      <c r="S19" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="T19" t="inlineStr"/>
-      <c r="U19" t="inlineStr">
-        <is>
-          <t>확률·표본·모델합의 기준 미달</t>
-        </is>
-      </c>
-      <c r="V19" t="n">
-        <v>42.32</v>
-      </c>
-      <c r="W19" t="n">
-        <v>60</v>
-      </c>
-      <c r="X19" t="n">
-        <v>45.8</v>
-      </c>
-      <c r="Y19" t="n">
-        <v>54.2</v>
-      </c>
-      <c r="Z19" t="n">
-        <v>46.8</v>
-      </c>
-      <c r="AA19" t="n">
-        <v>30.6</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>9:05</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Texas Rangers</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Toronto Blue Jays</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E20" t="n">
-        <v>53</v>
-      </c>
-      <c r="F20" t="n">
-        <v>47</v>
-      </c>
-      <c r="G20" t="n">
-        <v>49.9</v>
-      </c>
-      <c r="H20" t="n">
-        <v>50.1</v>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>3-2</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L20" t="n">
-        <v>12.3</v>
-      </c>
-      <c r="M20" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="N20" t="n">
-        <v>41</v>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="P20" t="n">
-        <v>31.4</v>
-      </c>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>언더</t>
-        </is>
-      </c>
-      <c r="R20" t="inlineStr">
-        <is>
-          <t>⏭</t>
-        </is>
-      </c>
-      <c r="S20" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="T20" t="inlineStr"/>
-      <c r="U20" t="inlineStr">
-        <is>
-          <t>확률·표본·모델합의 기준 미달</t>
-        </is>
-      </c>
-      <c r="V20" t="n">
-        <v>43.33</v>
-      </c>
-      <c r="W20" t="n">
-        <v>60</v>
-      </c>
-      <c r="X20" t="n">
-        <v>45.2</v>
-      </c>
-      <c r="Y20" t="n">
-        <v>54.8</v>
-      </c>
-      <c r="Z20" t="n">
-        <v>50.5</v>
-      </c>
-      <c r="AA20" t="n">
-        <v>40.8</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>9:10</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Colorado Rockies</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Seattle Mariners</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E21" t="n">
-        <v>45</v>
-      </c>
-      <c r="F21" t="n">
-        <v>55</v>
-      </c>
-      <c r="G21" t="n">
-        <v>47.3</v>
-      </c>
-      <c r="H21" t="n">
-        <v>52.7</v>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>3-5</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L21" t="n">
-        <v>47.7</v>
-      </c>
-      <c r="M21" t="n">
-        <v>23.7</v>
-      </c>
-      <c r="N21" t="n">
-        <v>48.4</v>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="P21" t="n">
-        <v>35.4</v>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>언더</t>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>⏭</t>
-        </is>
-      </c>
-      <c r="S21" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="T21" t="inlineStr"/>
-      <c r="U21" t="inlineStr">
-        <is>
-          <t>확률·표본·모델합의 기준 미달</t>
-        </is>
-      </c>
-      <c r="V21" t="n">
-        <v>43.65</v>
-      </c>
-      <c r="W21" t="n">
-        <v>60</v>
-      </c>
-      <c r="X21" t="n">
-        <v>50.8</v>
-      </c>
-      <c r="Y21" t="n">
-        <v>49.2</v>
-      </c>
-      <c r="Z21" t="n">
-        <v>48.7</v>
-      </c>
-      <c r="AA21" t="n">
-        <v>39.4</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>9:10</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Houston Astros</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Atlanta Braves</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E22" t="n">
-        <v>52</v>
-      </c>
-      <c r="F22" t="n">
-        <v>48</v>
-      </c>
-      <c r="G22" t="n">
-        <v>51.1</v>
-      </c>
-      <c r="H22" t="n">
-        <v>48.9</v>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>4-3</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L22" t="n">
-        <v>29.7</v>
-      </c>
-      <c r="M22" t="n">
-        <v>11.3</v>
-      </c>
-      <c r="N22" t="n">
-        <v>44.9</v>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="P22" t="n">
-        <v>30.9</v>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>언더</t>
-        </is>
-      </c>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>⏭</t>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="T22" t="inlineStr"/>
-      <c r="U22" t="inlineStr">
-        <is>
-          <t>확률·표본·모델합의 기준 미달</t>
-        </is>
-      </c>
-      <c r="V22" t="n">
-        <v>40.92</v>
-      </c>
-      <c r="W22" t="n">
-        <v>60</v>
-      </c>
-      <c r="X22" t="n">
-        <v>49.7</v>
-      </c>
-      <c r="Y22" t="n">
-        <v>50.3</v>
-      </c>
-      <c r="Z22" t="n">
-        <v>50</v>
-      </c>
-      <c r="AA22" t="n">
-        <v>37.4</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>9:15</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>St.Louis Cardinals</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Washington Nationals</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E23" t="n">
-        <v>45</v>
-      </c>
-      <c r="F23" t="n">
-        <v>55</v>
-      </c>
-      <c r="G23" t="n">
-        <v>47.3</v>
-      </c>
-      <c r="H23" t="n">
-        <v>52.7</v>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>4-6</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L23" t="n">
-        <v>42.1</v>
-      </c>
-      <c r="M23" t="n">
-        <v>19.4</v>
-      </c>
-      <c r="N23" t="n">
-        <v>54.5</v>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="P23" t="n">
-        <v>33.6</v>
-      </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>언더</t>
-        </is>
-      </c>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t>⏭</t>
-        </is>
-      </c>
-      <c r="S23" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="T23" t="inlineStr"/>
-      <c r="U23" t="inlineStr">
-        <is>
-          <t>확률·표본·모델합의 기준 미달</t>
-        </is>
-      </c>
-      <c r="V23" t="n">
-        <v>43.65</v>
-      </c>
-      <c r="W23" t="n">
-        <v>60</v>
-      </c>
-      <c r="X23" t="n">
-        <v>50.8</v>
-      </c>
-      <c r="Y23" t="n">
-        <v>49.2</v>
-      </c>
-      <c r="Z23" t="n">
-        <v>58.6</v>
-      </c>
-      <c r="AA23" t="n">
-        <v>38.4</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>10:40</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Arizona Diamondbacks</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>New York Yankees</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E24" t="n">
-        <v>54</v>
-      </c>
-      <c r="F24" t="n">
-        <v>46</v>
-      </c>
-      <c r="G24" t="n">
-        <v>51.8</v>
-      </c>
-      <c r="H24" t="n">
-        <v>48.2</v>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>5-4</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L24" t="n">
-        <v>51.8</v>
-      </c>
-      <c r="M24" t="n">
-        <v>27.1</v>
-      </c>
-      <c r="N24" t="n">
-        <v>51.3</v>
-      </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="P24" t="n">
-        <v>32.9</v>
-      </c>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t>언더</t>
-        </is>
-      </c>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t>⏭</t>
-        </is>
-      </c>
-      <c r="S24" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="T24" t="inlineStr"/>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t>확률·표본·모델합의 기준 미달</t>
-        </is>
-      </c>
-      <c r="V24" t="n">
-        <v>43.69</v>
-      </c>
-      <c r="W24" t="n">
-        <v>60</v>
-      </c>
-      <c r="X24" t="n">
-        <v>48.4</v>
-      </c>
-      <c r="Y24" t="n">
-        <v>51.6</v>
-      </c>
-      <c r="Z24" t="n">
-        <v>51.1</v>
-      </c>
-      <c r="AA24" t="n">
-        <v>34.9</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>11:15</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Los Angeles Dodgers</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>San Francisco Giants</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E25" t="n">
-        <v>60</v>
-      </c>
-      <c r="F25" t="n">
-        <v>40</v>
-      </c>
-      <c r="G25" t="n">
-        <v>59.4</v>
-      </c>
-      <c r="H25" t="n">
-        <v>40.6</v>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>5-4</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L25" t="n">
-        <v>42.1</v>
-      </c>
-      <c r="M25" t="n">
-        <v>19.4</v>
-      </c>
-      <c r="N25" t="n">
-        <v>54.3</v>
-      </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="P25" t="n">
-        <v>34.6</v>
-      </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t>언더</t>
-        </is>
-      </c>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>⏭</t>
-        </is>
-      </c>
-      <c r="S25" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="T25" t="inlineStr"/>
-      <c r="U25" t="inlineStr">
-        <is>
-          <t>확률·표본·모델합의 기준 미달</t>
-        </is>
-      </c>
-      <c r="V25" t="n">
-        <v>44.58</v>
-      </c>
-      <c r="W25" t="n">
-        <v>60</v>
-      </c>
-      <c r="X25" t="n">
-        <v>58.5</v>
-      </c>
-      <c r="Y25" t="n">
-        <v>41.5</v>
-      </c>
-      <c r="Z25" t="n">
-        <v>58.4</v>
-      </c>
-      <c r="AA25" t="n">
-        <v>39.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-09-21 14:35
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA15"/>
+  <dimension ref="A1:AA16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -556,39 +556,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>5:10</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Nippon Ham Fighters</t>
+          <t>Los Angeles Dodgers</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>San Francisco Giants</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F2" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G2" t="n">
-        <v>63.4</v>
+        <v>63.9</v>
       </c>
       <c r="H2" t="n">
-        <v>36.6</v>
+        <v>36.1</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>6-4</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -602,13 +602,13 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>60.8</v>
+        <v>53.1</v>
       </c>
       <c r="M2" t="n">
-        <v>35.5</v>
+        <v>28.2</v>
       </c>
       <c r="N2" t="n">
-        <v>40.9</v>
+        <v>54.3</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>24.2</v>
+        <v>32.2</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -644,60 +644,60 @@
         </is>
       </c>
       <c r="V2" t="n">
-        <v>37.3</v>
+        <v>43.21</v>
       </c>
       <c r="W2" t="n">
         <v>60</v>
       </c>
       <c r="X2" t="n">
-        <v>54.9</v>
+        <v>54.8</v>
       </c>
       <c r="Y2" t="n">
-        <v>45.1</v>
+        <v>45.2</v>
       </c>
       <c r="Z2" t="n">
-        <v>34.2</v>
+        <v>54.7</v>
       </c>
       <c r="AA2" t="n">
-        <v>20.4</v>
+        <v>33.6</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>5:10</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>LG Twins</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F3" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G3" t="n">
-        <v>64.09999999999999</v>
+        <v>63.5</v>
       </c>
       <c r="H3" t="n">
-        <v>35.9</v>
+        <v>36.5</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>4-1</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -711,13 +711,13 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>16.3</v>
+        <v>43.5</v>
       </c>
       <c r="M3" t="n">
-        <v>4.7</v>
+        <v>20.4</v>
       </c>
       <c r="N3" t="n">
-        <v>40.1</v>
+        <v>46.3</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>25.4</v>
+        <v>28.8</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -753,65 +753,65 @@
         </is>
       </c>
       <c r="V3" t="n">
-        <v>33.14</v>
+        <v>44.48</v>
       </c>
       <c r="W3" t="n">
         <v>60</v>
       </c>
       <c r="X3" t="n">
-        <v>58.2</v>
+        <v>59.7</v>
       </c>
       <c r="Y3" t="n">
-        <v>41.8</v>
+        <v>40.3</v>
       </c>
       <c r="Z3" t="n">
-        <v>48</v>
+        <v>47.3</v>
       </c>
       <c r="AA3" t="n">
-        <v>32.3</v>
+        <v>31.6</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>65</v>
+        <v>44</v>
       </c>
       <c r="F4" t="n">
-        <v>35</v>
+        <v>56</v>
       </c>
       <c r="G4" t="n">
-        <v>62.5</v>
+        <v>48.2</v>
       </c>
       <c r="H4" t="n">
-        <v>37.5</v>
+        <v>51.8</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -820,21 +820,21 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>46.3</v>
+        <v>28.4</v>
       </c>
       <c r="M4" t="n">
-        <v>22.6</v>
+        <v>10.6</v>
       </c>
       <c r="N4" t="n">
-        <v>52.3</v>
+        <v>34.3</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -843,79 +843,75 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>⏭</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr">
         <is>
-          <t>Forebet·과거모델 합의</t>
+          <t>확률·표본·모델합의 기준 미달</t>
         </is>
       </c>
       <c r="V4" t="n">
-        <v>37.6</v>
+        <v>40.63</v>
       </c>
       <c r="W4" t="n">
         <v>60</v>
       </c>
       <c r="X4" t="n">
-        <v>58.8</v>
+        <v>54.4</v>
       </c>
       <c r="Y4" t="n">
-        <v>41.2</v>
+        <v>45.6</v>
       </c>
       <c r="Z4" t="n">
-        <v>54.3</v>
+        <v>36.2</v>
       </c>
       <c r="AA4" t="n">
-        <v>36.4</v>
+        <v>19.2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>5:10</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="F5" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="G5" t="n">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="H5" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>6-3</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -929,13 +925,13 @@
         </is>
       </c>
       <c r="L5" t="n">
-        <v>39.3</v>
+        <v>50.4</v>
       </c>
       <c r="M5" t="n">
-        <v>17.4</v>
+        <v>25.9</v>
       </c>
       <c r="N5" t="n">
-        <v>47.6</v>
+        <v>40</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -943,7 +939,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>28.7</v>
+        <v>24.8</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -952,41 +948,37 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>⏭</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr">
         <is>
-          <t>Forebet·과거모델 합의</t>
+          <t>확률·표본·모델합의 기준 미달</t>
         </is>
       </c>
       <c r="V5" t="n">
-        <v>43.63</v>
+        <v>43.05</v>
       </c>
       <c r="W5" t="n">
         <v>60</v>
       </c>
       <c r="X5" t="n">
-        <v>59.9</v>
+        <v>57.6</v>
       </c>
       <c r="Y5" t="n">
-        <v>40.1</v>
+        <v>42.4</v>
       </c>
       <c r="Z5" t="n">
-        <v>50.4</v>
+        <v>36.5</v>
       </c>
       <c r="AA5" t="n">
-        <v>32.4</v>
+        <v>24.5</v>
       </c>
     </row>
     <row r="6">
@@ -997,12 +989,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1011,20 +1003,20 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F6" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G6" t="n">
-        <v>57.7</v>
+        <v>55.2</v>
       </c>
       <c r="H6" t="n">
-        <v>42.3</v>
+        <v>44.8</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -1038,13 +1030,13 @@
         </is>
       </c>
       <c r="L6" t="n">
-        <v>3.6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="M6" t="n">
-        <v>0.6</v>
+        <v>2.3</v>
       </c>
       <c r="N6" t="n">
-        <v>26.2</v>
+        <v>29.8</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1052,7 +1044,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>9</v>
+        <v>16.5</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1076,22 +1068,22 @@
         </is>
       </c>
       <c r="V6" t="n">
-        <v>42.64</v>
+        <v>42.09</v>
       </c>
       <c r="W6" t="n">
         <v>60</v>
       </c>
       <c r="X6" t="n">
-        <v>60.2</v>
+        <v>56.9</v>
       </c>
       <c r="Y6" t="n">
-        <v>39.8</v>
+        <v>43.1</v>
       </c>
       <c r="Z6" t="n">
-        <v>33.7</v>
+        <v>36.5</v>
       </c>
       <c r="AA6" t="n">
-        <v>11.8</v>
+        <v>21.3</v>
       </c>
     </row>
     <row r="7">
@@ -1102,12 +1094,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Rakuten Gold. Eagles</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1116,25 +1108,25 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>48</v>
+        <v>52.5</v>
       </c>
       <c r="F7" t="n">
-        <v>52</v>
+        <v>47.5</v>
       </c>
       <c r="G7" t="n">
-        <v>49.7</v>
+        <v>51.5</v>
       </c>
       <c r="H7" t="n">
-        <v>50.3</v>
+        <v>48.5</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -1143,13 +1135,13 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>17.4</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="M7" t="n">
-        <v>5.1</v>
+        <v>1.8</v>
       </c>
       <c r="N7" t="n">
-        <v>27.5</v>
+        <v>23.8</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1157,7 +1149,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>16.5</v>
+        <v>14.9</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1181,65 +1173,65 @@
         </is>
       </c>
       <c r="V7" t="n">
-        <v>41.54</v>
+        <v>41.78</v>
       </c>
       <c r="W7" t="n">
         <v>60</v>
       </c>
       <c r="X7" t="n">
-        <v>52.3</v>
+        <v>49.9</v>
       </c>
       <c r="Y7" t="n">
-        <v>47.7</v>
+        <v>50.1</v>
       </c>
       <c r="Z7" t="n">
-        <v>30.9</v>
+        <v>29</v>
       </c>
       <c r="AA7" t="n">
-        <v>20.3</v>
+        <v>19.2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>2:10</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>Philadelphia Phillies</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="F8" t="n">
-        <v>56</v>
+        <v>39</v>
       </c>
       <c r="G8" t="n">
-        <v>46.5</v>
+        <v>59</v>
       </c>
       <c r="H8" t="n">
-        <v>53.5</v>
+        <v>41</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1248,21 +1240,21 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>8.9</v>
+        <v>40.7</v>
       </c>
       <c r="M8" t="n">
-        <v>2</v>
+        <v>18.4</v>
       </c>
       <c r="N8" t="n">
-        <v>25.6</v>
+        <v>52</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>언더</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>14.5</v>
+        <v>30.6</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1286,65 +1278,65 @@
         </is>
       </c>
       <c r="V8" t="n">
-        <v>39.49</v>
+        <v>43.75</v>
       </c>
       <c r="W8" t="n">
         <v>60</v>
       </c>
       <c r="X8" t="n">
-        <v>50.3</v>
+        <v>56.1</v>
       </c>
       <c r="Y8" t="n">
-        <v>49.7</v>
+        <v>43.9</v>
       </c>
       <c r="Z8" t="n">
-        <v>31.1</v>
+        <v>55.8</v>
       </c>
       <c r="AA8" t="n">
-        <v>18.7</v>
+        <v>34.6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>2:40</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>Tampa Bay Rays</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>Boston Red Sox</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="F9" t="n">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="G9" t="n">
-        <v>47.3</v>
+        <v>49.8</v>
       </c>
       <c r="H9" t="n">
-        <v>52.7</v>
+        <v>50.2</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1353,21 +1345,21 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>14.3</v>
+        <v>27.1</v>
       </c>
       <c r="M9" t="n">
-        <v>3.9</v>
+        <v>9.9</v>
       </c>
       <c r="N9" t="n">
-        <v>24.9</v>
+        <v>39.4</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>언더</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>12.2</v>
+        <v>21.6</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1391,65 +1383,65 @@
         </is>
       </c>
       <c r="V9" t="n">
-        <v>41.18</v>
+        <v>42.58</v>
       </c>
       <c r="W9" t="n">
         <v>60</v>
       </c>
       <c r="X9" t="n">
-        <v>50.8</v>
+        <v>45</v>
       </c>
       <c r="Y9" t="n">
-        <v>49.2</v>
+        <v>55</v>
       </c>
       <c r="Z9" t="n">
-        <v>28.4</v>
+        <v>43.6</v>
       </c>
       <c r="AA9" t="n">
-        <v>15</v>
+        <v>25.5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>3:10</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Chiba Lotte Marines</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Seibu Lions</t>
+          <t>Detroit Tigers</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="F10" t="n">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="G10" t="n">
-        <v>49.4</v>
+        <v>52.3</v>
       </c>
       <c r="H10" t="n">
-        <v>50.6</v>
+        <v>47.7</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1458,21 +1450,21 @@
         </is>
       </c>
       <c r="L10" t="n">
-        <v>8.9</v>
+        <v>12.3</v>
       </c>
       <c r="M10" t="n">
-        <v>2</v>
+        <v>3.1</v>
       </c>
       <c r="N10" t="n">
-        <v>25.6</v>
+        <v>39.9</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>언더</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>14.5</v>
+        <v>28.4</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1496,65 +1488,65 @@
         </is>
       </c>
       <c r="V10" t="n">
-        <v>41.54</v>
+        <v>42.55</v>
       </c>
       <c r="W10" t="n">
         <v>60</v>
       </c>
       <c r="X10" t="n">
-        <v>53.1</v>
+        <v>48.3</v>
       </c>
       <c r="Y10" t="n">
-        <v>46.9</v>
+        <v>51.7</v>
       </c>
       <c r="Z10" t="n">
-        <v>31.1</v>
+        <v>49.1</v>
       </c>
       <c r="AA10" t="n">
-        <v>18.7</v>
+        <v>36.9</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>3:10</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>Houston Astros</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>Atlanta Braves</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>61</v>
+        <v>48</v>
       </c>
       <c r="F11" t="n">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="G11" t="n">
-        <v>60.9</v>
+        <v>52</v>
       </c>
       <c r="H11" t="n">
-        <v>39.1</v>
+        <v>48</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1563,13 +1555,13 @@
         </is>
       </c>
       <c r="L11" t="n">
-        <v>57</v>
+        <v>19.7</v>
       </c>
       <c r="M11" t="n">
-        <v>31.8</v>
+        <v>6.1</v>
       </c>
       <c r="N11" t="n">
-        <v>57.9</v>
+        <v>39.4</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1577,11 +1569,11 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>41.1</v>
+        <v>27.1</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -1601,65 +1593,65 @@
         </is>
       </c>
       <c r="V11" t="n">
-        <v>42.9</v>
+        <v>43.14</v>
       </c>
       <c r="W11" t="n">
         <v>60</v>
       </c>
       <c r="X11" t="n">
-        <v>60.7</v>
+        <v>58</v>
       </c>
       <c r="Y11" t="n">
-        <v>39.3</v>
+        <v>42</v>
       </c>
       <c r="Z11" t="n">
-        <v>58.3</v>
+        <v>46</v>
       </c>
       <c r="AA11" t="n">
-        <v>44.2</v>
+        <v>34.1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>3:15</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>KT Wiz Suwon</t>
+          <t>St.Louis Cardinals</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>Washington Nationals</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E12" t="n">
+        <v>43</v>
+      </c>
+      <c r="F12" t="n">
         <v>57</v>
       </c>
-      <c r="F12" t="n">
-        <v>43</v>
-      </c>
       <c r="G12" t="n">
-        <v>57.4</v>
+        <v>42.7</v>
       </c>
       <c r="H12" t="n">
-        <v>42.6</v>
+        <v>57.3</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>6-3</t>
+          <t>4-6</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1668,13 +1660,13 @@
         </is>
       </c>
       <c r="L12" t="n">
-        <v>54.4</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="M12" t="n">
-        <v>29.4</v>
+        <v>39.2</v>
       </c>
       <c r="N12" t="n">
-        <v>57.7</v>
+        <v>53.9</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1682,11 +1674,11 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>40.7</v>
+        <v>34</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -1706,60 +1698,60 @@
         </is>
       </c>
       <c r="V12" t="n">
-        <v>42.3</v>
+        <v>42.32</v>
       </c>
       <c r="W12" t="n">
         <v>60</v>
       </c>
       <c r="X12" t="n">
-        <v>58.1</v>
+        <v>42.4</v>
       </c>
       <c r="Y12" t="n">
-        <v>41.9</v>
+        <v>57.6</v>
       </c>
       <c r="Z12" t="n">
-        <v>58.7</v>
+        <v>50.4</v>
       </c>
       <c r="AA12" t="n">
-        <v>44.4</v>
+        <v>32.3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>3:35</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Lotte Giants</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>Toronto Blue Jays</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="F13" t="n">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="G13" t="n">
-        <v>55.5</v>
+        <v>58.7</v>
       </c>
       <c r="H13" t="n">
-        <v>44.5</v>
+        <v>41.3</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>8-7</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1773,25 +1765,25 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>90.90000000000001</v>
+        <v>6.2</v>
       </c>
       <c r="M13" t="n">
-        <v>76.5</v>
+        <v>1.2</v>
       </c>
       <c r="N13" t="n">
-        <v>64.3</v>
+        <v>39.2</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>오버</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>48</v>
+        <v>28.9</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -1811,38 +1803,38 @@
         </is>
       </c>
       <c r="V13" t="n">
-        <v>40.29</v>
+        <v>43.78</v>
       </c>
       <c r="W13" t="n">
         <v>60</v>
       </c>
       <c r="X13" t="n">
-        <v>57.7</v>
+        <v>58.3</v>
       </c>
       <c r="Y13" t="n">
-        <v>42.3</v>
+        <v>41.7</v>
       </c>
       <c r="Z13" t="n">
-        <v>55.4</v>
+        <v>50.2</v>
       </c>
       <c r="AA13" t="n">
-        <v>38.5</v>
+        <v>38.1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>5:10</t>
+          <t>4:10</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>Colorado Rockies</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Boston Red Sox</t>
+          <t>Seattle Mariners</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1851,25 +1843,25 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="F14" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="G14" t="n">
-        <v>51.4</v>
+        <v>48.3</v>
       </c>
       <c r="H14" t="n">
-        <v>48.6</v>
+        <v>51.7</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>6-4</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1878,13 +1870,13 @@
         </is>
       </c>
       <c r="L14" t="n">
-        <v>39.3</v>
+        <v>47.7</v>
       </c>
       <c r="M14" t="n">
-        <v>17.4</v>
+        <v>23.7</v>
       </c>
       <c r="N14" t="n">
-        <v>47.6</v>
+        <v>51.5</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1892,7 +1884,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>28.7</v>
+        <v>31.7</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1916,38 +1908,38 @@
         </is>
       </c>
       <c r="V14" t="n">
-        <v>42.08</v>
+        <v>43.78</v>
       </c>
       <c r="W14" t="n">
         <v>60</v>
       </c>
       <c r="X14" t="n">
-        <v>50.5</v>
+        <v>51.7</v>
       </c>
       <c r="Y14" t="n">
-        <v>49.5</v>
+        <v>48.3</v>
       </c>
       <c r="Z14" t="n">
-        <v>50.4</v>
+        <v>52.8</v>
       </c>
       <c r="AA14" t="n">
-        <v>32.4</v>
+        <v>34.3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>7:10</t>
+          <t>5:10</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Cleveland Guardians</t>
+          <t>Arizona Diamondbacks</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Athletics</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1956,25 +1948,25 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>59</v>
+        <v>46</v>
       </c>
       <c r="F15" t="n">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="G15" t="n">
-        <v>57.2</v>
+        <v>48.3</v>
       </c>
       <c r="H15" t="n">
-        <v>42.8</v>
+        <v>51.7</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1983,13 +1975,13 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>33.8</v>
+        <v>51.8</v>
       </c>
       <c r="M15" t="n">
-        <v>13.8</v>
+        <v>27.1</v>
       </c>
       <c r="N15" t="n">
-        <v>46</v>
+        <v>54.1</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1997,7 +1989,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>33.7</v>
+        <v>32.2</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -2021,22 +2013,127 @@
         </is>
       </c>
       <c r="V15" t="n">
-        <v>44.6</v>
+        <v>43.76</v>
       </c>
       <c r="W15" t="n">
         <v>60</v>
       </c>
       <c r="X15" t="n">
-        <v>54.5</v>
+        <v>51.7</v>
       </c>
       <c r="Y15" t="n">
-        <v>45.5</v>
+        <v>48.3</v>
       </c>
       <c r="Z15" t="n">
-        <v>50.1</v>
+        <v>54.9</v>
       </c>
       <c r="AA15" t="n">
-        <v>40.3</v>
+        <v>33.9</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>8:20</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Baltimore Orioles</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>36</v>
+      </c>
+      <c r="F16" t="n">
+        <v>64</v>
+      </c>
+      <c r="G16" t="n">
+        <v>39.6</v>
+      </c>
+      <c r="H16" t="n">
+        <v>60.4</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>5-7</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L16" t="n">
+        <v>63.2</v>
+      </c>
+      <c r="M16" t="n">
+        <v>37.9</v>
+      </c>
+      <c r="N16" t="n">
+        <v>52.7</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P16" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>언더</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V16" t="n">
+        <v>40.61</v>
+      </c>
+      <c r="W16" t="n">
+        <v>60</v>
+      </c>
+      <c r="X16" t="n">
+        <v>44.9</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>55.1</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>49.2</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>33.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-09-22 14:20
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA7"/>
+  <dimension ref="A1:AA18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -556,17 +556,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Rakuten Gold. Eagles</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -575,20 +575,20 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="F2" t="n">
-        <v>56</v>
+        <v>73</v>
       </c>
       <c r="G2" t="n">
-        <v>48.2</v>
+        <v>33.8</v>
       </c>
       <c r="H2" t="n">
-        <v>51.8</v>
+        <v>66.2</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -602,13 +602,13 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>28.4</v>
+        <v>36.6</v>
       </c>
       <c r="M2" t="n">
-        <v>10.6</v>
+        <v>15.5</v>
       </c>
       <c r="N2" t="n">
-        <v>34.3</v>
+        <v>33.8</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>17</v>
+        <v>20.4</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -625,53 +625,57 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>⏭</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr"/>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>원정승</t>
+        </is>
+      </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>확률·표본·모델합의 기준 미달</t>
+          <t>Forebet·과거모델 합의</t>
         </is>
       </c>
       <c r="V2" t="n">
-        <v>40.63</v>
+        <v>24.51</v>
       </c>
       <c r="W2" t="n">
         <v>60</v>
       </c>
       <c r="X2" t="n">
-        <v>54.4</v>
+        <v>44.1</v>
       </c>
       <c r="Y2" t="n">
-        <v>45.6</v>
+        <v>55.9</v>
       </c>
       <c r="Z2" t="n">
-        <v>36.2</v>
+        <v>32.8</v>
       </c>
       <c r="AA2" t="n">
-        <v>19.2</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Nippon Ham Fighters</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -680,20 +684,20 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="F3" t="n">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="G3" t="n">
-        <v>59</v>
+        <v>62.4</v>
       </c>
       <c r="H3" t="n">
-        <v>41</v>
+        <v>37.6</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>6-3</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -707,21 +711,21 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>50.4</v>
+        <v>17.4</v>
       </c>
       <c r="M3" t="n">
-        <v>25.9</v>
+        <v>5.1</v>
       </c>
       <c r="N3" t="n">
-        <v>40</v>
+        <v>28.2</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>24.8</v>
+        <v>15.2</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -730,75 +734,79 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>⏭</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr"/>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>확률·표본·모델합의 기준 미달</t>
+          <t>Forebet·과거모델 합의</t>
         </is>
       </c>
       <c r="V3" t="n">
-        <v>43.05</v>
+        <v>37.79</v>
       </c>
       <c r="W3" t="n">
         <v>60</v>
       </c>
       <c r="X3" t="n">
-        <v>57.6</v>
+        <v>54</v>
       </c>
       <c r="Y3" t="n">
-        <v>42.4</v>
+        <v>46</v>
       </c>
       <c r="Z3" t="n">
-        <v>36.5</v>
+        <v>31.8</v>
       </c>
       <c r="AA3" t="n">
-        <v>24.5</v>
+        <v>18.5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>Samsung Lions</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="F4" t="n">
-        <v>46</v>
+        <v>33</v>
       </c>
       <c r="G4" t="n">
-        <v>55.2</v>
+        <v>63.8</v>
       </c>
       <c r="H4" t="n">
-        <v>44.8</v>
+        <v>36.2</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>7-4</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -812,98 +820,102 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>9.699999999999999</v>
+        <v>74</v>
       </c>
       <c r="M4" t="n">
-        <v>2.3</v>
+        <v>50.4</v>
       </c>
       <c r="N4" t="n">
-        <v>29.8</v>
+        <v>62.8</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>언더</t>
+          <t>오버</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>16.5</v>
+        <v>44.6</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>언더</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>⏭</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr"/>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>확률·표본·모델합의 기준 미달</t>
+          <t>Forebet·과거모델 합의</t>
         </is>
       </c>
       <c r="V4" t="n">
-        <v>42.09</v>
+        <v>35.78</v>
       </c>
       <c r="W4" t="n">
         <v>60</v>
       </c>
       <c r="X4" t="n">
-        <v>56.9</v>
+        <v>58.9</v>
       </c>
       <c r="Y4" t="n">
-        <v>43.1</v>
+        <v>41.1</v>
       </c>
       <c r="Z4" t="n">
-        <v>36.5</v>
+        <v>59</v>
       </c>
       <c r="AA4" t="n">
-        <v>21.3</v>
+        <v>42.7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>10:40</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>Seattle Mariners</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>Houston Astros</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>52.5</v>
+        <v>66</v>
       </c>
       <c r="F5" t="n">
-        <v>47.5</v>
+        <v>34</v>
       </c>
       <c r="G5" t="n">
-        <v>51.5</v>
+        <v>62.9</v>
       </c>
       <c r="H5" t="n">
-        <v>48.5</v>
+        <v>37.1</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>6-3</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -917,76 +929,80 @@
         </is>
       </c>
       <c r="L5" t="n">
-        <v>8.199999999999999</v>
+        <v>53.1</v>
       </c>
       <c r="M5" t="n">
-        <v>1.8</v>
+        <v>28.2</v>
       </c>
       <c r="N5" t="n">
-        <v>23.8</v>
+        <v>52.7</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P5" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
           <t>언더</t>
         </is>
       </c>
-      <c r="P5" t="n">
-        <v>14.9</v>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>언더</t>
-        </is>
-      </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>⏭</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr"/>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>확률·표본·모델합의 기준 미달</t>
+          <t>Forebet·과거모델 합의</t>
         </is>
       </c>
       <c r="V5" t="n">
-        <v>41.78</v>
+        <v>43.59</v>
       </c>
       <c r="W5" t="n">
         <v>60</v>
       </c>
       <c r="X5" t="n">
-        <v>49.9</v>
+        <v>58.3</v>
       </c>
       <c r="Y5" t="n">
-        <v>50.1</v>
+        <v>41.7</v>
       </c>
       <c r="Z5" t="n">
-        <v>29</v>
+        <v>52.5</v>
       </c>
       <c r="AA5" t="n">
-        <v>19.2</v>
+        <v>33.6</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>7:35</t>
+          <t>11:10</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>Los Angeles Dodgers</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Toronto Blue Jays</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -995,25 +1011,25 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>46</v>
+        <v>71</v>
       </c>
       <c r="F6" t="n">
-        <v>54</v>
+        <v>29</v>
       </c>
       <c r="G6" t="n">
-        <v>48.3</v>
+        <v>64.7</v>
       </c>
       <c r="H6" t="n">
-        <v>51.7</v>
+        <v>35.3</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>5-6</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -1022,13 +1038,13 @@
         </is>
       </c>
       <c r="L6" t="n">
-        <v>71</v>
+        <v>53.1</v>
       </c>
       <c r="M6" t="n">
-        <v>46.7</v>
+        <v>28.2</v>
       </c>
       <c r="N6" t="n">
-        <v>51.8</v>
+        <v>52.7</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1036,7 +1052,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>32</v>
+        <v>32.3</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1045,58 +1061,62 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>⏭</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr"/>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>확률·표본·모델합의 기준 미달</t>
+          <t>Forebet·과거모델 합의</t>
         </is>
       </c>
       <c r="V6" t="n">
-        <v>43.5</v>
+        <v>41.96</v>
       </c>
       <c r="W6" t="n">
         <v>60</v>
       </c>
       <c r="X6" t="n">
-        <v>51.7</v>
+        <v>55.2</v>
       </c>
       <c r="Y6" t="n">
-        <v>48.3</v>
+        <v>44.8</v>
       </c>
       <c r="Z6" t="n">
-        <v>45.4</v>
+        <v>52.5</v>
       </c>
       <c r="AA6" t="n">
-        <v>27.1</v>
+        <v>33.6</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>10:45</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>San Francisco Giants</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -1106,14 +1126,14 @@
         <v>42</v>
       </c>
       <c r="G7" t="n">
-        <v>55.8</v>
+        <v>59</v>
       </c>
       <c r="H7" t="n">
-        <v>44.2</v>
+        <v>41</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>6-3</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1127,21 +1147,21 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>51.8</v>
+        <v>27.1</v>
       </c>
       <c r="M7" t="n">
-        <v>27.1</v>
+        <v>9.9</v>
       </c>
       <c r="N7" t="n">
-        <v>54.1</v>
+        <v>33.9</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>32.2</v>
+        <v>16.7</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1165,22 +1185,1177 @@
         </is>
       </c>
       <c r="V7" t="n">
-        <v>43.77</v>
+        <v>41.63</v>
       </c>
       <c r="W7" t="n">
         <v>60</v>
       </c>
       <c r="X7" t="n">
-        <v>52.4</v>
+        <v>60.5</v>
       </c>
       <c r="Y7" t="n">
-        <v>47.6</v>
+        <v>39.5</v>
       </c>
       <c r="Z7" t="n">
-        <v>54.9</v>
+        <v>36.2</v>
       </c>
       <c r="AA7" t="n">
-        <v>33.9</v>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Chiba Lotte Marines</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Orix Buffaloes</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>NPB</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>40</v>
+      </c>
+      <c r="F8" t="n">
+        <v>60</v>
+      </c>
+      <c r="G8" t="n">
+        <v>42.6</v>
+      </c>
+      <c r="H8" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>3-5</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
+        <v>15.3</v>
+      </c>
+      <c r="M8" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="N8" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>언더</t>
+        </is>
+      </c>
+      <c r="P8" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>언더</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V8" t="n">
+        <v>39.8</v>
+      </c>
+      <c r="W8" t="n">
+        <v>60</v>
+      </c>
+      <c r="X8" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>53.5</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>32.4</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>16.6</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Kiwoom Heroes</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Doosan Bears</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>36</v>
+      </c>
+      <c r="F9" t="n">
+        <v>64</v>
+      </c>
+      <c r="G9" t="n">
+        <v>41.1</v>
+      </c>
+      <c r="H9" t="n">
+        <v>58.9</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>4-8</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L9" t="n">
+        <v>80.2</v>
+      </c>
+      <c r="M9" t="n">
+        <v>58.7</v>
+      </c>
+      <c r="N9" t="n">
+        <v>64.8</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>오버</t>
+        </is>
+      </c>
+      <c r="P9" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V9" t="n">
+        <v>37.29</v>
+      </c>
+      <c r="W9" t="n">
+        <v>60</v>
+      </c>
+      <c r="X9" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>51.3</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>59.7</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>43.5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>SSG Landers</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>KT Wiz Suwon</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>53</v>
+      </c>
+      <c r="F10" t="n">
+        <v>47</v>
+      </c>
+      <c r="G10" t="n">
+        <v>55.5</v>
+      </c>
+      <c r="H10" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>5-3</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L10" t="n">
+        <v>23.3</v>
+      </c>
+      <c r="M10" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="N10" t="n">
+        <v>40.1</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P10" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>언더</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V10" t="n">
+        <v>40.16</v>
+      </c>
+      <c r="W10" t="n">
+        <v>60</v>
+      </c>
+      <c r="X10" t="n">
+        <v>59.2</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>40.8</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>45.7</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>32.9</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Hanwha Eagles</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Lotte Giants</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>52</v>
+      </c>
+      <c r="F11" t="n">
+        <v>48</v>
+      </c>
+      <c r="G11" t="n">
+        <v>51.6</v>
+      </c>
+      <c r="H11" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>6-4</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L11" t="n">
+        <v>46.3</v>
+      </c>
+      <c r="M11" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="N11" t="n">
+        <v>53.7</v>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P11" t="n">
+        <v>33.4</v>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>언더</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V11" t="n">
+        <v>39.47</v>
+      </c>
+      <c r="W11" t="n">
+        <v>60</v>
+      </c>
+      <c r="X11" t="n">
+        <v>51.1</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>48.9</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>56.1</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2:05</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>New York Yankees</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>56</v>
+      </c>
+      <c r="F12" t="n">
+        <v>44</v>
+      </c>
+      <c r="G12" t="n">
+        <v>56</v>
+      </c>
+      <c r="H12" t="n">
+        <v>44</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L12" t="n">
+        <v>28.4</v>
+      </c>
+      <c r="M12" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="N12" t="n">
+        <v>40.3</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P12" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>언더</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V12" t="n">
+        <v>45.35</v>
+      </c>
+      <c r="W12" t="n">
+        <v>60</v>
+      </c>
+      <c r="X12" t="n">
+        <v>55.9</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>44.1</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>44.3</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>25.7</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>7:40</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Philadelphia Phillies</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>41</v>
+      </c>
+      <c r="F13" t="n">
+        <v>59</v>
+      </c>
+      <c r="G13" t="n">
+        <v>43.3</v>
+      </c>
+      <c r="H13" t="n">
+        <v>56.7</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>4-5</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
+        <v>51.8</v>
+      </c>
+      <c r="M13" t="n">
+        <v>27.1</v>
+      </c>
+      <c r="N13" t="n">
+        <v>53.3</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P13" t="n">
+        <v>33.5</v>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>언더</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V13" t="n">
+        <v>41.13</v>
+      </c>
+      <c r="W13" t="n">
+        <v>60</v>
+      </c>
+      <c r="X13" t="n">
+        <v>46.9</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>53.1</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>53.8</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>35.7</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>7:45</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Boston Red Sox</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>47</v>
+      </c>
+      <c r="F14" t="n">
+        <v>53</v>
+      </c>
+      <c r="G14" t="n">
+        <v>48.9</v>
+      </c>
+      <c r="H14" t="n">
+        <v>51.1</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>4-6</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L14" t="n">
+        <v>63.2</v>
+      </c>
+      <c r="M14" t="n">
+        <v>37.9</v>
+      </c>
+      <c r="N14" t="n">
+        <v>51.9</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P14" t="n">
+        <v>34.2</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>언더</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V14" t="n">
+        <v>43.29</v>
+      </c>
+      <c r="W14" t="n">
+        <v>60</v>
+      </c>
+      <c r="X14" t="n">
+        <v>51.7</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>48.3</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>48.2</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>9:05</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Texas Rangers</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>New York Mets</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>62</v>
+      </c>
+      <c r="F15" t="n">
+        <v>38</v>
+      </c>
+      <c r="G15" t="n">
+        <v>60.6</v>
+      </c>
+      <c r="H15" t="n">
+        <v>39.4</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>6-3</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L15" t="n">
+        <v>54.4</v>
+      </c>
+      <c r="M15" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="N15" t="n">
+        <v>53.3</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P15" t="n">
+        <v>36.9</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>언더</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V15" t="n">
+        <v>41.33</v>
+      </c>
+      <c r="W15" t="n">
+        <v>60</v>
+      </c>
+      <c r="X15" t="n">
+        <v>58.4</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>39.3</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>9:40</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Colorado Rockies</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>39</v>
+      </c>
+      <c r="F16" t="n">
+        <v>61</v>
+      </c>
+      <c r="G16" t="n">
+        <v>42.2</v>
+      </c>
+      <c r="H16" t="n">
+        <v>57.8</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>4-8</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L16" t="n">
+        <v>80.90000000000001</v>
+      </c>
+      <c r="M16" t="n">
+        <v>59.8</v>
+      </c>
+      <c r="N16" t="n">
+        <v>64</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>오버</t>
+        </is>
+      </c>
+      <c r="P16" t="n">
+        <v>45</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V16" t="n">
+        <v>40.3</v>
+      </c>
+      <c r="W16" t="n">
+        <v>60</v>
+      </c>
+      <c r="X16" t="n">
+        <v>46.9</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>53.1</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>58.4</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>40.1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Athletics</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Los Angeles Angels</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>47</v>
+      </c>
+      <c r="F17" t="n">
+        <v>53</v>
+      </c>
+      <c r="G17" t="n">
+        <v>48.9</v>
+      </c>
+      <c r="H17" t="n">
+        <v>51.1</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>6-7</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L17" t="n">
+        <v>85.8</v>
+      </c>
+      <c r="M17" t="n">
+        <v>67.3</v>
+      </c>
+      <c r="N17" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>오버</t>
+        </is>
+      </c>
+      <c r="P17" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr"/>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V17" t="n">
+        <v>43.16</v>
+      </c>
+      <c r="W17" t="n">
+        <v>60</v>
+      </c>
+      <c r="X17" t="n">
+        <v>51.7</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>48.3</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>60.4</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>42.6</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>10:45</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>San Francisco Giants</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Minnesota Twins</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>54</v>
+      </c>
+      <c r="F18" t="n">
+        <v>46</v>
+      </c>
+      <c r="G18" t="n">
+        <v>51.4</v>
+      </c>
+      <c r="H18" t="n">
+        <v>48.6</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L18" t="n">
+        <v>51.8</v>
+      </c>
+      <c r="M18" t="n">
+        <v>27.1</v>
+      </c>
+      <c r="N18" t="n">
+        <v>53.3</v>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P18" t="n">
+        <v>33.5</v>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>언더</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr"/>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V18" t="n">
+        <v>42.45</v>
+      </c>
+      <c r="W18" t="n">
+        <v>60</v>
+      </c>
+      <c r="X18" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>52.5</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>53.8</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>35.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-09-23 15:11
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA18"/>
+  <dimension ref="A1:AA13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -556,7 +556,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -575,20 +575,20 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F2" t="n">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="G2" t="n">
-        <v>33.8</v>
+        <v>31.3</v>
       </c>
       <c r="H2" t="n">
-        <v>66.2</v>
+        <v>68.7</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>2-4</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -602,13 +602,13 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>36.6</v>
+        <v>17.4</v>
       </c>
       <c r="M2" t="n">
-        <v>15.5</v>
+        <v>5.1</v>
       </c>
       <c r="N2" t="n">
-        <v>33.8</v>
+        <v>27.9</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>20.4</v>
+        <v>14.1</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -644,22 +644,22 @@
         </is>
       </c>
       <c r="V2" t="n">
-        <v>24.51</v>
+        <v>16.48</v>
       </c>
       <c r="W2" t="n">
         <v>60</v>
       </c>
       <c r="X2" t="n">
-        <v>44.1</v>
+        <v>43.8</v>
       </c>
       <c r="Y2" t="n">
-        <v>55.9</v>
+        <v>56.2</v>
       </c>
       <c r="Z2" t="n">
-        <v>32.8</v>
+        <v>31.5</v>
       </c>
       <c r="AA2" t="n">
-        <v>22</v>
+        <v>17.1</v>
       </c>
     </row>
     <row r="3">
@@ -684,20 +684,20 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="F3" t="n">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="G3" t="n">
-        <v>62.4</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="H3" t="n">
-        <v>37.6</v>
+        <v>34.9</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -711,13 +711,13 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>17.4</v>
+        <v>27.1</v>
       </c>
       <c r="M3" t="n">
-        <v>5.1</v>
+        <v>9.9</v>
       </c>
       <c r="N3" t="n">
-        <v>28.2</v>
+        <v>33.2</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>15.2</v>
+        <v>16.7</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -753,60 +753,60 @@
         </is>
       </c>
       <c r="V3" t="n">
-        <v>37.79</v>
+        <v>31.41</v>
       </c>
       <c r="W3" t="n">
         <v>60</v>
       </c>
       <c r="X3" t="n">
-        <v>54</v>
+        <v>53.2</v>
       </c>
       <c r="Y3" t="n">
-        <v>46</v>
+        <v>46.8</v>
       </c>
       <c r="Z3" t="n">
-        <v>31.8</v>
+        <v>35.2</v>
       </c>
       <c r="AA3" t="n">
-        <v>18.5</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="F4" t="n">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="G4" t="n">
-        <v>63.8</v>
+        <v>58.7</v>
       </c>
       <c r="H4" t="n">
-        <v>36.2</v>
+        <v>41.3</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>7-4</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -820,107 +820,103 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>74</v>
+        <v>35.2</v>
       </c>
       <c r="M4" t="n">
-        <v>50.4</v>
+        <v>14.6</v>
       </c>
       <c r="N4" t="n">
-        <v>62.8</v>
+        <v>34.5</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>오버</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>44.6</v>
+        <v>21.2</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
+          <t>언더</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>★★</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
+      <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr">
         <is>
-          <t>Forebet·과거모델 합의</t>
+          <t>확률·표본·모델합의 기준 미달</t>
         </is>
       </c>
       <c r="V4" t="n">
-        <v>35.78</v>
+        <v>41.5</v>
       </c>
       <c r="W4" t="n">
         <v>60</v>
       </c>
       <c r="X4" t="n">
-        <v>58.9</v>
+        <v>59.8</v>
       </c>
       <c r="Y4" t="n">
-        <v>41.1</v>
+        <v>40.2</v>
       </c>
       <c r="Z4" t="n">
-        <v>59</v>
+        <v>34.2</v>
       </c>
       <c r="AA4" t="n">
-        <v>42.7</v>
+        <v>23.4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Seattle Mariners</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Houston Astros</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="F5" t="n">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="G5" t="n">
-        <v>62.9</v>
+        <v>51</v>
       </c>
       <c r="H5" t="n">
-        <v>37.1</v>
+        <v>49</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>6-3</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -929,107 +925,103 @@
         </is>
       </c>
       <c r="L5" t="n">
-        <v>53.1</v>
+        <v>18.5</v>
       </c>
       <c r="M5" t="n">
-        <v>28.2</v>
+        <v>5.6</v>
       </c>
       <c r="N5" t="n">
-        <v>52.7</v>
+        <v>29.1</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
+          <t>언더</t>
+        </is>
+      </c>
+      <c r="P5" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>언더</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="P5" t="n">
-        <v>32.3</v>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>언더</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>★★</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
+      <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr">
         <is>
-          <t>Forebet·과거모델 합의</t>
+          <t>확률·표본·모델합의 기준 미달</t>
         </is>
       </c>
       <c r="V5" t="n">
-        <v>43.59</v>
+        <v>41.49</v>
       </c>
       <c r="W5" t="n">
         <v>60</v>
       </c>
       <c r="X5" t="n">
-        <v>58.3</v>
+        <v>55.5</v>
       </c>
       <c r="Y5" t="n">
-        <v>41.7</v>
+        <v>44.5</v>
       </c>
       <c r="Z5" t="n">
-        <v>52.5</v>
+        <v>32.6</v>
       </c>
       <c r="AA5" t="n">
-        <v>33.6</v>
+        <v>18.4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>11:10</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="F6" t="n">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="G6" t="n">
-        <v>64.7</v>
+        <v>42.5</v>
       </c>
       <c r="H6" t="n">
-        <v>35.3</v>
+        <v>57.5</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -1038,13 +1030,13 @@
         </is>
       </c>
       <c r="L6" t="n">
-        <v>53.1</v>
+        <v>29.7</v>
       </c>
       <c r="M6" t="n">
-        <v>28.2</v>
+        <v>11.3</v>
       </c>
       <c r="N6" t="n">
-        <v>52.7</v>
+        <v>43</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1052,7 +1044,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>32.3</v>
+        <v>26.6</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1061,79 +1053,75 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>⏭</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr">
         <is>
-          <t>Forebet·과거모델 합의</t>
+          <t>확률·표본·모델합의 기준 미달</t>
         </is>
       </c>
       <c r="V6" t="n">
-        <v>41.96</v>
+        <v>41.42</v>
       </c>
       <c r="W6" t="n">
         <v>60</v>
       </c>
       <c r="X6" t="n">
-        <v>55.2</v>
+        <v>43.2</v>
       </c>
       <c r="Y6" t="n">
-        <v>44.8</v>
+        <v>56.8</v>
       </c>
       <c r="Z6" t="n">
-        <v>52.5</v>
+        <v>47.5</v>
       </c>
       <c r="AA6" t="n">
-        <v>33.6</v>
+        <v>31.7</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="F7" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="G7" t="n">
-        <v>59</v>
+        <v>55.5</v>
       </c>
       <c r="H7" t="n">
-        <v>41</v>
+        <v>44.5</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1147,25 +1135,25 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>27.1</v>
+        <v>58.3</v>
       </c>
       <c r="M7" t="n">
-        <v>9.9</v>
+        <v>33</v>
       </c>
       <c r="N7" t="n">
-        <v>33.9</v>
+        <v>58.8</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>언더</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>16.7</v>
+        <v>43.6</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>언더</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1185,65 +1173,65 @@
         </is>
       </c>
       <c r="V7" t="n">
-        <v>41.63</v>
+        <v>40.75</v>
       </c>
       <c r="W7" t="n">
         <v>60</v>
       </c>
       <c r="X7" t="n">
-        <v>60.5</v>
+        <v>57.8</v>
       </c>
       <c r="Y7" t="n">
-        <v>39.5</v>
+        <v>42.2</v>
       </c>
       <c r="Z7" t="n">
-        <v>36.2</v>
+        <v>58.9</v>
       </c>
       <c r="AA7" t="n">
-        <v>19</v>
+        <v>47.2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Chiba Lotte Marines</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>Lotte Giants</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="F8" t="n">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="G8" t="n">
-        <v>42.6</v>
+        <v>51.8</v>
       </c>
       <c r="H8" t="n">
-        <v>57.4</v>
+        <v>48.2</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1252,21 +1240,21 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>15.3</v>
+        <v>35.2</v>
       </c>
       <c r="M8" t="n">
-        <v>4.3</v>
+        <v>14.6</v>
       </c>
       <c r="N8" t="n">
-        <v>28.2</v>
+        <v>44.4</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>언더</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>13.5</v>
+        <v>30</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1290,65 +1278,65 @@
         </is>
       </c>
       <c r="V8" t="n">
-        <v>39.8</v>
+        <v>40.33</v>
       </c>
       <c r="W8" t="n">
         <v>60</v>
       </c>
       <c r="X8" t="n">
-        <v>46.5</v>
+        <v>51.6</v>
       </c>
       <c r="Y8" t="n">
-        <v>53.5</v>
+        <v>48.4</v>
       </c>
       <c r="Z8" t="n">
-        <v>32.4</v>
+        <v>47.5</v>
       </c>
       <c r="AA8" t="n">
-        <v>16.6</v>
+        <v>35.1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>4:45</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>San Francisco Giants</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>36</v>
+        <v>57</v>
       </c>
       <c r="F9" t="n">
-        <v>64</v>
+        <v>43</v>
       </c>
       <c r="G9" t="n">
-        <v>41.1</v>
+        <v>57.1</v>
       </c>
       <c r="H9" t="n">
-        <v>58.9</v>
+        <v>42.9</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>4-8</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1357,25 +1345,25 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>80.2</v>
+        <v>29.7</v>
       </c>
       <c r="M9" t="n">
-        <v>58.7</v>
+        <v>11.3</v>
       </c>
       <c r="N9" t="n">
-        <v>64.8</v>
+        <v>44.6</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>오버</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>47.3</v>
+        <v>28.4</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -1395,60 +1383,60 @@
         </is>
       </c>
       <c r="V9" t="n">
-        <v>37.29</v>
+        <v>45.1</v>
       </c>
       <c r="W9" t="n">
         <v>60</v>
       </c>
       <c r="X9" t="n">
-        <v>48.7</v>
+        <v>57.3</v>
       </c>
       <c r="Y9" t="n">
-        <v>51.3</v>
+        <v>42.7</v>
       </c>
       <c r="Z9" t="n">
-        <v>59.7</v>
+        <v>49.6</v>
       </c>
       <c r="AA9" t="n">
-        <v>43.5</v>
+        <v>34.1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>7:35</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>KT Wiz Suwon</t>
+          <t>Toronto Blue Jays</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="F10" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="G10" t="n">
-        <v>55.5</v>
+        <v>56</v>
       </c>
       <c r="H10" t="n">
-        <v>44.5</v>
+        <v>44</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1462,13 +1450,13 @@
         </is>
       </c>
       <c r="L10" t="n">
-        <v>23.3</v>
+        <v>51.8</v>
       </c>
       <c r="M10" t="n">
-        <v>7.9</v>
+        <v>27.1</v>
       </c>
       <c r="N10" t="n">
-        <v>40.1</v>
+        <v>53.2</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1476,7 +1464,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>26.6</v>
+        <v>33.9</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1500,60 +1488,60 @@
         </is>
       </c>
       <c r="V10" t="n">
-        <v>40.16</v>
+        <v>45</v>
       </c>
       <c r="W10" t="n">
         <v>60</v>
       </c>
       <c r="X10" t="n">
-        <v>59.2</v>
+        <v>56</v>
       </c>
       <c r="Y10" t="n">
-        <v>40.8</v>
+        <v>44</v>
       </c>
       <c r="Z10" t="n">
-        <v>45.7</v>
+        <v>53.7</v>
       </c>
       <c r="AA10" t="n">
-        <v>32.9</v>
+        <v>36.1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>8:05</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Lotte Giants</t>
+          <t>Tampa Bay Rays</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F11" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G11" t="n">
-        <v>51.6</v>
+        <v>51.8</v>
       </c>
       <c r="H11" t="n">
-        <v>48.4</v>
+        <v>48.2</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>6-4</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1567,13 +1555,13 @@
         </is>
       </c>
       <c r="L11" t="n">
-        <v>46.3</v>
+        <v>17.4</v>
       </c>
       <c r="M11" t="n">
-        <v>22.6</v>
+        <v>5.1</v>
       </c>
       <c r="N11" t="n">
-        <v>53.7</v>
+        <v>38.3</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1581,7 +1569,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>33.4</v>
+        <v>25</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1605,38 +1593,38 @@
         </is>
       </c>
       <c r="V11" t="n">
-        <v>39.47</v>
+        <v>41.7</v>
       </c>
       <c r="W11" t="n">
         <v>60</v>
       </c>
       <c r="X11" t="n">
-        <v>51.1</v>
+        <v>52.9</v>
       </c>
       <c r="Y11" t="n">
-        <v>48.9</v>
+        <v>47.1</v>
       </c>
       <c r="Z11" t="n">
-        <v>56.1</v>
+        <v>45.2</v>
       </c>
       <c r="AA11" t="n">
-        <v>37</v>
+        <v>31.6</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2:05</t>
+          <t>9:05</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1658,7 +1646,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1672,13 +1660,13 @@
         </is>
       </c>
       <c r="L12" t="n">
-        <v>28.4</v>
+        <v>12.3</v>
       </c>
       <c r="M12" t="n">
-        <v>10.6</v>
+        <v>3.1</v>
       </c>
       <c r="N12" t="n">
-        <v>40.3</v>
+        <v>41.3</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1686,7 +1674,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>21.9</v>
+        <v>28.3</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1710,38 +1698,38 @@
         </is>
       </c>
       <c r="V12" t="n">
-        <v>45.35</v>
+        <v>44.86</v>
       </c>
       <c r="W12" t="n">
         <v>60</v>
       </c>
       <c r="X12" t="n">
-        <v>55.9</v>
+        <v>56</v>
       </c>
       <c r="Y12" t="n">
-        <v>44.1</v>
+        <v>44</v>
       </c>
       <c r="Z12" t="n">
-        <v>44.3</v>
+        <v>50.9</v>
       </c>
       <c r="AA12" t="n">
-        <v>25.7</v>
+        <v>36.6</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>7:40</t>
+          <t>9:40</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies</t>
+          <t>Colorado Rockies</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Arizona Diamondbacks</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1750,20 +1738,20 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F13" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="G13" t="n">
-        <v>43.3</v>
+        <v>43.5</v>
       </c>
       <c r="H13" t="n">
-        <v>56.7</v>
+        <v>56.5</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>4-7</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1777,13 +1765,13 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>51.8</v>
+        <v>74</v>
       </c>
       <c r="M13" t="n">
-        <v>27.1</v>
+        <v>50.4</v>
       </c>
       <c r="N13" t="n">
-        <v>53.3</v>
+        <v>56.2</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1791,7 +1779,7 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>33.5</v>
+        <v>34.5</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1815,547 +1803,22 @@
         </is>
       </c>
       <c r="V13" t="n">
-        <v>41.13</v>
+        <v>42</v>
       </c>
       <c r="W13" t="n">
         <v>60</v>
       </c>
       <c r="X13" t="n">
-        <v>46.9</v>
+        <v>44.4</v>
       </c>
       <c r="Y13" t="n">
-        <v>53.1</v>
+        <v>55.6</v>
       </c>
       <c r="Z13" t="n">
-        <v>53.8</v>
+        <v>50.2</v>
       </c>
       <c r="AA13" t="n">
-        <v>35.7</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>7:45</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Boston Red Sox</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Cleveland Guardians</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>47</v>
-      </c>
-      <c r="F14" t="n">
-        <v>53</v>
-      </c>
-      <c r="G14" t="n">
-        <v>48.9</v>
-      </c>
-      <c r="H14" t="n">
-        <v>51.1</v>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>4-6</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L14" t="n">
-        <v>63.2</v>
-      </c>
-      <c r="M14" t="n">
-        <v>37.9</v>
-      </c>
-      <c r="N14" t="n">
-        <v>51.9</v>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="P14" t="n">
-        <v>34.2</v>
-      </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>언더</t>
-        </is>
-      </c>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>⏭</t>
-        </is>
-      </c>
-      <c r="S14" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="T14" t="inlineStr"/>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>확률·표본·모델합의 기준 미달</t>
-        </is>
-      </c>
-      <c r="V14" t="n">
-        <v>43.29</v>
-      </c>
-      <c r="W14" t="n">
-        <v>60</v>
-      </c>
-      <c r="X14" t="n">
-        <v>51.7</v>
-      </c>
-      <c r="Y14" t="n">
-        <v>48.3</v>
-      </c>
-      <c r="Z14" t="n">
-        <v>48.2</v>
-      </c>
-      <c r="AA14" t="n">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>9:05</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Texas Rangers</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>New York Mets</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>62</v>
-      </c>
-      <c r="F15" t="n">
-        <v>38</v>
-      </c>
-      <c r="G15" t="n">
-        <v>60.6</v>
-      </c>
-      <c r="H15" t="n">
-        <v>39.4</v>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>6-3</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L15" t="n">
-        <v>54.4</v>
-      </c>
-      <c r="M15" t="n">
-        <v>29.4</v>
-      </c>
-      <c r="N15" t="n">
-        <v>53.3</v>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="P15" t="n">
-        <v>36.9</v>
-      </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>언더</t>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>⏭</t>
-        </is>
-      </c>
-      <c r="S15" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="T15" t="inlineStr"/>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>확률·표본·모델합의 기준 미달</t>
-        </is>
-      </c>
-      <c r="V15" t="n">
-        <v>41.33</v>
-      </c>
-      <c r="W15" t="n">
-        <v>60</v>
-      </c>
-      <c r="X15" t="n">
-        <v>58.4</v>
-      </c>
-      <c r="Y15" t="n">
-        <v>41.6</v>
-      </c>
-      <c r="Z15" t="n">
-        <v>52.9</v>
-      </c>
-      <c r="AA15" t="n">
-        <v>39.3</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>9:40</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Colorado Rockies</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Arizona Diamondbacks</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>39</v>
-      </c>
-      <c r="F16" t="n">
-        <v>61</v>
-      </c>
-      <c r="G16" t="n">
-        <v>42.2</v>
-      </c>
-      <c r="H16" t="n">
-        <v>57.8</v>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>4-8</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L16" t="n">
-        <v>80.90000000000001</v>
-      </c>
-      <c r="M16" t="n">
-        <v>59.8</v>
-      </c>
-      <c r="N16" t="n">
-        <v>64</v>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>오버</t>
-        </is>
-      </c>
-      <c r="P16" t="n">
-        <v>45</v>
-      </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>⏭</t>
-        </is>
-      </c>
-      <c r="S16" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="T16" t="inlineStr"/>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>확률·표본·모델합의 기준 미달</t>
-        </is>
-      </c>
-      <c r="V16" t="n">
-        <v>40.3</v>
-      </c>
-      <c r="W16" t="n">
-        <v>60</v>
-      </c>
-      <c r="X16" t="n">
-        <v>46.9</v>
-      </c>
-      <c r="Y16" t="n">
-        <v>53.1</v>
-      </c>
-      <c r="Z16" t="n">
-        <v>58.4</v>
-      </c>
-      <c r="AA16" t="n">
-        <v>40.1</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>10:40</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Athletics</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Los Angeles Angels</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E17" t="n">
-        <v>47</v>
-      </c>
-      <c r="F17" t="n">
-        <v>53</v>
-      </c>
-      <c r="G17" t="n">
-        <v>48.9</v>
-      </c>
-      <c r="H17" t="n">
-        <v>51.1</v>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>6-7</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L17" t="n">
-        <v>85.8</v>
-      </c>
-      <c r="M17" t="n">
-        <v>67.3</v>
-      </c>
-      <c r="N17" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>오버</t>
-        </is>
-      </c>
-      <c r="P17" t="n">
-        <v>48.7</v>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>⏭</t>
-        </is>
-      </c>
-      <c r="S17" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="T17" t="inlineStr"/>
-      <c r="U17" t="inlineStr">
-        <is>
-          <t>확률·표본·모델합의 기준 미달</t>
-        </is>
-      </c>
-      <c r="V17" t="n">
-        <v>43.16</v>
-      </c>
-      <c r="W17" t="n">
-        <v>60</v>
-      </c>
-      <c r="X17" t="n">
-        <v>51.7</v>
-      </c>
-      <c r="Y17" t="n">
-        <v>48.3</v>
-      </c>
-      <c r="Z17" t="n">
-        <v>60.4</v>
-      </c>
-      <c r="AA17" t="n">
-        <v>42.6</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>10:45</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>San Francisco Giants</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Minnesota Twins</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E18" t="n">
-        <v>54</v>
-      </c>
-      <c r="F18" t="n">
-        <v>46</v>
-      </c>
-      <c r="G18" t="n">
-        <v>51.4</v>
-      </c>
-      <c r="H18" t="n">
-        <v>48.6</v>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>5-4</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L18" t="n">
-        <v>51.8</v>
-      </c>
-      <c r="M18" t="n">
-        <v>27.1</v>
-      </c>
-      <c r="N18" t="n">
-        <v>53.3</v>
-      </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="P18" t="n">
-        <v>33.5</v>
-      </c>
-      <c r="Q18" t="inlineStr">
-        <is>
-          <t>언더</t>
-        </is>
-      </c>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>⏭</t>
-        </is>
-      </c>
-      <c r="S18" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="T18" t="inlineStr"/>
-      <c r="U18" t="inlineStr">
-        <is>
-          <t>확률·표본·모델합의 기준 미달</t>
-        </is>
-      </c>
-      <c r="V18" t="n">
-        <v>42.45</v>
-      </c>
-      <c r="W18" t="n">
-        <v>60</v>
-      </c>
-      <c r="X18" t="n">
-        <v>47.5</v>
-      </c>
-      <c r="Y18" t="n">
-        <v>52.5</v>
-      </c>
-      <c r="Z18" t="n">
-        <v>53.8</v>
-      </c>
-      <c r="AA18" t="n">
-        <v>35.7</v>
+        <v>29.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-09-25 15:49
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA13"/>
+  <dimension ref="A1:AA17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -556,17 +556,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -575,25 +575,25 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>23</v>
+        <v>72</v>
       </c>
       <c r="F2" t="n">
-        <v>77</v>
+        <v>28</v>
       </c>
       <c r="G2" t="n">
-        <v>31.3</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="H2" t="n">
-        <v>68.7</v>
+        <v>35.4</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>3-1</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -602,13 +602,13 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>17.4</v>
+        <v>4.5</v>
       </c>
       <c r="M2" t="n">
-        <v>5.1</v>
+        <v>0.8</v>
       </c>
       <c r="N2" t="n">
-        <v>27.9</v>
+        <v>28.1</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>14.1</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -635,7 +635,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>원정승</t>
+          <t>홈승</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -644,60 +644,60 @@
         </is>
       </c>
       <c r="V2" t="n">
-        <v>16.48</v>
+        <v>33.05</v>
       </c>
       <c r="W2" t="n">
         <v>60</v>
       </c>
       <c r="X2" t="n">
-        <v>43.8</v>
+        <v>53.4</v>
       </c>
       <c r="Y2" t="n">
-        <v>56.2</v>
+        <v>46.6</v>
       </c>
       <c r="Z2" t="n">
-        <v>31.5</v>
+        <v>36</v>
       </c>
       <c r="AA2" t="n">
-        <v>17.1</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>8:05</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="F3" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="G3" t="n">
-        <v>65.09999999999999</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="H3" t="n">
-        <v>34.9</v>
+        <v>31.1</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>7-2</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -711,27 +711,27 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>27.1</v>
+        <v>53.1</v>
       </c>
       <c r="M3" t="n">
-        <v>9.9</v>
+        <v>28.2</v>
       </c>
       <c r="N3" t="n">
-        <v>33.2</v>
+        <v>52.7</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P3" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
           <t>언더</t>
         </is>
       </c>
-      <c r="P3" t="n">
-        <v>16.7</v>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>언더</t>
-        </is>
-      </c>
       <c r="R3" t="inlineStr">
         <is>
           <t>★★</t>
@@ -753,60 +753,60 @@
         </is>
       </c>
       <c r="V3" t="n">
-        <v>31.41</v>
+        <v>32.77</v>
       </c>
       <c r="W3" t="n">
         <v>60</v>
       </c>
       <c r="X3" t="n">
-        <v>53.2</v>
+        <v>58.3</v>
       </c>
       <c r="Y3" t="n">
-        <v>46.8</v>
+        <v>41.7</v>
       </c>
       <c r="Z3" t="n">
-        <v>35.2</v>
+        <v>52.6</v>
       </c>
       <c r="AA3" t="n">
-        <v>19</v>
+        <v>32.5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>8:40</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>Colorado Rockies</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="F4" t="n">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="G4" t="n">
-        <v>58.7</v>
+        <v>64</v>
       </c>
       <c r="H4" t="n">
-        <v>41.3</v>
+        <v>36</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>6-3</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -820,103 +820,107 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>35.2</v>
+        <v>54.4</v>
       </c>
       <c r="M4" t="n">
-        <v>14.6</v>
+        <v>29.4</v>
       </c>
       <c r="N4" t="n">
-        <v>34.5</v>
+        <v>55.4</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P4" t="n">
+        <v>34.7</v>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
           <t>언더</t>
         </is>
       </c>
-      <c r="P4" t="n">
-        <v>21.2</v>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>언더</t>
-        </is>
-      </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>⏭</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr"/>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>확률·표본·모델합의 기준 미달</t>
+          <t>Forebet·과거모델 합의</t>
         </is>
       </c>
       <c r="V4" t="n">
-        <v>41.5</v>
+        <v>43.4</v>
       </c>
       <c r="W4" t="n">
         <v>60</v>
       </c>
       <c r="X4" t="n">
-        <v>59.8</v>
+        <v>56.4</v>
       </c>
       <c r="Y4" t="n">
-        <v>40.2</v>
+        <v>43.6</v>
       </c>
       <c r="Z4" t="n">
-        <v>34.2</v>
+        <v>55.7</v>
       </c>
       <c r="AA4" t="n">
-        <v>23.4</v>
+        <v>36.5</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>11:10</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Chiba Lotte Marines</t>
+          <t>Seattle Mariners</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>Los Angeles Angels</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>48</v>
+        <v>66</v>
       </c>
       <c r="F5" t="n">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="G5" t="n">
-        <v>51</v>
+        <v>62.9</v>
       </c>
       <c r="H5" t="n">
-        <v>49</v>
+        <v>37.1</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -925,94 +929,98 @@
         </is>
       </c>
       <c r="L5" t="n">
-        <v>18.5</v>
+        <v>40.7</v>
       </c>
       <c r="M5" t="n">
-        <v>5.6</v>
+        <v>18.4</v>
       </c>
       <c r="N5" t="n">
-        <v>29.1</v>
+        <v>55.8</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P5" t="n">
+        <v>33.2</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
           <t>언더</t>
         </is>
       </c>
-      <c r="P5" t="n">
-        <v>15.2</v>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>언더</t>
-        </is>
-      </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>⏭</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr"/>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>확률·표본·모델합의 기준 미달</t>
+          <t>Forebet·과거모델 합의</t>
         </is>
       </c>
       <c r="V5" t="n">
-        <v>41.49</v>
+        <v>42.81</v>
       </c>
       <c r="W5" t="n">
         <v>60</v>
       </c>
       <c r="X5" t="n">
-        <v>55.5</v>
+        <v>58.3</v>
       </c>
       <c r="Y5" t="n">
-        <v>44.5</v>
+        <v>41.7</v>
       </c>
       <c r="Z5" t="n">
-        <v>32.6</v>
+        <v>60.9</v>
       </c>
       <c r="AA5" t="n">
-        <v>18.4</v>
+        <v>38.1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>Fukuoka S. Hawks</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="F6" t="n">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="G6" t="n">
-        <v>42.5</v>
+        <v>38.8</v>
       </c>
       <c r="H6" t="n">
-        <v>57.5</v>
+        <v>61.2</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -1030,21 +1038,21 @@
         </is>
       </c>
       <c r="L6" t="n">
-        <v>29.7</v>
+        <v>28.4</v>
       </c>
       <c r="M6" t="n">
-        <v>11.3</v>
+        <v>10.6</v>
       </c>
       <c r="N6" t="n">
-        <v>43</v>
+        <v>33.6</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>26.6</v>
+        <v>17.7</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1068,65 +1076,65 @@
         </is>
       </c>
       <c r="V6" t="n">
-        <v>41.42</v>
+        <v>36.95</v>
       </c>
       <c r="W6" t="n">
         <v>60</v>
       </c>
       <c r="X6" t="n">
-        <v>43.2</v>
+        <v>44.5</v>
       </c>
       <c r="Y6" t="n">
-        <v>56.8</v>
+        <v>55.5</v>
       </c>
       <c r="Z6" t="n">
-        <v>47.5</v>
+        <v>35.3</v>
       </c>
       <c r="AA6" t="n">
-        <v>31.7</v>
+        <v>20.1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>KT Wiz Suwon</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>54</v>
+        <v>39</v>
       </c>
       <c r="F7" t="n">
-        <v>46</v>
+        <v>61</v>
       </c>
       <c r="G7" t="n">
-        <v>55.5</v>
+        <v>42.6</v>
       </c>
       <c r="H7" t="n">
-        <v>44.5</v>
+        <v>57.4</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>2-4</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -1135,25 +1143,25 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>58.3</v>
+        <v>17.4</v>
       </c>
       <c r="M7" t="n">
-        <v>33</v>
+        <v>5.1</v>
       </c>
       <c r="N7" t="n">
-        <v>58.8</v>
+        <v>28</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>43.6</v>
+        <v>14.1</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1173,65 +1181,65 @@
         </is>
       </c>
       <c r="V7" t="n">
-        <v>40.75</v>
+        <v>39.37</v>
       </c>
       <c r="W7" t="n">
         <v>60</v>
       </c>
       <c r="X7" t="n">
-        <v>57.8</v>
+        <v>48</v>
       </c>
       <c r="Y7" t="n">
-        <v>42.2</v>
+        <v>52</v>
       </c>
       <c r="Z7" t="n">
-        <v>58.9</v>
+        <v>31.5</v>
       </c>
       <c r="AA7" t="n">
-        <v>47.2</v>
+        <v>17.1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Lotte Giants</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="F8" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="G8" t="n">
-        <v>51.8</v>
+        <v>51</v>
       </c>
       <c r="H8" t="n">
-        <v>48.2</v>
+        <v>49</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>2-4</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1240,21 +1248,21 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>35.2</v>
+        <v>17.4</v>
       </c>
       <c r="M8" t="n">
-        <v>14.6</v>
+        <v>5.1</v>
       </c>
       <c r="N8" t="n">
-        <v>44.4</v>
+        <v>28</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>30</v>
+        <v>14.1</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1278,65 +1286,65 @@
         </is>
       </c>
       <c r="V8" t="n">
-        <v>40.33</v>
+        <v>40.92</v>
       </c>
       <c r="W8" t="n">
         <v>60</v>
       </c>
       <c r="X8" t="n">
-        <v>51.6</v>
+        <v>54.1</v>
       </c>
       <c r="Y8" t="n">
-        <v>48.4</v>
+        <v>45.9</v>
       </c>
       <c r="Z8" t="n">
-        <v>47.5</v>
+        <v>31.5</v>
       </c>
       <c r="AA8" t="n">
-        <v>35.1</v>
+        <v>17.1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>4:45</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>San Francisco Giants</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="F9" t="n">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="G9" t="n">
-        <v>57.1</v>
+        <v>49.6</v>
       </c>
       <c r="H9" t="n">
-        <v>42.9</v>
+        <v>50.4</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1345,21 +1353,21 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>29.7</v>
+        <v>23.3</v>
       </c>
       <c r="M9" t="n">
-        <v>11.3</v>
+        <v>7.9</v>
       </c>
       <c r="N9" t="n">
-        <v>44.6</v>
+        <v>30.3</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>28.4</v>
+        <v>15.5</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1383,65 +1391,65 @@
         </is>
       </c>
       <c r="V9" t="n">
-        <v>45.1</v>
+        <v>40.95</v>
       </c>
       <c r="W9" t="n">
         <v>60</v>
       </c>
       <c r="X9" t="n">
-        <v>57.3</v>
+        <v>56.5</v>
       </c>
       <c r="Y9" t="n">
-        <v>42.7</v>
+        <v>43.5</v>
       </c>
       <c r="Z9" t="n">
-        <v>49.6</v>
+        <v>32.6</v>
       </c>
       <c r="AA9" t="n">
-        <v>34.1</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>7:35</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Toronto Blue Jays</t>
+          <t>Samsung Lions</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>56</v>
+        <v>33</v>
       </c>
       <c r="F10" t="n">
-        <v>44</v>
+        <v>67</v>
       </c>
       <c r="G10" t="n">
-        <v>56</v>
+        <v>38.1</v>
       </c>
       <c r="H10" t="n">
-        <v>44</v>
+        <v>61.9</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>3-6</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1450,13 +1458,13 @@
         </is>
       </c>
       <c r="L10" t="n">
-        <v>51.8</v>
+        <v>55.7</v>
       </c>
       <c r="M10" t="n">
-        <v>27.1</v>
+        <v>30.6</v>
       </c>
       <c r="N10" t="n">
-        <v>53.2</v>
+        <v>59.4</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1464,11 +1472,11 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>33.9</v>
+        <v>41.9</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>언더</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -1488,60 +1496,60 @@
         </is>
       </c>
       <c r="V10" t="n">
-        <v>45</v>
+        <v>34.36</v>
       </c>
       <c r="W10" t="n">
         <v>60</v>
       </c>
       <c r="X10" t="n">
-        <v>56</v>
+        <v>45.9</v>
       </c>
       <c r="Y10" t="n">
-        <v>44</v>
+        <v>54.1</v>
       </c>
       <c r="Z10" t="n">
-        <v>53.7</v>
+        <v>60.6</v>
       </c>
       <c r="AA10" t="n">
-        <v>36.1</v>
+        <v>45.7</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>8:05</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>Lotte Giants</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F11" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G11" t="n">
-        <v>51.8</v>
+        <v>55.2</v>
       </c>
       <c r="H11" t="n">
-        <v>48.2</v>
+        <v>44.8</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1555,13 +1563,13 @@
         </is>
       </c>
       <c r="L11" t="n">
-        <v>17.4</v>
+        <v>54.4</v>
       </c>
       <c r="M11" t="n">
-        <v>5.1</v>
+        <v>29.4</v>
       </c>
       <c r="N11" t="n">
-        <v>38.3</v>
+        <v>58</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1569,11 +1577,11 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>25</v>
+        <v>41.7</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>언더</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -1593,33 +1601,33 @@
         </is>
       </c>
       <c r="V11" t="n">
-        <v>41.7</v>
+        <v>40.15</v>
       </c>
       <c r="W11" t="n">
         <v>60</v>
       </c>
       <c r="X11" t="n">
-        <v>52.9</v>
+        <v>58.4</v>
       </c>
       <c r="Y11" t="n">
-        <v>47.1</v>
+        <v>41.6</v>
       </c>
       <c r="Z11" t="n">
-        <v>45.2</v>
+        <v>59.2</v>
       </c>
       <c r="AA11" t="n">
-        <v>31.6</v>
+        <v>45.8</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>9:05</t>
+          <t>7:45</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>Washington Nationals</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1633,25 +1641,25 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="F12" t="n">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="G12" t="n">
-        <v>56</v>
+        <v>51.8</v>
       </c>
       <c r="H12" t="n">
-        <v>44</v>
+        <v>48.2</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>5-6</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1660,13 +1668,13 @@
         </is>
       </c>
       <c r="L12" t="n">
-        <v>12.3</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="M12" t="n">
-        <v>3.1</v>
+        <v>49.2</v>
       </c>
       <c r="N12" t="n">
-        <v>41.3</v>
+        <v>53.4</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1674,7 +1682,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>28.3</v>
+        <v>33.7</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1698,38 +1706,38 @@
         </is>
       </c>
       <c r="V12" t="n">
-        <v>44.86</v>
+        <v>42.7</v>
       </c>
       <c r="W12" t="n">
         <v>60</v>
       </c>
       <c r="X12" t="n">
-        <v>56</v>
+        <v>57.5</v>
       </c>
       <c r="Y12" t="n">
-        <v>44</v>
+        <v>42.5</v>
       </c>
       <c r="Z12" t="n">
-        <v>50.9</v>
+        <v>46.8</v>
       </c>
       <c r="AA12" t="n">
-        <v>36.6</v>
+        <v>28.6</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>9:40</t>
+          <t>8:10</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Colorado Rockies</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Arizona Diamondbacks</t>
+          <t>Atlanta Braves</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1738,20 +1746,20 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F13" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G13" t="n">
-        <v>43.5</v>
+        <v>42.8</v>
       </c>
       <c r="H13" t="n">
-        <v>56.5</v>
+        <v>57.2</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>4-7</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1765,13 +1773,13 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>74</v>
+        <v>42.1</v>
       </c>
       <c r="M13" t="n">
-        <v>50.4</v>
+        <v>19.4</v>
       </c>
       <c r="N13" t="n">
-        <v>56.2</v>
+        <v>57.7</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1779,7 +1787,7 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>34.5</v>
+        <v>34.6</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1803,22 +1811,442 @@
         </is>
       </c>
       <c r="V13" t="n">
-        <v>42</v>
+        <v>41.9</v>
       </c>
       <c r="W13" t="n">
         <v>60</v>
       </c>
       <c r="X13" t="n">
-        <v>44.4</v>
+        <v>44</v>
       </c>
       <c r="Y13" t="n">
-        <v>55.6</v>
+        <v>56</v>
       </c>
       <c r="Z13" t="n">
-        <v>50.2</v>
+        <v>62.9</v>
       </c>
       <c r="AA13" t="n">
-        <v>29.2</v>
+        <v>39.6</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>9:10</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Minnesota Twins</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Texas Rangers</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>44</v>
+      </c>
+      <c r="F14" t="n">
+        <v>56</v>
+      </c>
+      <c r="G14" t="n">
+        <v>43.8</v>
+      </c>
+      <c r="H14" t="n">
+        <v>56.2</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>4-5</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L14" t="n">
+        <v>51.8</v>
+      </c>
+      <c r="M14" t="n">
+        <v>27.1</v>
+      </c>
+      <c r="N14" t="n">
+        <v>52.4</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P14" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>언더</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V14" t="n">
+        <v>42.48</v>
+      </c>
+      <c r="W14" t="n">
+        <v>60</v>
+      </c>
+      <c r="X14" t="n">
+        <v>43.4</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>56.6</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>32.8</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>San Diego Padres</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>59</v>
+      </c>
+      <c r="F15" t="n">
+        <v>41</v>
+      </c>
+      <c r="G15" t="n">
+        <v>57.8</v>
+      </c>
+      <c r="H15" t="n">
+        <v>42.2</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>6-4</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L15" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="M15" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="N15" t="n">
+        <v>52</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P15" t="n">
+        <v>33.4</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>언더</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V15" t="n">
+        <v>42.83</v>
+      </c>
+      <c r="W15" t="n">
+        <v>60</v>
+      </c>
+      <c r="X15" t="n">
+        <v>56</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>44</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>37.7</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>10:40</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Athletics</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Houston Astros</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>42</v>
+      </c>
+      <c r="F16" t="n">
+        <v>58</v>
+      </c>
+      <c r="G16" t="n">
+        <v>42.8</v>
+      </c>
+      <c r="H16" t="n">
+        <v>57.2</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>5-7</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L16" t="n">
+        <v>80.2</v>
+      </c>
+      <c r="M16" t="n">
+        <v>58.7</v>
+      </c>
+      <c r="N16" t="n">
+        <v>62.8</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>오버</t>
+        </is>
+      </c>
+      <c r="P16" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V16" t="n">
+        <v>41.79</v>
+      </c>
+      <c r="W16" t="n">
+        <v>60</v>
+      </c>
+      <c r="X16" t="n">
+        <v>44</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>56</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>57.1</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>San Francisco Giants</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Los Angeles Dodgers</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>54</v>
+      </c>
+      <c r="F17" t="n">
+        <v>46</v>
+      </c>
+      <c r="G17" t="n">
+        <v>51.3</v>
+      </c>
+      <c r="H17" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L17" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="M17" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="N17" t="n">
+        <v>40.2</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P17" t="n">
+        <v>26.8</v>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>언더</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr"/>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V17" t="n">
+        <v>43.75</v>
+      </c>
+      <c r="W17" t="n">
+        <v>60</v>
+      </c>
+      <c r="X17" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>52.7</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>33.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-09-26 17:51
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA17"/>
+  <dimension ref="A1:AA15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -556,44 +556,44 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Seibu Lions</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Chiba Lotte Marines</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F2" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G2" t="n">
-        <v>64.59999999999999</v>
+        <v>66.2</v>
       </c>
       <c r="H2" t="n">
-        <v>35.4</v>
+        <v>33.8</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>3-1</t>
+          <t>5-2</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -602,27 +602,27 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>4.5</v>
+        <v>31.1</v>
       </c>
       <c r="M2" t="n">
-        <v>0.8</v>
+        <v>12.1</v>
       </c>
       <c r="N2" t="n">
-        <v>28.1</v>
+        <v>42.2</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P2" t="n">
+        <v>26.8</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
           <t>언더</t>
         </is>
       </c>
-      <c r="P2" t="n">
-        <v>9.199999999999999</v>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>언더</t>
-        </is>
-      </c>
       <c r="R2" t="inlineStr">
         <is>
           <t>★★</t>
@@ -644,38 +644,38 @@
         </is>
       </c>
       <c r="V2" t="n">
-        <v>33.05</v>
+        <v>30.15</v>
       </c>
       <c r="W2" t="n">
         <v>60</v>
       </c>
       <c r="X2" t="n">
-        <v>53.4</v>
+        <v>60.5</v>
       </c>
       <c r="Y2" t="n">
-        <v>46.6</v>
+        <v>39.5</v>
       </c>
       <c r="Z2" t="n">
-        <v>36</v>
+        <v>45.8</v>
       </c>
       <c r="AA2" t="n">
-        <v>12.1</v>
+        <v>31.8</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>8:05</t>
+          <t>8:10</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Baltimore Orioles</t>
+          <t>St.Louis Cardinals</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -684,20 +684,20 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="F3" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G3" t="n">
-        <v>68.90000000000001</v>
+        <v>64</v>
       </c>
       <c r="H3" t="n">
-        <v>31.1</v>
+        <v>36</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>7-2</t>
+          <t>5-2</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -711,13 +711,13 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>53.1</v>
+        <v>29.7</v>
       </c>
       <c r="M3" t="n">
-        <v>28.2</v>
+        <v>11.3</v>
       </c>
       <c r="N3" t="n">
-        <v>52.7</v>
+        <v>44.5</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>31.4</v>
+        <v>28.6</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -753,28 +753,28 @@
         </is>
       </c>
       <c r="V3" t="n">
-        <v>32.77</v>
+        <v>41.91</v>
       </c>
       <c r="W3" t="n">
         <v>60</v>
       </c>
       <c r="X3" t="n">
-        <v>58.3</v>
+        <v>54.9</v>
       </c>
       <c r="Y3" t="n">
-        <v>41.7</v>
+        <v>45.1</v>
       </c>
       <c r="Z3" t="n">
-        <v>52.6</v>
+        <v>49.5</v>
       </c>
       <c r="AA3" t="n">
-        <v>32.5</v>
+        <v>34.3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>8:40</t>
+          <t>8:10</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -793,10 +793,10 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F4" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G4" t="n">
         <v>64</v>
@@ -826,7 +826,7 @@
         <v>29.4</v>
       </c>
       <c r="N4" t="n">
-        <v>55.4</v>
+        <v>52.4</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -834,7 +834,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>34.7</v>
+        <v>33.9</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -862,28 +862,28 @@
         </is>
       </c>
       <c r="V4" t="n">
-        <v>43.4</v>
+        <v>41.91</v>
       </c>
       <c r="W4" t="n">
         <v>60</v>
       </c>
       <c r="X4" t="n">
-        <v>56.4</v>
+        <v>54.9</v>
       </c>
       <c r="Y4" t="n">
-        <v>43.6</v>
+        <v>45.1</v>
       </c>
       <c r="Z4" t="n">
-        <v>55.7</v>
+        <v>51.7</v>
       </c>
       <c r="AA4" t="n">
-        <v>36.5</v>
+        <v>35.3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>11:10</t>
+          <t>10:40</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -908,14 +908,14 @@
         <v>34</v>
       </c>
       <c r="G5" t="n">
-        <v>62.9</v>
+        <v>63</v>
       </c>
       <c r="H5" t="n">
-        <v>37.1</v>
+        <v>37</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>5-3</t>
+          <t>6-3</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -929,13 +929,13 @@
         </is>
       </c>
       <c r="L5" t="n">
-        <v>40.7</v>
+        <v>53.1</v>
       </c>
       <c r="M5" t="n">
-        <v>18.4</v>
+        <v>28.2</v>
       </c>
       <c r="N5" t="n">
-        <v>55.8</v>
+        <v>52.8</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -943,7 +943,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>33.2</v>
+        <v>32.3</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -971,22 +971,22 @@
         </is>
       </c>
       <c r="V5" t="n">
-        <v>42.81</v>
+        <v>42.89</v>
       </c>
       <c r="W5" t="n">
         <v>60</v>
       </c>
       <c r="X5" t="n">
-        <v>58.3</v>
+        <v>58.4</v>
       </c>
       <c r="Y5" t="n">
-        <v>41.7</v>
+        <v>41.6</v>
       </c>
       <c r="Z5" t="n">
-        <v>60.9</v>
+        <v>52.7</v>
       </c>
       <c r="AA5" t="n">
-        <v>38.1</v>
+        <v>33.7</v>
       </c>
     </row>
     <row r="6">
@@ -997,12 +997,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Orix Buffaloes</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Fukuoka S. Hawks</t>
+          <t>Chunichi Dragons</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1011,25 +1011,25 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="F6" t="n">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="G6" t="n">
-        <v>38.8</v>
+        <v>50.2</v>
       </c>
       <c r="H6" t="n">
-        <v>61.2</v>
+        <v>49.8</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -1044,7 +1044,7 @@
         <v>10.6</v>
       </c>
       <c r="N6" t="n">
-        <v>33.6</v>
+        <v>33.9</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1052,7 +1052,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>17.7</v>
+        <v>17.6</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1076,60 +1076,60 @@
         </is>
       </c>
       <c r="V6" t="n">
-        <v>36.95</v>
+        <v>40.96</v>
       </c>
       <c r="W6" t="n">
         <v>60</v>
       </c>
       <c r="X6" t="n">
-        <v>44.5</v>
+        <v>49.1</v>
       </c>
       <c r="Y6" t="n">
-        <v>55.5</v>
+        <v>50.9</v>
       </c>
       <c r="Z6" t="n">
-        <v>35.3</v>
+        <v>35.7</v>
       </c>
       <c r="AA6" t="n">
-        <v>20.1</v>
+        <v>19.9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="F7" t="n">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="G7" t="n">
-        <v>42.6</v>
+        <v>46.9</v>
       </c>
       <c r="H7" t="n">
-        <v>57.4</v>
+        <v>53.1</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1143,25 +1143,25 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>17.4</v>
+        <v>57</v>
       </c>
       <c r="M7" t="n">
-        <v>5.1</v>
+        <v>31.8</v>
       </c>
       <c r="N7" t="n">
-        <v>28</v>
+        <v>59</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>언더</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>14.1</v>
+        <v>43.2</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>언더</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1181,65 +1181,65 @@
         </is>
       </c>
       <c r="V7" t="n">
-        <v>39.37</v>
+        <v>39.46</v>
       </c>
       <c r="W7" t="n">
         <v>60</v>
       </c>
       <c r="X7" t="n">
-        <v>48</v>
+        <v>43.9</v>
       </c>
       <c r="Y7" t="n">
-        <v>52</v>
+        <v>56.1</v>
       </c>
       <c r="Z7" t="n">
-        <v>31.5</v>
+        <v>59.7</v>
       </c>
       <c r="AA7" t="n">
-        <v>17.1</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="F8" t="n">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="G8" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H8" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1248,25 +1248,25 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>17.4</v>
+        <v>57</v>
       </c>
       <c r="M8" t="n">
-        <v>5.1</v>
+        <v>31.8</v>
       </c>
       <c r="N8" t="n">
-        <v>28</v>
+        <v>59</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>언더</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>14.1</v>
+        <v>43.2</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>언더</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -1286,65 +1286,65 @@
         </is>
       </c>
       <c r="V8" t="n">
-        <v>40.92</v>
+        <v>39.67</v>
       </c>
       <c r="W8" t="n">
         <v>60</v>
       </c>
       <c r="X8" t="n">
-        <v>54.1</v>
+        <v>52</v>
       </c>
       <c r="Y8" t="n">
-        <v>45.9</v>
+        <v>48</v>
       </c>
       <c r="Z8" t="n">
-        <v>31.5</v>
+        <v>59.7</v>
       </c>
       <c r="AA8" t="n">
-        <v>17.1</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>5:05</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>Washington Nationals</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Yomiuri Giants</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="F9" t="n">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="G9" t="n">
-        <v>49.6</v>
+        <v>56</v>
       </c>
       <c r="H9" t="n">
-        <v>50.4</v>
+        <v>44</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>6-4</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1353,21 +1353,21 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>23.3</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="M9" t="n">
-        <v>7.9</v>
+        <v>40.4</v>
       </c>
       <c r="N9" t="n">
-        <v>30.3</v>
+        <v>52</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>언더</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>15.5</v>
+        <v>33.7</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1391,60 +1391,60 @@
         </is>
       </c>
       <c r="V9" t="n">
-        <v>40.95</v>
+        <v>44.72</v>
       </c>
       <c r="W9" t="n">
         <v>60</v>
       </c>
       <c r="X9" t="n">
-        <v>56.5</v>
+        <v>54.4</v>
       </c>
       <c r="Y9" t="n">
-        <v>43.5</v>
+        <v>45.6</v>
       </c>
       <c r="Z9" t="n">
-        <v>32.6</v>
+        <v>47.4</v>
       </c>
       <c r="AA9" t="n">
-        <v>18</v>
+        <v>31.5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>5:05</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>SSG Landers</t>
+          <t>San Francisco Giants</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>Los Angeles Dodgers</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="F10" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="G10" t="n">
-        <v>38.1</v>
+        <v>47.3</v>
       </c>
       <c r="H10" t="n">
-        <v>61.9</v>
+        <v>52.7</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>3-6</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1458,13 +1458,13 @@
         </is>
       </c>
       <c r="L10" t="n">
-        <v>55.7</v>
+        <v>18.5</v>
       </c>
       <c r="M10" t="n">
-        <v>30.6</v>
+        <v>5.6</v>
       </c>
       <c r="N10" t="n">
-        <v>59.4</v>
+        <v>39.3</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1472,11 +1472,11 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>41.9</v>
+        <v>23.9</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -1496,60 +1496,60 @@
         </is>
       </c>
       <c r="V10" t="n">
-        <v>34.36</v>
+        <v>43.56</v>
       </c>
       <c r="W10" t="n">
         <v>60</v>
       </c>
       <c r="X10" t="n">
-        <v>45.9</v>
+        <v>50.8</v>
       </c>
       <c r="Y10" t="n">
-        <v>54.1</v>
+        <v>49.2</v>
       </c>
       <c r="Z10" t="n">
-        <v>60.6</v>
+        <v>46.2</v>
       </c>
       <c r="AA10" t="n">
-        <v>45.7</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>5:10</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Lotte Giants</t>
+          <t>Atlanta Braves</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F11" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G11" t="n">
-        <v>55.2</v>
+        <v>50.5</v>
       </c>
       <c r="H11" t="n">
-        <v>44.8</v>
+        <v>49.5</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1563,13 +1563,13 @@
         </is>
       </c>
       <c r="L11" t="n">
-        <v>54.4</v>
+        <v>19.7</v>
       </c>
       <c r="M11" t="n">
-        <v>29.4</v>
+        <v>6.1</v>
       </c>
       <c r="N11" t="n">
-        <v>58</v>
+        <v>38.5</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1577,11 +1577,11 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>41.7</v>
+        <v>25.9</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -1601,38 +1601,38 @@
         </is>
       </c>
       <c r="V11" t="n">
-        <v>40.15</v>
+        <v>42.9</v>
       </c>
       <c r="W11" t="n">
         <v>60</v>
       </c>
       <c r="X11" t="n">
-        <v>58.4</v>
+        <v>48.1</v>
       </c>
       <c r="Y11" t="n">
-        <v>41.6</v>
+        <v>51.9</v>
       </c>
       <c r="Z11" t="n">
-        <v>59.2</v>
+        <v>44.7</v>
       </c>
       <c r="AA11" t="n">
-        <v>45.8</v>
+        <v>32.5</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>7:45</t>
+          <t>5:10</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Washington Nationals</t>
+          <t>Minnesota Twins</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>Texas Rangers</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1641,20 +1641,20 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F12" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G12" t="n">
-        <v>51.8</v>
+        <v>50.5</v>
       </c>
       <c r="H12" t="n">
-        <v>48.2</v>
+        <v>49.5</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>5-6</t>
+          <t>4-6</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1668,13 +1668,13 @@
         </is>
       </c>
       <c r="L12" t="n">
-        <v>73.09999999999999</v>
+        <v>39.3</v>
       </c>
       <c r="M12" t="n">
-        <v>49.2</v>
+        <v>17.4</v>
       </c>
       <c r="N12" t="n">
-        <v>53.4</v>
+        <v>49.5</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1682,7 +1682,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>33.7</v>
+        <v>32.3</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1706,38 +1706,38 @@
         </is>
       </c>
       <c r="V12" t="n">
-        <v>42.7</v>
+        <v>42.24</v>
       </c>
       <c r="W12" t="n">
         <v>60</v>
       </c>
       <c r="X12" t="n">
-        <v>57.5</v>
+        <v>52.7</v>
       </c>
       <c r="Y12" t="n">
-        <v>42.5</v>
+        <v>47.3</v>
       </c>
       <c r="Z12" t="n">
-        <v>46.8</v>
+        <v>52.9</v>
       </c>
       <c r="AA12" t="n">
-        <v>28.6</v>
+        <v>37.3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>8:15</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>Philadelphia Phillies</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Atlanta Braves</t>
+          <t>Tampa Bay Rays</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1746,20 +1746,20 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="F13" t="n">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="G13" t="n">
-        <v>42.8</v>
+        <v>47.8</v>
       </c>
       <c r="H13" t="n">
-        <v>57.2</v>
+        <v>52.2</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>3-5</t>
+          <t>2-3</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1773,13 +1773,13 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>42.1</v>
+        <v>11.4</v>
       </c>
       <c r="M13" t="n">
-        <v>19.4</v>
+        <v>2.8</v>
       </c>
       <c r="N13" t="n">
-        <v>57.7</v>
+        <v>42.6</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1787,7 +1787,7 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>34.6</v>
+        <v>29.1</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1811,38 +1811,38 @@
         </is>
       </c>
       <c r="V13" t="n">
-        <v>41.9</v>
+        <v>42.7</v>
       </c>
       <c r="W13" t="n">
         <v>60</v>
       </c>
       <c r="X13" t="n">
-        <v>44</v>
+        <v>50.6</v>
       </c>
       <c r="Y13" t="n">
-        <v>56</v>
+        <v>49.4</v>
       </c>
       <c r="Z13" t="n">
-        <v>62.9</v>
+        <v>53</v>
       </c>
       <c r="AA13" t="n">
-        <v>39.6</v>
+        <v>37.8</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>9:10</t>
+          <t>9:40</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>Arizona Diamondbacks</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1851,25 +1851,25 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="F14" t="n">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="G14" t="n">
-        <v>43.8</v>
+        <v>51</v>
       </c>
       <c r="H14" t="n">
-        <v>56.2</v>
+        <v>49</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>6-4</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1878,13 +1878,13 @@
         </is>
       </c>
       <c r="L14" t="n">
-        <v>51.8</v>
+        <v>43.5</v>
       </c>
       <c r="M14" t="n">
-        <v>27.1</v>
+        <v>20.4</v>
       </c>
       <c r="N14" t="n">
-        <v>52.4</v>
+        <v>49.8</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1892,7 +1892,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>31.4</v>
+        <v>29.5</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1916,22 +1916,22 @@
         </is>
       </c>
       <c r="V14" t="n">
-        <v>42.48</v>
+        <v>42.01</v>
       </c>
       <c r="W14" t="n">
         <v>60</v>
       </c>
       <c r="X14" t="n">
-        <v>43.4</v>
+        <v>46.6</v>
       </c>
       <c r="Y14" t="n">
-        <v>56.6</v>
+        <v>53.4</v>
       </c>
       <c r="Z14" t="n">
-        <v>52.6</v>
+        <v>52</v>
       </c>
       <c r="AA14" t="n">
-        <v>32.8</v>
+        <v>32.6</v>
       </c>
     </row>
     <row r="15">
@@ -1942,12 +1942,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Athletics</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Arizona Diamondbacks</t>
+          <t>Houston Astros</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1956,20 +1956,20 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="F15" t="n">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="G15" t="n">
-        <v>57.8</v>
+        <v>52.1</v>
       </c>
       <c r="H15" t="n">
-        <v>42.2</v>
+        <v>47.9</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>6-4</t>
+          <t>7-5</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1983,25 +1983,25 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>43.5</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="M15" t="n">
-        <v>20.4</v>
+        <v>59.8</v>
       </c>
       <c r="N15" t="n">
-        <v>52</v>
+        <v>63.5</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>오버</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>33.4</v>
+        <v>44.6</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>언더</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -2021,232 +2021,22 @@
         </is>
       </c>
       <c r="V15" t="n">
-        <v>42.83</v>
+        <v>41.44</v>
       </c>
       <c r="W15" t="n">
         <v>60</v>
       </c>
       <c r="X15" t="n">
-        <v>56</v>
+        <v>53.8</v>
       </c>
       <c r="Y15" t="n">
-        <v>44</v>
+        <v>46.2</v>
       </c>
       <c r="Z15" t="n">
-        <v>54.9</v>
+        <v>57.7</v>
       </c>
       <c r="AA15" t="n">
-        <v>37.7</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>10:40</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Athletics</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Houston Astros</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>42</v>
-      </c>
-      <c r="F16" t="n">
-        <v>58</v>
-      </c>
-      <c r="G16" t="n">
-        <v>42.8</v>
-      </c>
-      <c r="H16" t="n">
-        <v>57.2</v>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>5-7</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L16" t="n">
-        <v>80.2</v>
-      </c>
-      <c r="M16" t="n">
-        <v>58.7</v>
-      </c>
-      <c r="N16" t="n">
-        <v>62.8</v>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>오버</t>
-        </is>
-      </c>
-      <c r="P16" t="n">
-        <v>43.9</v>
-      </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>⏭</t>
-        </is>
-      </c>
-      <c r="S16" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="T16" t="inlineStr"/>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>확률·표본·모델합의 기준 미달</t>
-        </is>
-      </c>
-      <c r="V16" t="n">
-        <v>41.79</v>
-      </c>
-      <c r="W16" t="n">
-        <v>60</v>
-      </c>
-      <c r="X16" t="n">
-        <v>44</v>
-      </c>
-      <c r="Y16" t="n">
-        <v>56</v>
-      </c>
-      <c r="Z16" t="n">
-        <v>57.1</v>
-      </c>
-      <c r="AA16" t="n">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>11:15</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>San Francisco Giants</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Los Angeles Dodgers</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="E17" t="n">
-        <v>54</v>
-      </c>
-      <c r="F17" t="n">
-        <v>46</v>
-      </c>
-      <c r="G17" t="n">
-        <v>51.3</v>
-      </c>
-      <c r="H17" t="n">
-        <v>48.7</v>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>4-3</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L17" t="n">
-        <v>19.7</v>
-      </c>
-      <c r="M17" t="n">
-        <v>6.1</v>
-      </c>
-      <c r="N17" t="n">
-        <v>40.2</v>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="P17" t="n">
-        <v>26.8</v>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>언더</t>
-        </is>
-      </c>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>⏭</t>
-        </is>
-      </c>
-      <c r="S17" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="T17" t="inlineStr"/>
-      <c r="U17" t="inlineStr">
-        <is>
-          <t>확률·표본·모델합의 기준 미달</t>
-        </is>
-      </c>
-      <c r="V17" t="n">
-        <v>43.75</v>
-      </c>
-      <c r="W17" t="n">
-        <v>60</v>
-      </c>
-      <c r="X17" t="n">
-        <v>47.3</v>
-      </c>
-      <c r="Y17" t="n">
-        <v>52.7</v>
-      </c>
-      <c r="Z17" t="n">
-        <v>47.1</v>
-      </c>
-      <c r="AA17" t="n">
-        <v>33.7</v>
+        <v>39.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-09-27 14:47
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA15"/>
+  <dimension ref="A1:AA16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -556,67 +556,67 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>KT Wiz Suwon</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F2" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="G2" t="n">
-        <v>66.2</v>
+        <v>62</v>
       </c>
       <c r="H2" t="n">
-        <v>33.8</v>
+        <v>38</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>5-2</t>
+          <t>4-2</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="L2" t="n">
-        <v>31.1</v>
+        <v>15.3</v>
       </c>
       <c r="M2" t="n">
-        <v>12.1</v>
+        <v>4.3</v>
       </c>
       <c r="N2" t="n">
-        <v>42.2</v>
+        <v>32.1</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>26.8</v>
+        <v>12.9</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -644,65 +644,65 @@
         </is>
       </c>
       <c r="V2" t="n">
-        <v>30.15</v>
+        <v>37.51</v>
       </c>
       <c r="W2" t="n">
         <v>60</v>
       </c>
       <c r="X2" t="n">
-        <v>60.5</v>
+        <v>53.1</v>
       </c>
       <c r="Y2" t="n">
-        <v>39.5</v>
+        <v>46.9</v>
       </c>
       <c r="Z2" t="n">
-        <v>45.8</v>
+        <v>37.7</v>
       </c>
       <c r="AA2" t="n">
-        <v>31.8</v>
+        <v>15.7</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Doosan Bears</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>St.Louis Cardinals</t>
+          <t>KT Wiz Suwon</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>70</v>
+        <v>31</v>
       </c>
       <c r="F3" t="n">
-        <v>30</v>
+        <v>69</v>
       </c>
       <c r="G3" t="n">
-        <v>64</v>
+        <v>37.4</v>
       </c>
       <c r="H3" t="n">
-        <v>36</v>
+        <v>62.6</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>5-2</t>
+          <t>3-6</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -711,13 +711,13 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>29.7</v>
+        <v>51.8</v>
       </c>
       <c r="M3" t="n">
-        <v>11.3</v>
+        <v>27.1</v>
       </c>
       <c r="N3" t="n">
-        <v>44.5</v>
+        <v>55.5</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>28.6</v>
+        <v>34.5</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -744,7 +744,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -753,28 +753,28 @@
         </is>
       </c>
       <c r="V3" t="n">
-        <v>41.91</v>
+        <v>31</v>
       </c>
       <c r="W3" t="n">
         <v>60</v>
       </c>
       <c r="X3" t="n">
-        <v>54.9</v>
+        <v>46.9</v>
       </c>
       <c r="Y3" t="n">
-        <v>45.1</v>
+        <v>53.1</v>
       </c>
       <c r="Z3" t="n">
-        <v>49.5</v>
+        <v>56.7</v>
       </c>
       <c r="AA3" t="n">
-        <v>34.3</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>8:10</t>
+          <t>4:10</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -793,16 +793,16 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="F4" t="n">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="G4" t="n">
-        <v>64</v>
+        <v>63.4</v>
       </c>
       <c r="H4" t="n">
-        <v>36</v>
+        <v>36.6</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -820,13 +820,13 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>54.4</v>
+        <v>55.7</v>
       </c>
       <c r="M4" t="n">
-        <v>29.4</v>
+        <v>30.6</v>
       </c>
       <c r="N4" t="n">
-        <v>52.4</v>
+        <v>54</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -834,11 +834,11 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>33.9</v>
+        <v>39.5</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>언더</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -862,38 +862,38 @@
         </is>
       </c>
       <c r="V4" t="n">
-        <v>41.91</v>
+        <v>41.1</v>
       </c>
       <c r="W4" t="n">
         <v>60</v>
       </c>
       <c r="X4" t="n">
-        <v>54.9</v>
+        <v>62.5</v>
       </c>
       <c r="Y4" t="n">
-        <v>45.1</v>
+        <v>37.5</v>
       </c>
       <c r="Z4" t="n">
-        <v>51.7</v>
+        <v>53.5</v>
       </c>
       <c r="AA4" t="n">
-        <v>35.3</v>
+        <v>42.4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>4:10</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Seattle Mariners</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Los Angeles Angels</t>
+          <t>St.Louis Cardinals</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -915,7 +915,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>6-3</t>
+          <t>5-2</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -929,13 +929,13 @@
         </is>
       </c>
       <c r="L5" t="n">
-        <v>53.1</v>
+        <v>29.7</v>
       </c>
       <c r="M5" t="n">
-        <v>28.2</v>
+        <v>11.3</v>
       </c>
       <c r="N5" t="n">
-        <v>52.8</v>
+        <v>45.6</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -943,7 +943,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>32.3</v>
+        <v>27.9</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -971,7 +971,7 @@
         </is>
       </c>
       <c r="V5" t="n">
-        <v>42.89</v>
+        <v>43.47</v>
       </c>
       <c r="W5" t="n">
         <v>60</v>
@@ -983,48 +983,48 @@
         <v>41.6</v>
       </c>
       <c r="Z5" t="n">
-        <v>52.7</v>
+        <v>51</v>
       </c>
       <c r="AA5" t="n">
-        <v>33.7</v>
+        <v>33.4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>4:20</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Chunichi Dragons</t>
+          <t>Baltimore Orioles</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>NPB</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>51</v>
+        <v>67</v>
       </c>
       <c r="F6" t="n">
-        <v>49</v>
+        <v>33</v>
       </c>
       <c r="G6" t="n">
-        <v>50.2</v>
+        <v>64</v>
       </c>
       <c r="H6" t="n">
-        <v>49.8</v>
+        <v>36</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>6-3</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -1038,103 +1038,107 @@
         </is>
       </c>
       <c r="L6" t="n">
-        <v>28.4</v>
+        <v>53.1</v>
       </c>
       <c r="M6" t="n">
-        <v>10.6</v>
+        <v>28.2</v>
       </c>
       <c r="N6" t="n">
-        <v>33.9</v>
+        <v>55.6</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P6" t="n">
+        <v>30.9</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
           <t>언더</t>
         </is>
       </c>
-      <c r="P6" t="n">
-        <v>17.6</v>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>언더</t>
-        </is>
-      </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>⏭</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr"/>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>확률·표본·모델합의 기준 미달</t>
+          <t>Forebet·과거모델 합의</t>
         </is>
       </c>
       <c r="V6" t="n">
-        <v>40.96</v>
+        <v>44.57</v>
       </c>
       <c r="W6" t="n">
         <v>60</v>
       </c>
       <c r="X6" t="n">
-        <v>49.1</v>
+        <v>59.5</v>
       </c>
       <c r="Y6" t="n">
-        <v>50.9</v>
+        <v>40.5</v>
       </c>
       <c r="Z6" t="n">
-        <v>35.7</v>
+        <v>56.4</v>
       </c>
       <c r="AA6" t="n">
-        <v>19.9</v>
+        <v>31.9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>KIA Tigers</t>
+          <t>Yokohama BayStars</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>LG Twins</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E7" t="n">
+        <v>51</v>
+      </c>
+      <c r="F7" t="n">
         <v>49</v>
       </c>
-      <c r="F7" t="n">
-        <v>51</v>
-      </c>
       <c r="G7" t="n">
-        <v>46.9</v>
+        <v>50.8</v>
       </c>
       <c r="H7" t="n">
-        <v>53.1</v>
+        <v>49.2</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>6-4</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -1143,25 +1147,25 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>57</v>
+        <v>36.6</v>
       </c>
       <c r="M7" t="n">
-        <v>31.8</v>
+        <v>15.5</v>
       </c>
       <c r="N7" t="n">
-        <v>59</v>
+        <v>35.5</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>43.2</v>
+        <v>21.3</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1181,60 +1185,60 @@
         </is>
       </c>
       <c r="V7" t="n">
-        <v>39.46</v>
+        <v>41.12</v>
       </c>
       <c r="W7" t="n">
         <v>60</v>
       </c>
       <c r="X7" t="n">
-        <v>43.9</v>
+        <v>50.6</v>
       </c>
       <c r="Y7" t="n">
-        <v>56.1</v>
+        <v>49.4</v>
       </c>
       <c r="Z7" t="n">
-        <v>59.7</v>
+        <v>35.1</v>
       </c>
       <c r="AA7" t="n">
-        <v>47</v>
+        <v>23.2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>Nippon Ham Fighters</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F8" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G8" t="n">
-        <v>52</v>
+        <v>56.1</v>
       </c>
       <c r="H8" t="n">
-        <v>48</v>
+        <v>43.9</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>5-2</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -1248,25 +1252,25 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>57</v>
+        <v>31.1</v>
       </c>
       <c r="M8" t="n">
-        <v>31.8</v>
+        <v>12.1</v>
       </c>
       <c r="N8" t="n">
-        <v>59</v>
+        <v>31.4</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>43.2</v>
+        <v>15.9</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -1286,65 +1290,65 @@
         </is>
       </c>
       <c r="V8" t="n">
-        <v>39.67</v>
+        <v>41.42</v>
       </c>
       <c r="W8" t="n">
         <v>60</v>
       </c>
       <c r="X8" t="n">
-        <v>52</v>
+        <v>59.3</v>
       </c>
       <c r="Y8" t="n">
-        <v>48</v>
+        <v>40.7</v>
       </c>
       <c r="Z8" t="n">
-        <v>59.7</v>
+        <v>31.5</v>
       </c>
       <c r="AA8" t="n">
-        <v>47</v>
+        <v>17.2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>5:05</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Washington Nationals</t>
+          <t>KIA Tigers</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>New York Mets</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="F9" t="n">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="G9" t="n">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="H9" t="n">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>6-4</t>
+          <t>4-5</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1353,13 +1357,13 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>65.59999999999999</v>
+        <v>53.1</v>
       </c>
       <c r="M9" t="n">
-        <v>40.4</v>
+        <v>28.2</v>
       </c>
       <c r="N9" t="n">
-        <v>52</v>
+        <v>56.6</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1367,11 +1371,11 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>33.7</v>
+        <v>38.6</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>언더</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -1391,56 +1395,56 @@
         </is>
       </c>
       <c r="V9" t="n">
-        <v>44.72</v>
+        <v>41.01</v>
       </c>
       <c r="W9" t="n">
         <v>60</v>
       </c>
       <c r="X9" t="n">
-        <v>54.4</v>
+        <v>39</v>
       </c>
       <c r="Y9" t="n">
-        <v>45.6</v>
+        <v>61</v>
       </c>
       <c r="Z9" t="n">
-        <v>47.4</v>
+        <v>57.8</v>
       </c>
       <c r="AA9" t="n">
-        <v>31.5</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>5:05</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>San Francisco Giants</t>
+          <t>Lotte Giants</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F10" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G10" t="n">
-        <v>47.3</v>
+        <v>43.5</v>
       </c>
       <c r="H10" t="n">
-        <v>52.7</v>
+        <v>56.5</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -1458,13 +1462,13 @@
         </is>
       </c>
       <c r="L10" t="n">
-        <v>18.5</v>
+        <v>35.2</v>
       </c>
       <c r="M10" t="n">
-        <v>5.6</v>
+        <v>14.6</v>
       </c>
       <c r="N10" t="n">
-        <v>39.3</v>
+        <v>44.3</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1472,7 +1476,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>23.9</v>
+        <v>30</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1496,65 +1500,65 @@
         </is>
       </c>
       <c r="V10" t="n">
-        <v>43.56</v>
+        <v>41.22</v>
       </c>
       <c r="W10" t="n">
         <v>60</v>
       </c>
       <c r="X10" t="n">
-        <v>50.8</v>
+        <v>38.3</v>
       </c>
       <c r="Y10" t="n">
-        <v>49.2</v>
+        <v>61.7</v>
       </c>
       <c r="Z10" t="n">
-        <v>46.2</v>
+        <v>47.3</v>
       </c>
       <c r="AA10" t="n">
-        <v>30</v>
+        <v>35.1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>5:10</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>NC Dinos</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Atlanta Braves</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E11" t="n">
+        <v>49</v>
+      </c>
+      <c r="F11" t="n">
+        <v>51</v>
+      </c>
+      <c r="G11" t="n">
+        <v>48</v>
+      </c>
+      <c r="H11" t="n">
         <v>52</v>
       </c>
-      <c r="F11" t="n">
-        <v>48</v>
-      </c>
-      <c r="G11" t="n">
-        <v>50.5</v>
-      </c>
-      <c r="H11" t="n">
-        <v>49.5</v>
-      </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>3-5</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1563,13 +1567,13 @@
         </is>
       </c>
       <c r="L11" t="n">
-        <v>19.7</v>
+        <v>42.1</v>
       </c>
       <c r="M11" t="n">
-        <v>6.1</v>
+        <v>19.4</v>
       </c>
       <c r="N11" t="n">
-        <v>38.5</v>
+        <v>51.8</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1577,7 +1581,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>25.9</v>
+        <v>33.5</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1601,38 +1605,38 @@
         </is>
       </c>
       <c r="V11" t="n">
-        <v>42.9</v>
+        <v>40.16</v>
       </c>
       <c r="W11" t="n">
         <v>60</v>
       </c>
       <c r="X11" t="n">
-        <v>48.1</v>
+        <v>46.5</v>
       </c>
       <c r="Y11" t="n">
-        <v>51.9</v>
+        <v>53.5</v>
       </c>
       <c r="Z11" t="n">
-        <v>44.7</v>
+        <v>55.1</v>
       </c>
       <c r="AA11" t="n">
-        <v>32.5</v>
+        <v>38.2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>5:10</t>
+          <t>4:05</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Minnesota Twins</t>
+          <t>Washington Nationals</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Texas Rangers</t>
+          <t>New York Mets</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1641,25 +1645,25 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="F12" t="n">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="G12" t="n">
-        <v>50.5</v>
+        <v>56.5</v>
       </c>
       <c r="H12" t="n">
-        <v>49.5</v>
+        <v>43.5</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>4-6</t>
+          <t>6-4</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1668,13 +1672,13 @@
         </is>
       </c>
       <c r="L12" t="n">
-        <v>39.3</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="M12" t="n">
-        <v>17.4</v>
+        <v>40.4</v>
       </c>
       <c r="N12" t="n">
-        <v>49.5</v>
+        <v>52.6</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1682,7 +1686,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>32.3</v>
+        <v>33.8</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1706,38 +1710,38 @@
         </is>
       </c>
       <c r="V12" t="n">
-        <v>42.24</v>
+        <v>44.77</v>
       </c>
       <c r="W12" t="n">
         <v>60</v>
       </c>
       <c r="X12" t="n">
-        <v>52.7</v>
+        <v>55.8</v>
       </c>
       <c r="Y12" t="n">
-        <v>47.3</v>
+        <v>44.2</v>
       </c>
       <c r="Z12" t="n">
-        <v>52.9</v>
+        <v>48.3</v>
       </c>
       <c r="AA12" t="n">
-        <v>37.3</v>
+        <v>31.6</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>8:15</t>
+          <t>4:05</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies</t>
+          <t>San Francisco Giants</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>Los Angeles Dodgers</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1746,20 +1750,20 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="F13" t="n">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="G13" t="n">
-        <v>47.8</v>
+        <v>44.1</v>
       </c>
       <c r="H13" t="n">
-        <v>52.2</v>
+        <v>55.9</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2-3</t>
+          <t>3-4</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1773,13 +1777,13 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>11.4</v>
+        <v>28.4</v>
       </c>
       <c r="M13" t="n">
-        <v>2.8</v>
+        <v>10.6</v>
       </c>
       <c r="N13" t="n">
-        <v>42.6</v>
+        <v>40.1</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1787,7 +1791,7 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>29.1</v>
+        <v>22.5</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1811,38 +1815,38 @@
         </is>
       </c>
       <c r="V13" t="n">
-        <v>42.7</v>
+        <v>40.71</v>
       </c>
       <c r="W13" t="n">
         <v>60</v>
       </c>
       <c r="X13" t="n">
-        <v>50.6</v>
+        <v>50.2</v>
       </c>
       <c r="Y13" t="n">
-        <v>49.4</v>
+        <v>49.8</v>
       </c>
       <c r="Z13" t="n">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="AA13" t="n">
-        <v>37.8</v>
+        <v>26.4</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>9:40</t>
+          <t>4:05</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Philadelphia Phillies</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Arizona Diamondbacks</t>
+          <t>Tampa Bay Rays</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1851,25 +1855,25 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="F14" t="n">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="G14" t="n">
-        <v>51</v>
+        <v>50.8</v>
       </c>
       <c r="H14" t="n">
-        <v>49</v>
+        <v>49.2</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>6-4</t>
+          <t>2-3</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1878,13 +1882,13 @@
         </is>
       </c>
       <c r="L14" t="n">
-        <v>43.5</v>
+        <v>10.6</v>
       </c>
       <c r="M14" t="n">
-        <v>20.4</v>
+        <v>2.5</v>
       </c>
       <c r="N14" t="n">
-        <v>49.8</v>
+        <v>42.5</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1892,7 +1896,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>29.5</v>
+        <v>29.1</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1916,38 +1920,38 @@
         </is>
       </c>
       <c r="V14" t="n">
-        <v>42.01</v>
+        <v>41.71</v>
       </c>
       <c r="W14" t="n">
         <v>60</v>
       </c>
       <c r="X14" t="n">
-        <v>46.6</v>
+        <v>53.6</v>
       </c>
       <c r="Y14" t="n">
-        <v>53.4</v>
+        <v>46.4</v>
       </c>
       <c r="Z14" t="n">
-        <v>52</v>
+        <v>53.2</v>
       </c>
       <c r="AA14" t="n">
-        <v>32.6</v>
+        <v>37.9</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>10:40</t>
+          <t>4:10</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Athletics</t>
+          <t>Miami Marlins</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Houston Astros</t>
+          <t>Atlanta Braves</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1956,25 +1960,25 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="F15" t="n">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="G15" t="n">
-        <v>52.1</v>
+        <v>42.9</v>
       </c>
       <c r="H15" t="n">
-        <v>47.9</v>
+        <v>57.1</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>7-5</t>
+          <t>3-7</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1983,25 +1987,25 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>80.90000000000001</v>
+        <v>62</v>
       </c>
       <c r="M15" t="n">
-        <v>59.8</v>
+        <v>36.7</v>
       </c>
       <c r="N15" t="n">
-        <v>63.5</v>
+        <v>50.2</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>오버</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="P15" t="n">
-        <v>44.6</v>
+        <v>31.3</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -2021,22 +2025,127 @@
         </is>
       </c>
       <c r="V15" t="n">
-        <v>41.44</v>
+        <v>41.94</v>
       </c>
       <c r="W15" t="n">
         <v>60</v>
       </c>
       <c r="X15" t="n">
-        <v>53.8</v>
+        <v>44.1</v>
       </c>
       <c r="Y15" t="n">
+        <v>55.9</v>
+      </c>
+      <c r="Z15" t="n">
         <v>46.2</v>
       </c>
-      <c r="Z15" t="n">
-        <v>57.7</v>
-      </c>
       <c r="AA15" t="n">
-        <v>39.6</v>
+        <v>29.5</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>4:10</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>San Diego Padres</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>59</v>
+      </c>
+      <c r="F16" t="n">
+        <v>41</v>
+      </c>
+      <c r="G16" t="n">
+        <v>55.7</v>
+      </c>
+      <c r="H16" t="n">
+        <v>44.3</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>6-4</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L16" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="M16" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="N16" t="n">
+        <v>50.3</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P16" t="n">
+        <v>30.9</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>언더</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V16" t="n">
+        <v>44</v>
+      </c>
+      <c r="W16" t="n">
+        <v>60</v>
+      </c>
+      <c r="X16" t="n">
+        <v>50.8</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>49.2</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>52.5</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>34.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-09-29 17:23
</commit_message>
<xml_diff>
--- a/baseball_today.xlsx
+++ b/baseball_today.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA9"/>
+  <dimension ref="A1:AA13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -561,12 +561,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Yokohama BayStars</t>
+          <t>Hanshin Tigers</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Hiroshima Carp</t>
+          <t>Yakult Swallows</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -575,20 +575,20 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="F2" t="n">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="G2" t="n">
-        <v>57.6</v>
+        <v>62.5</v>
       </c>
       <c r="H2" t="n">
-        <v>42.4</v>
+        <v>37.5</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -602,13 +602,13 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>16.3</v>
+        <v>7.5</v>
       </c>
       <c r="M2" t="n">
-        <v>4.7</v>
+        <v>1.6</v>
       </c>
       <c r="N2" t="n">
-        <v>29.3</v>
+        <v>24.5</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>15.1</v>
+        <v>13</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -625,37 +625,41 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>⏭</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr"/>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>홈승</t>
+        </is>
+      </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>확률·표본·모델합의 기준 미달</t>
+          <t>Forebet·과거모델 합의</t>
         </is>
       </c>
       <c r="V2" t="n">
-        <v>41.19</v>
+        <v>39.16</v>
       </c>
       <c r="W2" t="n">
         <v>60</v>
       </c>
       <c r="X2" t="n">
-        <v>61.6</v>
+        <v>60.3</v>
       </c>
       <c r="Y2" t="n">
-        <v>38.4</v>
+        <v>39.7</v>
       </c>
       <c r="Z2" t="n">
-        <v>33.6</v>
+        <v>30.2</v>
       </c>
       <c r="AA2" t="n">
-        <v>18.6</v>
+        <v>16.8</v>
       </c>
     </row>
     <row r="3">
@@ -666,12 +670,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Hanshin Tigers</t>
+          <t>Seibu Lions</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Yakult Swallows</t>
+          <t>Orix Buffaloes</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -680,20 +684,20 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F3" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G3" t="n">
-        <v>57.6</v>
+        <v>59.4</v>
       </c>
       <c r="H3" t="n">
-        <v>42.4</v>
+        <v>40.6</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -707,13 +711,13 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>7.5</v>
+        <v>18.5</v>
       </c>
       <c r="M3" t="n">
-        <v>1.6</v>
+        <v>5.6</v>
       </c>
       <c r="N3" t="n">
-        <v>23.7</v>
+        <v>30.1</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -721,7 +725,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>13</v>
+        <v>17.1</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -745,22 +749,22 @@
         </is>
       </c>
       <c r="V3" t="n">
-        <v>41.19</v>
+        <v>41.07</v>
       </c>
       <c r="W3" t="n">
         <v>60</v>
       </c>
       <c r="X3" t="n">
-        <v>61.6</v>
+        <v>63</v>
       </c>
       <c r="Y3" t="n">
-        <v>38.4</v>
+        <v>37</v>
       </c>
       <c r="Z3" t="n">
-        <v>29.2</v>
+        <v>34</v>
       </c>
       <c r="AA3" t="n">
-        <v>16.8</v>
+        <v>20.9</v>
       </c>
     </row>
     <row r="4">
@@ -771,12 +775,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Chiba Lotte Marines</t>
+          <t>Yomiuri Giants</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Nippon Ham Fighters</t>
+          <t>Hiroshima Carp</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -785,25 +789,25 @@
         </is>
       </c>
       <c r="E4" t="n">
+        <v>58</v>
+      </c>
+      <c r="F4" t="n">
         <v>42</v>
       </c>
-      <c r="F4" t="n">
-        <v>58</v>
-      </c>
       <c r="G4" t="n">
-        <v>44.8</v>
+        <v>59.1</v>
       </c>
       <c r="H4" t="n">
-        <v>55.2</v>
+        <v>40.9</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>3-4</t>
+          <t>5-3</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -812,13 +816,13 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>29.7</v>
+        <v>15.3</v>
       </c>
       <c r="M4" t="n">
-        <v>11.3</v>
+        <v>4.3</v>
       </c>
       <c r="N4" t="n">
-        <v>33.9</v>
+        <v>31.7</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -826,7 +830,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>18.2</v>
+        <v>17.3</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -850,60 +854,60 @@
         </is>
       </c>
       <c r="V4" t="n">
-        <v>39.62</v>
+        <v>40.18</v>
       </c>
       <c r="W4" t="n">
         <v>60</v>
       </c>
       <c r="X4" t="n">
-        <v>48.9</v>
+        <v>60.7</v>
       </c>
       <c r="Y4" t="n">
-        <v>51.1</v>
+        <v>39.3</v>
       </c>
       <c r="Z4" t="n">
-        <v>35.4</v>
+        <v>37.2</v>
       </c>
       <c r="AA4" t="n">
-        <v>20.5</v>
+        <v>21.7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Lotte Giants</t>
+          <t>Rakuten Gold. Eagles</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Kiwoom Heroes</t>
+          <t>Chiba Lotte Marines</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>KBO</t>
+          <t>NPB</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>58</v>
+        <v>53.5</v>
       </c>
       <c r="F5" t="n">
-        <v>42</v>
+        <v>46.5</v>
       </c>
       <c r="G5" t="n">
-        <v>58.7</v>
+        <v>55.1</v>
       </c>
       <c r="H5" t="n">
-        <v>41.3</v>
+        <v>44.9</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>6-4</t>
+          <t>4-3</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -917,25 +921,25 @@
         </is>
       </c>
       <c r="L5" t="n">
-        <v>64.40000000000001</v>
+        <v>31.1</v>
       </c>
       <c r="M5" t="n">
-        <v>39.2</v>
+        <v>12.1</v>
       </c>
       <c r="N5" t="n">
-        <v>58.7</v>
+        <v>33.3</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>41.5</v>
+        <v>17.2</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>언더</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -955,22 +959,22 @@
         </is>
       </c>
       <c r="V5" t="n">
-        <v>41.93</v>
+        <v>41.74</v>
       </c>
       <c r="W5" t="n">
         <v>60</v>
       </c>
       <c r="X5" t="n">
-        <v>59.6</v>
+        <v>57.3</v>
       </c>
       <c r="Y5" t="n">
-        <v>40.4</v>
+        <v>42.7</v>
       </c>
       <c r="Z5" t="n">
-        <v>56.7</v>
+        <v>34</v>
       </c>
       <c r="AA5" t="n">
-        <v>42.2</v>
+        <v>18.9</v>
       </c>
     </row>
     <row r="6">
@@ -1001,10 +1005,10 @@
         <v>56</v>
       </c>
       <c r="G6" t="n">
-        <v>41.5</v>
+        <v>41</v>
       </c>
       <c r="H6" t="n">
-        <v>58.5</v>
+        <v>59</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -1028,7 +1032,7 @@
         <v>30.6</v>
       </c>
       <c r="N6" t="n">
-        <v>57.2</v>
+        <v>56.3</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1036,7 +1040,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>40.9</v>
+        <v>41.9</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -1060,22 +1064,22 @@
         </is>
       </c>
       <c r="V6" t="n">
-        <v>41.02</v>
+        <v>40.79</v>
       </c>
       <c r="W6" t="n">
         <v>60</v>
       </c>
       <c r="X6" t="n">
-        <v>37.8</v>
+        <v>36.5</v>
       </c>
       <c r="Y6" t="n">
-        <v>62.2</v>
+        <v>63.5</v>
       </c>
       <c r="Z6" t="n">
-        <v>57.7</v>
+        <v>56.5</v>
       </c>
       <c r="AA6" t="n">
-        <v>44.4</v>
+        <v>45.7</v>
       </c>
     </row>
     <row r="7">
@@ -1086,12 +1090,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Doosan Bears</t>
+          <t>SSG Landers</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>NC Dinos</t>
+          <t>LG Twins</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1100,20 +1104,20 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="F7" t="n">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="G7" t="n">
-        <v>41.9</v>
+        <v>41.1</v>
       </c>
       <c r="H7" t="n">
-        <v>58.1</v>
+        <v>58.9</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>4-5</t>
+          <t>4-6</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1127,13 +1131,13 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>53.1</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="M7" t="n">
-        <v>28.2</v>
+        <v>44.2</v>
       </c>
       <c r="N7" t="n">
-        <v>56.4</v>
+        <v>60.5</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1141,7 +1145,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>40.6</v>
+        <v>41.3</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1165,22 +1169,22 @@
         </is>
       </c>
       <c r="V7" t="n">
-        <v>40.39</v>
+        <v>39.2</v>
       </c>
       <c r="W7" t="n">
         <v>60</v>
       </c>
       <c r="X7" t="n">
-        <v>37.2</v>
+        <v>44.3</v>
       </c>
       <c r="Y7" t="n">
-        <v>62.8</v>
+        <v>55.7</v>
       </c>
       <c r="Z7" t="n">
-        <v>57.6</v>
+        <v>57.7</v>
       </c>
       <c r="AA7" t="n">
-        <v>44.8</v>
+        <v>40.4</v>
       </c>
     </row>
     <row r="8">
@@ -1191,12 +1195,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Samsung Lions</t>
+          <t>Lotte Giants</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Hanwha Eagles</t>
+          <t>Kiwoom Heroes</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1205,20 +1209,20 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F8" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G8" t="n">
-        <v>57.5</v>
+        <v>58.4</v>
       </c>
       <c r="H8" t="n">
-        <v>42.5</v>
+        <v>41.6</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>5-4</t>
+          <t>6-4</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -1232,10 +1236,10 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>55.7</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="M8" t="n">
-        <v>30.6</v>
+        <v>39.2</v>
       </c>
       <c r="N8" t="n">
         <v>57.2</v>
@@ -1246,7 +1250,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>40.9</v>
+        <v>41.2</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1270,60 +1274,60 @@
         </is>
       </c>
       <c r="V8" t="n">
-        <v>41.46</v>
+        <v>41.68</v>
       </c>
       <c r="W8" t="n">
         <v>60</v>
       </c>
       <c r="X8" t="n">
-        <v>58.3</v>
+        <v>58.9</v>
       </c>
       <c r="Y8" t="n">
-        <v>41.7</v>
+        <v>41.1</v>
       </c>
       <c r="Z8" t="n">
-        <v>57.7</v>
+        <v>54.8</v>
       </c>
       <c r="AA8" t="n">
-        <v>44.4</v>
+        <v>41.9</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>5:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Samsung Lions</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Boston Red Sox</t>
+          <t>Hanwha Eagles</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>KBO</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="F9" t="n">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G9" t="n">
-        <v>49.6</v>
+        <v>57.9</v>
       </c>
       <c r="H9" t="n">
-        <v>50.4</v>
+        <v>42.1</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>4-3</t>
+          <t>5-4</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1337,13 +1341,13 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>27.1</v>
+        <v>55.7</v>
       </c>
       <c r="M9" t="n">
-        <v>9.9</v>
+        <v>30.6</v>
       </c>
       <c r="N9" t="n">
-        <v>39.2</v>
+        <v>56.3</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1351,11 +1355,11 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>22.5</v>
+        <v>41.9</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>언더</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -1375,22 +1379,442 @@
         </is>
       </c>
       <c r="V9" t="n">
-        <v>41.72</v>
+        <v>41.36</v>
       </c>
       <c r="W9" t="n">
         <v>60</v>
       </c>
       <c r="X9" t="n">
-        <v>42.9</v>
+        <v>59.2</v>
       </c>
       <c r="Y9" t="n">
-        <v>57.1</v>
+        <v>40.8</v>
       </c>
       <c r="Z9" t="n">
-        <v>43.2</v>
+        <v>56.5</v>
       </c>
       <c r="AA9" t="n">
-        <v>26.6</v>
+        <v>45.7</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Doosan Bears</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>NC Dinos</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>KBO</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>45</v>
+      </c>
+      <c r="F10" t="n">
+        <v>55</v>
+      </c>
+      <c r="G10" t="n">
+        <v>42.2</v>
+      </c>
+      <c r="H10" t="n">
+        <v>57.8</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>4-5</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L10" t="n">
+        <v>53.1</v>
+      </c>
+      <c r="M10" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="N10" t="n">
+        <v>55.5</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P10" t="n">
+        <v>39.1</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V10" t="n">
+        <v>40.02</v>
+      </c>
+      <c r="W10" t="n">
+        <v>60</v>
+      </c>
+      <c r="X10" t="n">
+        <v>38.1</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>61.9</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>56.2</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>42.7</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>6:00</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Houston Astros</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Chicago White Sox</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>52</v>
+      </c>
+      <c r="F11" t="n">
+        <v>48</v>
+      </c>
+      <c r="G11" t="n">
+        <v>50.6</v>
+      </c>
+      <c r="H11" t="n">
+        <v>49.4</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L11" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="M11" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="N11" t="n">
+        <v>44</v>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P11" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>언더</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V11" t="n">
+        <v>41.53</v>
+      </c>
+      <c r="W11" t="n">
+        <v>60</v>
+      </c>
+      <c r="X11" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>54.8</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>39.1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>9:00</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>New York Yankees</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Boston Red Sox</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>54</v>
+      </c>
+      <c r="F12" t="n">
+        <v>46</v>
+      </c>
+      <c r="G12" t="n">
+        <v>52</v>
+      </c>
+      <c r="H12" t="n">
+        <v>48</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L12" t="n">
+        <v>27.1</v>
+      </c>
+      <c r="M12" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="N12" t="n">
+        <v>38.7</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P12" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>언더</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V12" t="n">
+        <v>42.22</v>
+      </c>
+      <c r="W12" t="n">
+        <v>60</v>
+      </c>
+      <c r="X12" t="n">
+        <v>49</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>51</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>42.6</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>26.7</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>San Diego Padres</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Chicago Cubs</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>59</v>
+      </c>
+      <c r="F13" t="n">
+        <v>41</v>
+      </c>
+      <c r="G13" t="n">
+        <v>57.9</v>
+      </c>
+      <c r="H13" t="n">
+        <v>42.1</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>5-4</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
+        <v>54.4</v>
+      </c>
+      <c r="M13" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="N13" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P13" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>언더</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>확률·표본·모델합의 기준 미달</t>
+        </is>
+      </c>
+      <c r="V13" t="n">
+        <v>43.02</v>
+      </c>
+      <c r="W13" t="n">
+        <v>60</v>
+      </c>
+      <c r="X13" t="n">
+        <v>56.2</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>43.8</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>38.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>